<commit_message>
Add SLA re-performance tab for the 6 supplemental accounts
Re-performs the 30-business-day SLA for MIA25103-06, MIA25249 and
MIA25250 (terminated identities approved instead of revoked) with
per-account answers and references to the sample file and walkthrough.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015rwvi2ZZV7Ac5SymUE9zfu
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7.06 Sample Response Evaluation - 2026 Q2.xlsx
+++ b/BSI.IT.27.C7.06 Sample Response Evaluation - 2026 Q2.xlsx
@@ -8,17 +8,17 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="1_Response Summary" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="2_Item Detail" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="3_Step-by-Step" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="4_Open Items" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="5_Follow-up Email" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="6_Sources" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="1_Response Summary" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="2_Item Detail" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="3_Step-by-Step" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="4_Open Items" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="5_Follow-up Email" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="6_Sources" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="7_SLA Re-performance" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Holidays" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'2_Item Detail'!$A$3:$R$62</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'2_Item Detail'!$A$3:$R$62</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1200" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1353" uniqueCount="437">
   <si>
     <t xml:space="preserve">BSI.IT.27.C7 - evaluation of the management response (C7.Sample.xlsx) to the A6 / A5 sample request - 10 accounts</t>
   </si>
@@ -1145,6 +1145,159 @@
     <t xml:space="preserve">478b98cad0b66e5989c71e3ee9f1bef3</t>
   </si>
   <si>
+    <t xml:space="preserve">Re-performance - 30-business-day SLA for the 6 supplemental accounts (Ivan Ramirez Gonzalez, Jefferson Paez Venegas, David Serrano Aguirre, Maiko Vazquez Arias, Richard Harris, Kevin Ackley)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identity (SanIAM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAMS Termination Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AD enabled 11/25/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AD enabled 05/15/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 Q3 decision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 Q1 decision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 Q2 SOX Manager decision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 Q2 CyberArk Manager decision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revocation raised in any review?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Access removal date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLA trigger date (first review after termination)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLA deadline (trigger + 30 business days)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deadline if measured from termination date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Access still held on (latest evidence)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Business days past SLA deadline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLA followed?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference (file / tab / rows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved 08/28/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved 7/27/26, 12:45 PM (Borges, Dayam)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved 8/17/26, 9:23 AM (Borges, Dayam)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None - access not removed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A72 (screenshots at A73 and A79); 2026Q2PamBsiSox-Manager rows 86-88; 2026Q2BsiPamCyberark-Manager rows 419-421; Oct10_2026Users row 1598. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 15, 2025 Q3 ISEAdmin row 53, 2026 Q1 CISCO Network Administrators row 103, 2026 Q1 ISEAdmin row 126; 5_Exceptions row 4. This workbook: 2_Item Detail.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A86 (screenshots at A87 and A93); 2026Q2PamBsiSox-Manager rows 89-91; 2026Q2BsiPamCyberark-Manager rows 422-424; Oct10_2026Users row 1596. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 16, 2025 Q3 ISEAdmin row 54, 2026 Q1 CISCO Network Administrators row 104, 2026 Q1 ISEAdmin row 127; 5_Exceptions row 5. This workbook: 2_Item Detail.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A100 (screenshots at A101 and A107); 2026Q2PamBsiSox-Manager rows 92-94; 2026Q2BsiPamCyberark-Manager rows 425-427; Oct10_2026Users row 1599. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 17, 2025 Q3 ISEAdmin row 55, 2026 Q1 CISCO Network Administrators row 105, 2026 Q1 ISEAdmin row 128; 5_Exceptions row 6. This workbook: 2_Item Detail.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A114 (screenshots at A115 and A121); 2026Q2PamBsiSox-Manager rows 95-97; 2026Q2BsiPamCyberark-Manager rows 428-430; Oct10_2026Users row 1597. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 18, 2025 Q3 ISEAdmin row 56, 2026 Q1 CISCO Network Administrators row 106, 2026 Q1 ISEAdmin row 129; 5_Exceptions row 7. This workbook: 2_Item Detail.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A128 (screenshots at A129 and A135); 2026Q2PamBsiSox-Manager rows 104-106; 2026Q2BsiPamCyberark-Manager rows 437-439; Oct10_2026Users row 1787. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 23, 2025 Q3 ISEAdmin row 58, 2026 Q1 CISCO Network Administrators row 110, 2026 Q1 ISEAdmin row 133; 5_Exceptions row 11. This workbook: 2_Item Detail.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A142 (screenshots at A143 and A149); 2026Q2PamBsiSox-Manager rows 101-103; 2026Q2BsiPamCyberark-Manager rows 434-436; Oct10_2026Users row 1785. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 24, 2025 Q3 ISEAdmin row 59, 2026 Q1 CISCO Network Administrators row 111, 2026 Q1 ISEAdmin row 134; 5_Exceptions row 12. This workbook: 2_Item Detail.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accounts not following the SLA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How the SLA was measured: none of the 6 accounts was revoked, so the SLA clock never started from a "Revoked" decision. Under PAM Recertification Procedure sec. 8 step 9 (revocation for rejects or terminated users) and IAM Standard SUS.IAMS.4.2.5.7 / 4.2.5.21, access of a terminated identity must be revoked at the review and removed within 30 business days.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The trigger is therefore the first certification decision after the IAMS termination date (12/31/2024): the 2025 Q3 decision on 08/28/2025, giving a deadline of 10/10/2025. Column P shows the stricter deadline counted from the termination date itself.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Access still held on: 08/17/2026 = the latest certification in C7.Sample.xlsx (2026 Q2 CyberArk Manager) in which each account is still listed with Cisco Network Administrators / ISEAdmin and Approved. The 10/10/2026 AD export has no group data, so membership after 08/17/2026 is not evidenced.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue text = inputs (dates from the certification exports / walkthrough). Columns O, P, R, S are formulas over the Holidays tab.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Answer to the test step, per account (with reference)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ivan Ramirez Gonzalez (MIA25103)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date the certification decision was made</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date access was removed (if revoked)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not removed. No revocation was raised, and the account is still listed with Cisco Network Administrators, ISEAdmin and CYBERARK_ALERO_USERS in the 2026 Q2 certifications.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Removal within the 30-business-day SLA?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/A - access was never removed and no remediation is evidenced.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supporting evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exception - A5 (terminated identity approved) and A6 (access not removed within SLA). The AD account is also disabled (11/25/2025, 05/15/2026, 10/10/2026) yet still holds and is re-approved for privileged network access. Root cause: the reviewer approved instead of revoking, so the PAM/IAM revocation and SLA process was never triggered.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jefferson Paez Venegas (MIA25104)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exception - A5 (terminated identity approved) and A6 (access not removed within SLA). Root cause: the reviewer approved instead of revoking, so the PAM/IAM revocation and SLA process was never triggered.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">David Serrano Aguirre (MIA25105)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maiko Vazquez Arias (MIA25106)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Richard Harris (MIA25249)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exception - A5 (terminated identity approved) and A6 (access not removed within SLA). AD shows the account disabled on 05/15/2026 and enabled again on 10/10/2026, with no request or audit event provided. Root cause: the reviewer approved instead of revoking, so the PAM/IAM revocation and SLA process was never triggered.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kevin Ackley (MIA25250)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exception - A5 (terminated identity approved) and A6 (access not removed within SLA). AD shows the account disabled on 05/15/2026 and enabled again on 10/10/2026, with no request or audit event provided. AD employeeID / employeeNumber are blank, so the SAMPLE tab hard-codes identity 100592068. Root cause: the reviewer approved instead of revoking, so the PAM/IAM revocation and SLA process was never triggered.</t>
+  </si>
+  <si>
     <t xml:space="preserve">US bank holidays (Federal Reserve) used for the 30-business-day SLA</t>
   </si>
   <si>
@@ -1154,6 +1307,24 @@
     <t xml:space="preserve">Holiday</t>
   </si>
   <si>
+    <t xml:space="preserve">New Year's Day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MLK Day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presidents' Day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Memorial Day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juneteenth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Independence Day</t>
+  </si>
+  <si>
     <t xml:space="preserve">Labor Day</t>
   </si>
   <si>
@@ -1167,21 +1338,6 @@
   </si>
   <si>
     <t xml:space="preserve">Christmas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New Year's Day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MLK Day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Presidents' Day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Memorial Day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Juneteenth</t>
   </si>
   <si>
     <t xml:space="preserve">Independence Day (obs.)</t>
@@ -1343,7 +1499,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1397,6 +1553,34 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1705,24 +1889,6 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
   <dimension ref="A1:U24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -1840,11 +2006,11 @@
         <v>45902</v>
       </c>
       <c r="H4" s="3" t="n">
-        <f aca="false">NETWORKDAYS(F4+1,G4,Holidays!$A$4:$A$17)</f>
+        <f aca="false">NETWORKDAYS(F4+1,G4,Holidays!$A$4:$A$23)</f>
         <v>2</v>
       </c>
       <c r="I4" s="5" t="n">
-        <f aca="false">WORKDAY(F4,30,Holidays!$A$4:$A$17)</f>
+        <f aca="false">WORKDAY(F4,30,Holidays!$A$4:$A$23)</f>
         <v>45940</v>
       </c>
       <c r="J4" s="3" t="str">
@@ -1909,11 +2075,11 @@
         <v>45902</v>
       </c>
       <c r="H5" s="3" t="n">
-        <f aca="false">NETWORKDAYS(F5+1,G5,Holidays!$A$4:$A$17)</f>
+        <f aca="false">NETWORKDAYS(F5+1,G5,Holidays!$A$4:$A$23)</f>
         <v>2</v>
       </c>
       <c r="I5" s="5" t="n">
-        <f aca="false">WORKDAY(F5,30,Holidays!$A$4:$A$17)</f>
+        <f aca="false">WORKDAY(F5,30,Holidays!$A$4:$A$23)</f>
         <v>45940</v>
       </c>
       <c r="J5" s="3" t="str">
@@ -1978,11 +2144,11 @@
         <v>45908</v>
       </c>
       <c r="H6" s="3" t="n">
-        <f aca="false">NETWORKDAYS(F6+1,G6,Holidays!$A$4:$A$17)</f>
+        <f aca="false">NETWORKDAYS(F6+1,G6,Holidays!$A$4:$A$23)</f>
         <v>6</v>
       </c>
       <c r="I6" s="5" t="n">
-        <f aca="false">WORKDAY(F6,30,Holidays!$A$4:$A$17)</f>
+        <f aca="false">WORKDAY(F6,30,Holidays!$A$4:$A$23)</f>
         <v>45940</v>
       </c>
       <c r="J6" s="3" t="str">
@@ -2047,11 +2213,11 @@
         <v>45908</v>
       </c>
       <c r="H7" s="3" t="n">
-        <f aca="false">NETWORKDAYS(F7+1,G7,Holidays!$A$4:$A$17)</f>
+        <f aca="false">NETWORKDAYS(F7+1,G7,Holidays!$A$4:$A$23)</f>
         <v>6</v>
       </c>
       <c r="I7" s="5" t="n">
-        <f aca="false">WORKDAY(F7,30,Holidays!$A$4:$A$17)</f>
+        <f aca="false">WORKDAY(F7,30,Holidays!$A$4:$A$23)</f>
         <v>45940</v>
       </c>
       <c r="J7" s="3" t="str">
@@ -2625,7 +2791,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -6029,7 +6195,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -6261,7 +6427,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -6492,7 +6658,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -6604,7 +6770,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -6805,12 +6971,1682 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:T70"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="10" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="14" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>100531048</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>45657</v>
+      </c>
+      <c r="E4" s="14" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="14" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="14" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>45897</v>
+      </c>
+      <c r="O4" s="5" t="n">
+        <f aca="false">WORKDAY(N4,30,Holidays!$A$4:$A$23)</f>
+        <v>45940</v>
+      </c>
+      <c r="P4" s="5" t="n">
+        <f aca="false">WORKDAY(D4,30,Holidays!$A$4:$A$23)</f>
+        <v>45701</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>46251</v>
+      </c>
+      <c r="R4" s="3" t="n">
+        <f aca="false">IF(Q4&gt;O4,NETWORKDAYS(O4+1,Q4,Holidays!$A$4:$A$23),0)</f>
+        <v>211</v>
+      </c>
+      <c r="S4" s="6" t="str">
+        <f aca="false">IF(AND(L4="No",Q4&gt;O4),"No - SLA not met",IF(R4=0,"Yes","No - late"))</f>
+        <v>No - SLA not met</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>100531049</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>45657</v>
+      </c>
+      <c r="E5" s="11" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F5" s="11" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="G5" s="11" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>45897</v>
+      </c>
+      <c r="O5" s="5" t="n">
+        <f aca="false">WORKDAY(N5,30,Holidays!$A$4:$A$23)</f>
+        <v>45940</v>
+      </c>
+      <c r="P5" s="5" t="n">
+        <f aca="false">WORKDAY(D5,30,Holidays!$A$4:$A$23)</f>
+        <v>45701</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>46251</v>
+      </c>
+      <c r="R5" s="3" t="n">
+        <f aca="false">IF(Q5&gt;O5,NETWORKDAYS(O5+1,Q5,Holidays!$A$4:$A$23),0)</f>
+        <v>211</v>
+      </c>
+      <c r="S5" s="6" t="str">
+        <f aca="false">IF(AND(L5="No",Q5&gt;O5),"No - SLA not met",IF(R5=0,"Yes","No - late"))</f>
+        <v>No - SLA not met</v>
+      </c>
+      <c r="T5" s="3" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>100531050</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>45657</v>
+      </c>
+      <c r="E6" s="11" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F6" s="11" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="G6" s="11" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>45897</v>
+      </c>
+      <c r="O6" s="5" t="n">
+        <f aca="false">WORKDAY(N6,30,Holidays!$A$4:$A$23)</f>
+        <v>45940</v>
+      </c>
+      <c r="P6" s="5" t="n">
+        <f aca="false">WORKDAY(D6,30,Holidays!$A$4:$A$23)</f>
+        <v>45701</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>46251</v>
+      </c>
+      <c r="R6" s="3" t="n">
+        <f aca="false">IF(Q6&gt;O6,NETWORKDAYS(O6+1,Q6,Holidays!$A$4:$A$23),0)</f>
+        <v>211</v>
+      </c>
+      <c r="S6" s="6" t="str">
+        <f aca="false">IF(AND(L6="No",Q6&gt;O6),"No - SLA not met",IF(R6=0,"Yes","No - late"))</f>
+        <v>No - SLA not met</v>
+      </c>
+      <c r="T6" s="3" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>100531051</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>45657</v>
+      </c>
+      <c r="E7" s="11" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F7" s="11" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="G7" s="11" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="N7" s="4" t="n">
+        <v>45897</v>
+      </c>
+      <c r="O7" s="5" t="n">
+        <f aca="false">WORKDAY(N7,30,Holidays!$A$4:$A$23)</f>
+        <v>45940</v>
+      </c>
+      <c r="P7" s="5" t="n">
+        <f aca="false">WORKDAY(D7,30,Holidays!$A$4:$A$23)</f>
+        <v>45701</v>
+      </c>
+      <c r="Q7" s="4" t="n">
+        <v>46251</v>
+      </c>
+      <c r="R7" s="3" t="n">
+        <f aca="false">IF(Q7&gt;O7,NETWORKDAYS(O7+1,Q7,Holidays!$A$4:$A$23),0)</f>
+        <v>211</v>
+      </c>
+      <c r="S7" s="6" t="str">
+        <f aca="false">IF(AND(L7="No",Q7&gt;O7),"No - SLA not met",IF(R7=0,"Yes","No - late"))</f>
+        <v>No - SLA not met</v>
+      </c>
+      <c r="T7" s="3" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>100592069</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>45657</v>
+      </c>
+      <c r="E8" s="11" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F8" s="14" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="11" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>45897</v>
+      </c>
+      <c r="O8" s="5" t="n">
+        <f aca="false">WORKDAY(N8,30,Holidays!$A$4:$A$23)</f>
+        <v>45940</v>
+      </c>
+      <c r="P8" s="5" t="n">
+        <f aca="false">WORKDAY(D8,30,Holidays!$A$4:$A$23)</f>
+        <v>45701</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>46251</v>
+      </c>
+      <c r="R8" s="3" t="n">
+        <f aca="false">IF(Q8&gt;O8,NETWORKDAYS(O8+1,Q8,Holidays!$A$4:$A$23),0)</f>
+        <v>211</v>
+      </c>
+      <c r="S8" s="6" t="str">
+        <f aca="false">IF(AND(L8="No",Q8&gt;O8),"No - SLA not met",IF(R8=0,"Yes","No - late"))</f>
+        <v>No - SLA not met</v>
+      </c>
+      <c r="T8" s="3" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>100592068</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>45657</v>
+      </c>
+      <c r="E9" s="11" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F9" s="14" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="11" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="M9" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="N9" s="4" t="n">
+        <v>45897</v>
+      </c>
+      <c r="O9" s="5" t="n">
+        <f aca="false">WORKDAY(N9,30,Holidays!$A$4:$A$23)</f>
+        <v>45940</v>
+      </c>
+      <c r="P9" s="5" t="n">
+        <f aca="false">WORKDAY(D9,30,Holidays!$A$4:$A$23)</f>
+        <v>45701</v>
+      </c>
+      <c r="Q9" s="4" t="n">
+        <v>46251</v>
+      </c>
+      <c r="R9" s="3" t="n">
+        <f aca="false">IF(Q9&gt;O9,NETWORKDAYS(O9+1,Q9,Holidays!$A$4:$A$23),0)</f>
+        <v>211</v>
+      </c>
+      <c r="S9" s="6" t="str">
+        <f aca="false">IF(AND(L9="No",Q9&gt;O9),"No - SLA not met",IF(R9=0,"Yes","No - late"))</f>
+        <v>No - SLA not met</v>
+      </c>
+      <c r="T9" s="3" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="15" t="s">
+        <v>399</v>
+      </c>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="9" t="str">
+        <f aca="false">COUNTIF(S4:S9,"No*")&amp;" of "&amp;COUNTA(A4:A9)</f>
+        <v>6 of 6</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="16" t="s">
+        <v>400</v>
+      </c>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="16"/>
+      <c r="M12" s="16"/>
+      <c r="N12" s="16"/>
+    </row>
+    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="16" t="s">
+        <v>401</v>
+      </c>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="16"/>
+      <c r="I13" s="16"/>
+      <c r="J13" s="16"/>
+      <c r="K13" s="16"/>
+      <c r="L13" s="16"/>
+      <c r="M13" s="16"/>
+      <c r="N13" s="16"/>
+    </row>
+    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="16" t="s">
+        <v>402</v>
+      </c>
+      <c r="B14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="16"/>
+      <c r="I14" s="16"/>
+      <c r="J14" s="16"/>
+      <c r="K14" s="16"/>
+      <c r="L14" s="16"/>
+      <c r="M14" s="16"/>
+      <c r="N14" s="16"/>
+    </row>
+    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="16" t="s">
+        <v>403</v>
+      </c>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="16"/>
+      <c r="M15" s="16"/>
+      <c r="N15" s="16"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="17" t="s">
+        <v>405</v>
+      </c>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="17"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="17"/>
+      <c r="L18" s="17"/>
+      <c r="M18" s="17"/>
+      <c r="N18" s="17"/>
+    </row>
+    <row r="19" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="18" t="s">
+        <v>406</v>
+      </c>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="19" t="str">
+        <f aca="false">"Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), "&amp;J4&amp;", "&amp;K4&amp;". No Revoked decision in any review."</f>
+        <v>Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), Approved 7/27/26, 12:45 PM (Borges, Dayam), Approved 8/17/26, 9:23 AM (Borges, Dayam). No Revoked decision in any review.</v>
+      </c>
+      <c r="E19" s="19"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="19"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19"/>
+      <c r="L19" s="19"/>
+      <c r="M19" s="19"/>
+      <c r="N19" s="19"/>
+    </row>
+    <row r="20" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="18" t="s">
+        <v>407</v>
+      </c>
+      <c r="B20" s="18"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="19" t="s">
+        <v>408</v>
+      </c>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="19"/>
+      <c r="K20" s="19"/>
+      <c r="L20" s="19"/>
+      <c r="M20" s="19"/>
+      <c r="N20" s="19"/>
+    </row>
+    <row r="21" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="18" t="s">
+        <v>409</v>
+      </c>
+      <c r="B21" s="18"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="20" t="str">
+        <f aca="false">"NO - SLA not met. IAMS termination date "&amp;TEXT(D4,"mm/dd/yyyy")&amp;"; removal was due by "&amp;TEXT(O4,"mm/dd/yyyy")&amp;" (30 business days after the 08/28/2025 review) and access was still held on "&amp;TEXT(Q4,"mm/dd/yyyy")&amp;", "&amp;R4&amp;" business days past the deadline."</f>
+        <v>NO - SLA not met. IAMS termination date 12/31/2024; removal was due by 10/10/2025 (30 business days after the 08/28/2025 review) and access was still held on 08/17/2026, 211 business days past the deadline.</v>
+      </c>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="20"/>
+      <c r="I21" s="20"/>
+      <c r="J21" s="20"/>
+      <c r="K21" s="20"/>
+      <c r="L21" s="20"/>
+      <c r="M21" s="20"/>
+      <c r="N21" s="20"/>
+    </row>
+    <row r="22" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" s="18"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="19" t="s">
+        <v>410</v>
+      </c>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="19"/>
+      <c r="H22" s="19"/>
+      <c r="I22" s="19"/>
+      <c r="J22" s="19"/>
+      <c r="K22" s="19"/>
+      <c r="L22" s="19"/>
+      <c r="M22" s="19"/>
+      <c r="N22" s="19"/>
+    </row>
+    <row r="23" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="B23" s="18"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="19" t="str">
+        <f aca="false">"C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = "&amp;IF(G4,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
+        <v>C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = FALSE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
+      </c>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
+      <c r="G23" s="19"/>
+      <c r="H23" s="19"/>
+      <c r="I23" s="19"/>
+      <c r="J23" s="19"/>
+      <c r="K23" s="19"/>
+      <c r="L23" s="19"/>
+      <c r="M23" s="19"/>
+      <c r="N23" s="19"/>
+    </row>
+    <row r="24" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="18"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="20" t="s">
+        <v>412</v>
+      </c>
+      <c r="E24" s="20"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="20"/>
+      <c r="H24" s="20"/>
+      <c r="I24" s="20"/>
+      <c r="J24" s="20"/>
+      <c r="K24" s="20"/>
+      <c r="L24" s="20"/>
+      <c r="M24" s="20"/>
+      <c r="N24" s="20"/>
+    </row>
+    <row r="25" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="18" t="s">
+        <v>413</v>
+      </c>
+      <c r="B25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="19" t="str">
+        <f aca="false">T4</f>
+        <v>C7.Sample.xlsx: SAMPLE!A72 (screenshots at A73 and A79); 2026Q2PamBsiSox-Manager rows 86-88; 2026Q2BsiPamCyberark-Manager rows 419-421; Oct10_2026Users row 1598. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 15, 2025 Q3 ISEAdmin row 53, 2026 Q1 CISCO Network Administrators row 103, 2026 Q1 ISEAdmin row 126; 5_Exceptions row 4. This workbook: 2_Item Detail.</v>
+      </c>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="19"/>
+      <c r="I25" s="19"/>
+      <c r="J25" s="19"/>
+      <c r="K25" s="19"/>
+      <c r="L25" s="19"/>
+      <c r="M25" s="19"/>
+      <c r="N25" s="19"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="17" t="s">
+        <v>414</v>
+      </c>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="17"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="17"/>
+      <c r="K27" s="17"/>
+      <c r="L27" s="17"/>
+      <c r="M27" s="17"/>
+      <c r="N27" s="17"/>
+    </row>
+    <row r="28" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="18" t="s">
+        <v>406</v>
+      </c>
+      <c r="B28" s="18"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="19" t="str">
+        <f aca="false">"Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), "&amp;J5&amp;", "&amp;K5&amp;". No Revoked decision in any review."</f>
+        <v>Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), Approved 7/27/26, 12:45 PM (Borges, Dayam), Approved 8/17/26, 9:23 AM (Borges, Dayam). No Revoked decision in any review.</v>
+      </c>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="19"/>
+      <c r="J28" s="19"/>
+      <c r="K28" s="19"/>
+      <c r="L28" s="19"/>
+      <c r="M28" s="19"/>
+      <c r="N28" s="19"/>
+    </row>
+    <row r="29" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="18" t="s">
+        <v>407</v>
+      </c>
+      <c r="B29" s="18"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="19" t="s">
+        <v>408</v>
+      </c>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
+      <c r="G29" s="19"/>
+      <c r="H29" s="19"/>
+      <c r="I29" s="19"/>
+      <c r="J29" s="19"/>
+      <c r="K29" s="19"/>
+      <c r="L29" s="19"/>
+      <c r="M29" s="19"/>
+      <c r="N29" s="19"/>
+    </row>
+    <row r="30" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="18" t="s">
+        <v>409</v>
+      </c>
+      <c r="B30" s="18"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="20" t="str">
+        <f aca="false">"NO - SLA not met. IAMS termination date "&amp;TEXT(D5,"mm/dd/yyyy")&amp;"; removal was due by "&amp;TEXT(O5,"mm/dd/yyyy")&amp;" (30 business days after the 08/28/2025 review) and access was still held on "&amp;TEXT(Q5,"mm/dd/yyyy")&amp;", "&amp;R5&amp;" business days past the deadline."</f>
+        <v>NO - SLA not met. IAMS termination date 12/31/2024; removal was due by 10/10/2025 (30 business days after the 08/28/2025 review) and access was still held on 08/17/2026, 211 business days past the deadline.</v>
+      </c>
+      <c r="E30" s="20"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="20"/>
+      <c r="H30" s="20"/>
+      <c r="I30" s="20"/>
+      <c r="J30" s="20"/>
+      <c r="K30" s="20"/>
+      <c r="L30" s="20"/>
+      <c r="M30" s="20"/>
+      <c r="N30" s="20"/>
+    </row>
+    <row r="31" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B31" s="18"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="19" t="s">
+        <v>410</v>
+      </c>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
+      <c r="G31" s="19"/>
+      <c r="H31" s="19"/>
+      <c r="I31" s="19"/>
+      <c r="J31" s="19"/>
+      <c r="K31" s="19"/>
+      <c r="L31" s="19"/>
+      <c r="M31" s="19"/>
+      <c r="N31" s="19"/>
+    </row>
+    <row r="32" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="B32" s="18"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="19" t="str">
+        <f aca="false">"C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = "&amp;IF(G5,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
+        <v>C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = TRUE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
+      </c>
+      <c r="E32" s="19"/>
+      <c r="F32" s="19"/>
+      <c r="G32" s="19"/>
+      <c r="H32" s="19"/>
+      <c r="I32" s="19"/>
+      <c r="J32" s="19"/>
+      <c r="K32" s="19"/>
+      <c r="L32" s="19"/>
+      <c r="M32" s="19"/>
+      <c r="N32" s="19"/>
+    </row>
+    <row r="33" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B33" s="18"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="20" t="s">
+        <v>415</v>
+      </c>
+      <c r="E33" s="20"/>
+      <c r="F33" s="20"/>
+      <c r="G33" s="20"/>
+      <c r="H33" s="20"/>
+      <c r="I33" s="20"/>
+      <c r="J33" s="20"/>
+      <c r="K33" s="20"/>
+      <c r="L33" s="20"/>
+      <c r="M33" s="20"/>
+      <c r="N33" s="20"/>
+    </row>
+    <row r="34" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="18" t="s">
+        <v>413</v>
+      </c>
+      <c r="B34" s="18"/>
+      <c r="C34" s="18"/>
+      <c r="D34" s="19" t="str">
+        <f aca="false">T5</f>
+        <v>C7.Sample.xlsx: SAMPLE!A86 (screenshots at A87 and A93); 2026Q2PamBsiSox-Manager rows 89-91; 2026Q2BsiPamCyberark-Manager rows 422-424; Oct10_2026Users row 1596. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 16, 2025 Q3 ISEAdmin row 54, 2026 Q1 CISCO Network Administrators row 104, 2026 Q1 ISEAdmin row 127; 5_Exceptions row 5. This workbook: 2_Item Detail.</v>
+      </c>
+      <c r="E34" s="19"/>
+      <c r="F34" s="19"/>
+      <c r="G34" s="19"/>
+      <c r="H34" s="19"/>
+      <c r="I34" s="19"/>
+      <c r="J34" s="19"/>
+      <c r="K34" s="19"/>
+      <c r="L34" s="19"/>
+      <c r="M34" s="19"/>
+      <c r="N34" s="19"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="17" t="s">
+        <v>416</v>
+      </c>
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="17"/>
+      <c r="H36" s="17"/>
+      <c r="I36" s="17"/>
+      <c r="J36" s="17"/>
+      <c r="K36" s="17"/>
+      <c r="L36" s="17"/>
+      <c r="M36" s="17"/>
+      <c r="N36" s="17"/>
+    </row>
+    <row r="37" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="18" t="s">
+        <v>406</v>
+      </c>
+      <c r="B37" s="18"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="19" t="str">
+        <f aca="false">"Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), "&amp;J6&amp;", "&amp;K6&amp;". No Revoked decision in any review."</f>
+        <v>Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), Approved 7/27/26, 12:45 PM (Borges, Dayam), Approved 8/17/26, 9:23 AM (Borges, Dayam). No Revoked decision in any review.</v>
+      </c>
+      <c r="E37" s="19"/>
+      <c r="F37" s="19"/>
+      <c r="G37" s="19"/>
+      <c r="H37" s="19"/>
+      <c r="I37" s="19"/>
+      <c r="J37" s="19"/>
+      <c r="K37" s="19"/>
+      <c r="L37" s="19"/>
+      <c r="M37" s="19"/>
+      <c r="N37" s="19"/>
+    </row>
+    <row r="38" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="18" t="s">
+        <v>407</v>
+      </c>
+      <c r="B38" s="18"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="19" t="s">
+        <v>408</v>
+      </c>
+      <c r="E38" s="19"/>
+      <c r="F38" s="19"/>
+      <c r="G38" s="19"/>
+      <c r="H38" s="19"/>
+      <c r="I38" s="19"/>
+      <c r="J38" s="19"/>
+      <c r="K38" s="19"/>
+      <c r="L38" s="19"/>
+      <c r="M38" s="19"/>
+      <c r="N38" s="19"/>
+    </row>
+    <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="18" t="s">
+        <v>409</v>
+      </c>
+      <c r="B39" s="18"/>
+      <c r="C39" s="18"/>
+      <c r="D39" s="20" t="str">
+        <f aca="false">"NO - SLA not met. IAMS termination date "&amp;TEXT(D6,"mm/dd/yyyy")&amp;"; removal was due by "&amp;TEXT(O6,"mm/dd/yyyy")&amp;" (30 business days after the 08/28/2025 review) and access was still held on "&amp;TEXT(Q6,"mm/dd/yyyy")&amp;", "&amp;R6&amp;" business days past the deadline."</f>
+        <v>NO - SLA not met. IAMS termination date 12/31/2024; removal was due by 10/10/2025 (30 business days after the 08/28/2025 review) and access was still held on 08/17/2026, 211 business days past the deadline.</v>
+      </c>
+      <c r="E39" s="20"/>
+      <c r="F39" s="20"/>
+      <c r="G39" s="20"/>
+      <c r="H39" s="20"/>
+      <c r="I39" s="20"/>
+      <c r="J39" s="20"/>
+      <c r="K39" s="20"/>
+      <c r="L39" s="20"/>
+      <c r="M39" s="20"/>
+      <c r="N39" s="20"/>
+    </row>
+    <row r="40" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B40" s="18"/>
+      <c r="C40" s="18"/>
+      <c r="D40" s="19" t="s">
+        <v>410</v>
+      </c>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="19"/>
+      <c r="H40" s="19"/>
+      <c r="I40" s="19"/>
+      <c r="J40" s="19"/>
+      <c r="K40" s="19"/>
+      <c r="L40" s="19"/>
+      <c r="M40" s="19"/>
+      <c r="N40" s="19"/>
+    </row>
+    <row r="41" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="B41" s="18"/>
+      <c r="C41" s="18"/>
+      <c r="D41" s="19" t="str">
+        <f aca="false">"C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = "&amp;IF(G6,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
+        <v>C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = TRUE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
+      </c>
+      <c r="E41" s="19"/>
+      <c r="F41" s="19"/>
+      <c r="G41" s="19"/>
+      <c r="H41" s="19"/>
+      <c r="I41" s="19"/>
+      <c r="J41" s="19"/>
+      <c r="K41" s="19"/>
+      <c r="L41" s="19"/>
+      <c r="M41" s="19"/>
+      <c r="N41" s="19"/>
+    </row>
+    <row r="42" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B42" s="18"/>
+      <c r="C42" s="18"/>
+      <c r="D42" s="20" t="s">
+        <v>415</v>
+      </c>
+      <c r="E42" s="20"/>
+      <c r="F42" s="20"/>
+      <c r="G42" s="20"/>
+      <c r="H42" s="20"/>
+      <c r="I42" s="20"/>
+      <c r="J42" s="20"/>
+      <c r="K42" s="20"/>
+      <c r="L42" s="20"/>
+      <c r="M42" s="20"/>
+      <c r="N42" s="20"/>
+    </row>
+    <row r="43" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="18" t="s">
+        <v>413</v>
+      </c>
+      <c r="B43" s="18"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="19" t="str">
+        <f aca="false">T6</f>
+        <v>C7.Sample.xlsx: SAMPLE!A100 (screenshots at A101 and A107); 2026Q2PamBsiSox-Manager rows 92-94; 2026Q2BsiPamCyberark-Manager rows 425-427; Oct10_2026Users row 1599. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 17, 2025 Q3 ISEAdmin row 55, 2026 Q1 CISCO Network Administrators row 105, 2026 Q1 ISEAdmin row 128; 5_Exceptions row 6. This workbook: 2_Item Detail.</v>
+      </c>
+      <c r="E43" s="19"/>
+      <c r="F43" s="19"/>
+      <c r="G43" s="19"/>
+      <c r="H43" s="19"/>
+      <c r="I43" s="19"/>
+      <c r="J43" s="19"/>
+      <c r="K43" s="19"/>
+      <c r="L43" s="19"/>
+      <c r="M43" s="19"/>
+      <c r="N43" s="19"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="17" t="s">
+        <v>417</v>
+      </c>
+      <c r="B45" s="17"/>
+      <c r="C45" s="17"/>
+      <c r="D45" s="17"/>
+      <c r="E45" s="17"/>
+      <c r="F45" s="17"/>
+      <c r="G45" s="17"/>
+      <c r="H45" s="17"/>
+      <c r="I45" s="17"/>
+      <c r="J45" s="17"/>
+      <c r="K45" s="17"/>
+      <c r="L45" s="17"/>
+      <c r="M45" s="17"/>
+      <c r="N45" s="17"/>
+    </row>
+    <row r="46" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="18" t="s">
+        <v>406</v>
+      </c>
+      <c r="B46" s="18"/>
+      <c r="C46" s="18"/>
+      <c r="D46" s="19" t="str">
+        <f aca="false">"Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), "&amp;J7&amp;", "&amp;K7&amp;". No Revoked decision in any review."</f>
+        <v>Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), Approved 7/27/26, 12:45 PM (Borges, Dayam), Approved 8/17/26, 9:23 AM (Borges, Dayam). No Revoked decision in any review.</v>
+      </c>
+      <c r="E46" s="19"/>
+      <c r="F46" s="19"/>
+      <c r="G46" s="19"/>
+      <c r="H46" s="19"/>
+      <c r="I46" s="19"/>
+      <c r="J46" s="19"/>
+      <c r="K46" s="19"/>
+      <c r="L46" s="19"/>
+      <c r="M46" s="19"/>
+      <c r="N46" s="19"/>
+    </row>
+    <row r="47" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="18" t="s">
+        <v>407</v>
+      </c>
+      <c r="B47" s="18"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="19" t="s">
+        <v>408</v>
+      </c>
+      <c r="E47" s="19"/>
+      <c r="F47" s="19"/>
+      <c r="G47" s="19"/>
+      <c r="H47" s="19"/>
+      <c r="I47" s="19"/>
+      <c r="J47" s="19"/>
+      <c r="K47" s="19"/>
+      <c r="L47" s="19"/>
+      <c r="M47" s="19"/>
+      <c r="N47" s="19"/>
+    </row>
+    <row r="48" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="18" t="s">
+        <v>409</v>
+      </c>
+      <c r="B48" s="18"/>
+      <c r="C48" s="18"/>
+      <c r="D48" s="20" t="str">
+        <f aca="false">"NO - SLA not met. IAMS termination date "&amp;TEXT(D7,"mm/dd/yyyy")&amp;"; removal was due by "&amp;TEXT(O7,"mm/dd/yyyy")&amp;" (30 business days after the 08/28/2025 review) and access was still held on "&amp;TEXT(Q7,"mm/dd/yyyy")&amp;", "&amp;R7&amp;" business days past the deadline."</f>
+        <v>NO - SLA not met. IAMS termination date 12/31/2024; removal was due by 10/10/2025 (30 business days after the 08/28/2025 review) and access was still held on 08/17/2026, 211 business days past the deadline.</v>
+      </c>
+      <c r="E48" s="20"/>
+      <c r="F48" s="20"/>
+      <c r="G48" s="20"/>
+      <c r="H48" s="20"/>
+      <c r="I48" s="20"/>
+      <c r="J48" s="20"/>
+      <c r="K48" s="20"/>
+      <c r="L48" s="20"/>
+      <c r="M48" s="20"/>
+      <c r="N48" s="20"/>
+    </row>
+    <row r="49" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B49" s="18"/>
+      <c r="C49" s="18"/>
+      <c r="D49" s="19" t="s">
+        <v>410</v>
+      </c>
+      <c r="E49" s="19"/>
+      <c r="F49" s="19"/>
+      <c r="G49" s="19"/>
+      <c r="H49" s="19"/>
+      <c r="I49" s="19"/>
+      <c r="J49" s="19"/>
+      <c r="K49" s="19"/>
+      <c r="L49" s="19"/>
+      <c r="M49" s="19"/>
+      <c r="N49" s="19"/>
+    </row>
+    <row r="50" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="B50" s="18"/>
+      <c r="C50" s="18"/>
+      <c r="D50" s="19" t="str">
+        <f aca="false">"C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = "&amp;IF(G7,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
+        <v>C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = TRUE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
+      </c>
+      <c r="E50" s="19"/>
+      <c r="F50" s="19"/>
+      <c r="G50" s="19"/>
+      <c r="H50" s="19"/>
+      <c r="I50" s="19"/>
+      <c r="J50" s="19"/>
+      <c r="K50" s="19"/>
+      <c r="L50" s="19"/>
+      <c r="M50" s="19"/>
+      <c r="N50" s="19"/>
+    </row>
+    <row r="51" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B51" s="18"/>
+      <c r="C51" s="18"/>
+      <c r="D51" s="20" t="s">
+        <v>415</v>
+      </c>
+      <c r="E51" s="20"/>
+      <c r="F51" s="20"/>
+      <c r="G51" s="20"/>
+      <c r="H51" s="20"/>
+      <c r="I51" s="20"/>
+      <c r="J51" s="20"/>
+      <c r="K51" s="20"/>
+      <c r="L51" s="20"/>
+      <c r="M51" s="20"/>
+      <c r="N51" s="20"/>
+    </row>
+    <row r="52" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="18" t="s">
+        <v>413</v>
+      </c>
+      <c r="B52" s="18"/>
+      <c r="C52" s="18"/>
+      <c r="D52" s="19" t="str">
+        <f aca="false">T7</f>
+        <v>C7.Sample.xlsx: SAMPLE!A114 (screenshots at A115 and A121); 2026Q2PamBsiSox-Manager rows 95-97; 2026Q2BsiPamCyberark-Manager rows 428-430; Oct10_2026Users row 1597. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 18, 2025 Q3 ISEAdmin row 56, 2026 Q1 CISCO Network Administrators row 106, 2026 Q1 ISEAdmin row 129; 5_Exceptions row 7. This workbook: 2_Item Detail.</v>
+      </c>
+      <c r="E52" s="19"/>
+      <c r="F52" s="19"/>
+      <c r="G52" s="19"/>
+      <c r="H52" s="19"/>
+      <c r="I52" s="19"/>
+      <c r="J52" s="19"/>
+      <c r="K52" s="19"/>
+      <c r="L52" s="19"/>
+      <c r="M52" s="19"/>
+      <c r="N52" s="19"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="17" t="s">
+        <v>418</v>
+      </c>
+      <c r="B54" s="17"/>
+      <c r="C54" s="17"/>
+      <c r="D54" s="17"/>
+      <c r="E54" s="17"/>
+      <c r="F54" s="17"/>
+      <c r="G54" s="17"/>
+      <c r="H54" s="17"/>
+      <c r="I54" s="17"/>
+      <c r="J54" s="17"/>
+      <c r="K54" s="17"/>
+      <c r="L54" s="17"/>
+      <c r="M54" s="17"/>
+      <c r="N54" s="17"/>
+    </row>
+    <row r="55" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="18" t="s">
+        <v>406</v>
+      </c>
+      <c r="B55" s="18"/>
+      <c r="C55" s="18"/>
+      <c r="D55" s="19" t="str">
+        <f aca="false">"Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), "&amp;J8&amp;", "&amp;K8&amp;". No Revoked decision in any review."</f>
+        <v>Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), Approved 7/27/26, 12:45 PM (Borges, Dayam), Approved 8/17/26, 9:23 AM (Borges, Dayam). No Revoked decision in any review.</v>
+      </c>
+      <c r="E55" s="19"/>
+      <c r="F55" s="19"/>
+      <c r="G55" s="19"/>
+      <c r="H55" s="19"/>
+      <c r="I55" s="19"/>
+      <c r="J55" s="19"/>
+      <c r="K55" s="19"/>
+      <c r="L55" s="19"/>
+      <c r="M55" s="19"/>
+      <c r="N55" s="19"/>
+    </row>
+    <row r="56" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="18" t="s">
+        <v>407</v>
+      </c>
+      <c r="B56" s="18"/>
+      <c r="C56" s="18"/>
+      <c r="D56" s="19" t="s">
+        <v>408</v>
+      </c>
+      <c r="E56" s="19"/>
+      <c r="F56" s="19"/>
+      <c r="G56" s="19"/>
+      <c r="H56" s="19"/>
+      <c r="I56" s="19"/>
+      <c r="J56" s="19"/>
+      <c r="K56" s="19"/>
+      <c r="L56" s="19"/>
+      <c r="M56" s="19"/>
+      <c r="N56" s="19"/>
+    </row>
+    <row r="57" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="18" t="s">
+        <v>409</v>
+      </c>
+      <c r="B57" s="18"/>
+      <c r="C57" s="18"/>
+      <c r="D57" s="20" t="str">
+        <f aca="false">"NO - SLA not met. IAMS termination date "&amp;TEXT(D8,"mm/dd/yyyy")&amp;"; removal was due by "&amp;TEXT(O8,"mm/dd/yyyy")&amp;" (30 business days after the 08/28/2025 review) and access was still held on "&amp;TEXT(Q8,"mm/dd/yyyy")&amp;", "&amp;R8&amp;" business days past the deadline."</f>
+        <v>NO - SLA not met. IAMS termination date 12/31/2024; removal was due by 10/10/2025 (30 business days after the 08/28/2025 review) and access was still held on 08/17/2026, 211 business days past the deadline.</v>
+      </c>
+      <c r="E57" s="20"/>
+      <c r="F57" s="20"/>
+      <c r="G57" s="20"/>
+      <c r="H57" s="20"/>
+      <c r="I57" s="20"/>
+      <c r="J57" s="20"/>
+      <c r="K57" s="20"/>
+      <c r="L57" s="20"/>
+      <c r="M57" s="20"/>
+      <c r="N57" s="20"/>
+    </row>
+    <row r="58" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B58" s="18"/>
+      <c r="C58" s="18"/>
+      <c r="D58" s="19" t="s">
+        <v>410</v>
+      </c>
+      <c r="E58" s="19"/>
+      <c r="F58" s="19"/>
+      <c r="G58" s="19"/>
+      <c r="H58" s="19"/>
+      <c r="I58" s="19"/>
+      <c r="J58" s="19"/>
+      <c r="K58" s="19"/>
+      <c r="L58" s="19"/>
+      <c r="M58" s="19"/>
+      <c r="N58" s="19"/>
+    </row>
+    <row r="59" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="B59" s="18"/>
+      <c r="C59" s="18"/>
+      <c r="D59" s="19" t="str">
+        <f aca="false">"C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = "&amp;IF(G8,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
+        <v>C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = TRUE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
+      </c>
+      <c r="E59" s="19"/>
+      <c r="F59" s="19"/>
+      <c r="G59" s="19"/>
+      <c r="H59" s="19"/>
+      <c r="I59" s="19"/>
+      <c r="J59" s="19"/>
+      <c r="K59" s="19"/>
+      <c r="L59" s="19"/>
+      <c r="M59" s="19"/>
+      <c r="N59" s="19"/>
+    </row>
+    <row r="60" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B60" s="18"/>
+      <c r="C60" s="18"/>
+      <c r="D60" s="20" t="s">
+        <v>419</v>
+      </c>
+      <c r="E60" s="20"/>
+      <c r="F60" s="20"/>
+      <c r="G60" s="20"/>
+      <c r="H60" s="20"/>
+      <c r="I60" s="20"/>
+      <c r="J60" s="20"/>
+      <c r="K60" s="20"/>
+      <c r="L60" s="20"/>
+      <c r="M60" s="20"/>
+      <c r="N60" s="20"/>
+    </row>
+    <row r="61" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="18" t="s">
+        <v>413</v>
+      </c>
+      <c r="B61" s="18"/>
+      <c r="C61" s="18"/>
+      <c r="D61" s="19" t="str">
+        <f aca="false">T8</f>
+        <v>C7.Sample.xlsx: SAMPLE!A128 (screenshots at A129 and A135); 2026Q2PamBsiSox-Manager rows 104-106; 2026Q2BsiPamCyberark-Manager rows 437-439; Oct10_2026Users row 1787. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 23, 2025 Q3 ISEAdmin row 58, 2026 Q1 CISCO Network Administrators row 110, 2026 Q1 ISEAdmin row 133; 5_Exceptions row 11. This workbook: 2_Item Detail.</v>
+      </c>
+      <c r="E61" s="19"/>
+      <c r="F61" s="19"/>
+      <c r="G61" s="19"/>
+      <c r="H61" s="19"/>
+      <c r="I61" s="19"/>
+      <c r="J61" s="19"/>
+      <c r="K61" s="19"/>
+      <c r="L61" s="19"/>
+      <c r="M61" s="19"/>
+      <c r="N61" s="19"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="17" t="s">
+        <v>420</v>
+      </c>
+      <c r="B63" s="17"/>
+      <c r="C63" s="17"/>
+      <c r="D63" s="17"/>
+      <c r="E63" s="17"/>
+      <c r="F63" s="17"/>
+      <c r="G63" s="17"/>
+      <c r="H63" s="17"/>
+      <c r="I63" s="17"/>
+      <c r="J63" s="17"/>
+      <c r="K63" s="17"/>
+      <c r="L63" s="17"/>
+      <c r="M63" s="17"/>
+      <c r="N63" s="17"/>
+    </row>
+    <row r="64" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="18" t="s">
+        <v>406</v>
+      </c>
+      <c r="B64" s="18"/>
+      <c r="C64" s="18"/>
+      <c r="D64" s="19" t="str">
+        <f aca="false">"Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), "&amp;J9&amp;", "&amp;K9&amp;". No Revoked decision in any review."</f>
+        <v>Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), Approved 7/27/26, 12:45 PM (Borges, Dayam), Approved 8/17/26, 9:23 AM (Borges, Dayam). No Revoked decision in any review.</v>
+      </c>
+      <c r="E64" s="19"/>
+      <c r="F64" s="19"/>
+      <c r="G64" s="19"/>
+      <c r="H64" s="19"/>
+      <c r="I64" s="19"/>
+      <c r="J64" s="19"/>
+      <c r="K64" s="19"/>
+      <c r="L64" s="19"/>
+      <c r="M64" s="19"/>
+      <c r="N64" s="19"/>
+    </row>
+    <row r="65" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="18" t="s">
+        <v>407</v>
+      </c>
+      <c r="B65" s="18"/>
+      <c r="C65" s="18"/>
+      <c r="D65" s="19" t="s">
+        <v>408</v>
+      </c>
+      <c r="E65" s="19"/>
+      <c r="F65" s="19"/>
+      <c r="G65" s="19"/>
+      <c r="H65" s="19"/>
+      <c r="I65" s="19"/>
+      <c r="J65" s="19"/>
+      <c r="K65" s="19"/>
+      <c r="L65" s="19"/>
+      <c r="M65" s="19"/>
+      <c r="N65" s="19"/>
+    </row>
+    <row r="66" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="18" t="s">
+        <v>409</v>
+      </c>
+      <c r="B66" s="18"/>
+      <c r="C66" s="18"/>
+      <c r="D66" s="20" t="str">
+        <f aca="false">"NO - SLA not met. IAMS termination date "&amp;TEXT(D9,"mm/dd/yyyy")&amp;"; removal was due by "&amp;TEXT(O9,"mm/dd/yyyy")&amp;" (30 business days after the 08/28/2025 review) and access was still held on "&amp;TEXT(Q9,"mm/dd/yyyy")&amp;", "&amp;R9&amp;" business days past the deadline."</f>
+        <v>NO - SLA not met. IAMS termination date 12/31/2024; removal was due by 10/10/2025 (30 business days after the 08/28/2025 review) and access was still held on 08/17/2026, 211 business days past the deadline.</v>
+      </c>
+      <c r="E66" s="20"/>
+      <c r="F66" s="20"/>
+      <c r="G66" s="20"/>
+      <c r="H66" s="20"/>
+      <c r="I66" s="20"/>
+      <c r="J66" s="20"/>
+      <c r="K66" s="20"/>
+      <c r="L66" s="20"/>
+      <c r="M66" s="20"/>
+      <c r="N66" s="20"/>
+    </row>
+    <row r="67" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B67" s="18"/>
+      <c r="C67" s="18"/>
+      <c r="D67" s="19" t="s">
+        <v>410</v>
+      </c>
+      <c r="E67" s="19"/>
+      <c r="F67" s="19"/>
+      <c r="G67" s="19"/>
+      <c r="H67" s="19"/>
+      <c r="I67" s="19"/>
+      <c r="J67" s="19"/>
+      <c r="K67" s="19"/>
+      <c r="L67" s="19"/>
+      <c r="M67" s="19"/>
+      <c r="N67" s="19"/>
+    </row>
+    <row r="68" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="B68" s="18"/>
+      <c r="C68" s="18"/>
+      <c r="D68" s="19" t="str">
+        <f aca="false">"C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = "&amp;IF(G9,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
+        <v>C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = TRUE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
+      </c>
+      <c r="E68" s="19"/>
+      <c r="F68" s="19"/>
+      <c r="G68" s="19"/>
+      <c r="H68" s="19"/>
+      <c r="I68" s="19"/>
+      <c r="J68" s="19"/>
+      <c r="K68" s="19"/>
+      <c r="L68" s="19"/>
+      <c r="M68" s="19"/>
+      <c r="N68" s="19"/>
+    </row>
+    <row r="69" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B69" s="18"/>
+      <c r="C69" s="18"/>
+      <c r="D69" s="20" t="s">
+        <v>421</v>
+      </c>
+      <c r="E69" s="20"/>
+      <c r="F69" s="20"/>
+      <c r="G69" s="20"/>
+      <c r="H69" s="20"/>
+      <c r="I69" s="20"/>
+      <c r="J69" s="20"/>
+      <c r="K69" s="20"/>
+      <c r="L69" s="20"/>
+      <c r="M69" s="20"/>
+      <c r="N69" s="20"/>
+    </row>
+    <row r="70" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="18" t="s">
+        <v>413</v>
+      </c>
+      <c r="B70" s="18"/>
+      <c r="C70" s="18"/>
+      <c r="D70" s="19" t="str">
+        <f aca="false">T9</f>
+        <v>C7.Sample.xlsx: SAMPLE!A142 (screenshots at A143 and A149); 2026Q2PamBsiSox-Manager rows 101-103; 2026Q2BsiPamCyberark-Manager rows 434-436; Oct10_2026Users row 1785. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 24, 2025 Q3 ISEAdmin row 59, 2026 Q1 CISCO Network Administrators row 111, 2026 Q1 ISEAdmin row 134; 5_Exceptions row 12. This workbook: 2_Item Detail.</v>
+      </c>
+      <c r="E70" s="19"/>
+      <c r="F70" s="19"/>
+      <c r="G70" s="19"/>
+      <c r="H70" s="19"/>
+      <c r="I70" s="19"/>
+      <c r="J70" s="19"/>
+      <c r="K70" s="19"/>
+      <c r="L70" s="19"/>
+      <c r="M70" s="19"/>
+      <c r="N70" s="19"/>
+    </row>
+  </sheetData>
+  <mergeCells count="95">
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A12:N12"/>
+    <mergeCell ref="A13:N13"/>
+    <mergeCell ref="A14:N14"/>
+    <mergeCell ref="A15:N15"/>
+    <mergeCell ref="A18:N18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:N19"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="D20:N20"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="D21:N21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="D22:N22"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="D23:N23"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="D24:N24"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="D25:N25"/>
+    <mergeCell ref="A27:N27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="D28:N28"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="D29:N29"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="D30:N30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="D31:N31"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="D32:N32"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="D33:N33"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="D34:N34"/>
+    <mergeCell ref="A36:N36"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="D37:N37"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="D38:N38"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="D39:N39"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="D40:N40"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="D41:N41"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="D42:N42"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="D43:N43"/>
+    <mergeCell ref="A45:N45"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="D46:N46"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="D47:N47"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="D48:N48"/>
+    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="D49:N49"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="D50:N50"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="D51:N51"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="D52:N52"/>
+    <mergeCell ref="A54:N54"/>
+    <mergeCell ref="A55:C55"/>
+    <mergeCell ref="D55:N55"/>
+    <mergeCell ref="A56:C56"/>
+    <mergeCell ref="D56:N56"/>
+    <mergeCell ref="A57:C57"/>
+    <mergeCell ref="D57:N57"/>
+    <mergeCell ref="A58:C58"/>
+    <mergeCell ref="D58:N58"/>
+    <mergeCell ref="A59:C59"/>
+    <mergeCell ref="D59:N59"/>
+    <mergeCell ref="A60:C60"/>
+    <mergeCell ref="D60:N60"/>
+    <mergeCell ref="A61:C61"/>
+    <mergeCell ref="D61:N61"/>
+    <mergeCell ref="A63:N63"/>
+    <mergeCell ref="A64:C64"/>
+    <mergeCell ref="D64:N64"/>
+    <mergeCell ref="A65:C65"/>
+    <mergeCell ref="D65:N65"/>
+    <mergeCell ref="A66:C66"/>
+    <mergeCell ref="D66:N66"/>
+    <mergeCell ref="A67:C67"/>
+    <mergeCell ref="D67:N67"/>
+    <mergeCell ref="A68:C68"/>
+    <mergeCell ref="D68:N68"/>
+    <mergeCell ref="A69:C69"/>
+    <mergeCell ref="D69:N69"/>
+    <mergeCell ref="A70:C70"/>
+    <mergeCell ref="D70:N70"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -6819,127 +8655,175 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>371</v>
+        <v>422</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>372</v>
+        <v>423</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>373</v>
+        <v>424</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="n">
+      <c r="A4" s="21" t="n">
+        <v>45658</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="21" t="n">
+        <v>45677</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="21" t="n">
+        <v>45705</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="21" t="n">
+        <v>45803</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="21" t="n">
+        <v>45827</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="21" t="n">
+        <v>45842</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21" t="n">
         <v>45901</v>
       </c>
-      <c r="B4" s="15" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="n">
+      <c r="B10" s="22" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="n">
         <v>45943</v>
       </c>
-      <c r="B5" s="15" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="n">
+      <c r="B11" s="22" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="n">
         <v>45972</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="n">
+      <c r="B12" s="22" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="21" t="n">
         <v>45988</v>
       </c>
-      <c r="B7" s="15" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="n">
+      <c r="B13" s="22" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21" t="n">
         <v>46016</v>
       </c>
-      <c r="B8" s="15" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="n">
+      <c r="B14" s="22" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="21" t="n">
         <v>46023</v>
       </c>
-      <c r="B9" s="15" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="n">
+      <c r="B15" s="22" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21" t="n">
         <v>46041</v>
       </c>
-      <c r="B10" s="15" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="n">
+      <c r="B16" s="22" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="21" t="n">
         <v>46069</v>
       </c>
-      <c r="B11" s="15" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14" t="n">
+      <c r="B17" s="22" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21" t="n">
         <v>46167</v>
       </c>
-      <c r="B12" s="15" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="n">
+      <c r="B18" s="22" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21" t="n">
         <v>46192</v>
       </c>
-      <c r="B13" s="15" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="14" t="n">
+      <c r="B19" s="22" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="n">
         <v>46206</v>
       </c>
-      <c r="B14" s="15" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="14" t="n">
+      <c r="B20" s="22" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="21" t="n">
         <v>46272</v>
       </c>
-      <c r="B15" s="15" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="n">
+      <c r="B21" s="22" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="21" t="n">
         <v>46307</v>
       </c>
-      <c r="B16" s="15" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="n">
+      <c r="B22" s="22" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21" t="n">
         <v>46337</v>
       </c>
-      <c r="B17" s="15" t="s">
-        <v>376</v>
+      <c r="B23" s="22" t="s">
+        <v>433</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Combine walkthrough with the 2026 Q2 sample tabs and add tab-by-tab review
One workbook with the BSI.IT.27.C7.05 walkthrough tabs, a new
9_Sample Tab Review tab tracing all 10 accounts through every sample
tab and screenshot, the response evaluation and SLA re-performance
tabs, and the SAMPLE / 2026 Q2 certification / AD tabs. Adds the
uncorrelated-identity observation for MIA25172 and MIA25175.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015rwvi2ZZV7Ac5SymUE9zfu
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7.06 Sample Response Evaluation - 2026 Q2.xlsx
+++ b/BSI.IT.27.C7.06 Sample Response Evaluation - 2026 Q2.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1353" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1358" uniqueCount="440">
   <si>
     <t xml:space="preserve">BSI.IT.27.C7 - evaluation of the management response (C7.Sample.xlsx) to the A6 / A5 sample request - 10 accounts</t>
   </si>
@@ -761,7 +761,7 @@
     <t xml:space="preserve">Tried to reconcile the certified network-group memberships to AD and checked the report generation evidence.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cannot be performed: the AD export has user attributes only (name, sAMAccountName, enabled, UPN, employeeID, employeeNumber) - no group membership, whenChanged or account expiration - so certified memberships cannot be reconciled to Cisco Network Administrators / ISEAdmin / CISCO ISE Administrators / F5FullAdmin. Report reliability observations: (a) the export is named Oct10_2026 but the command screenshot is time-stamped 10/13/2026 11:04 AM - the link between the screenshot and the file is not shown; (b) MIA25250 has blank employeeID / employeeNumber, and the SAMPLE tab hard-codes 100592068 instead of the VLOOKUP; (c) Account Status = "Account Removed" on every row, including approved access; (d) 1 AD row has a blank enabled value.</t>
+    <t xml:space="preserve">Cannot be performed: the AD export has user attributes only (name, sAMAccountName, enabled, UPN, employeeID, employeeNumber) - no group membership, whenChanged or account expiration - so certified memberships cannot be reconciled to Cisco Network Administrators / ISEAdmin / CISCO ISE Administrators / F5FullAdmin. Report reliability observations: (a) the export is named Oct10_2026 but the command screenshot is time-stamped 10/13/2026 11:04 AM - the link between the screenshot and the file is not shown; (b) MIA25250 has blank employeeID / employeeNumber, and the SAMPLE tab hard-codes 100592068 instead of the VLOOKUP; (c) Account Status = "Account Removed" on every row, including approved access; (d) 1 AD row has a blank enabled value; (e) MIA25172 and MIA25175 are uncorrelated - Identity = account name (not employee number 100546248 / 100546251) in both 2026 Q2 Manager certifications, so IAMS status is not evaluated for them; (f) SOX = No on every sample row, including the SOX Manager certification.</t>
   </si>
   <si>
     <t xml:space="preserve">Observation (A7)</t>
@@ -984,6 +984,15 @@
   </si>
   <si>
     <t xml:space="preserve">Control owner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MIA25172, MIA25175</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correlate both accounts to their SanIAM identity (AD employeeNumber 100546248 / 100546251). In both 2026 Q2 Manager certifications the Identity field holds the account name, so IAMS termination / inactive status cannot be checked.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uncorrelated accounts escape identity-based leaver controls (A7).</t>
   </si>
   <si>
     <t xml:space="preserve">All</t>
@@ -6432,7 +6441,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -6627,7 +6636,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="n">
         <v>9</v>
       </c>
@@ -6644,6 +6653,26 @@
         <v>314</v>
       </c>
       <c r="F12" s="7" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="F13" s="7" t="s">
         <v>295</v>
       </c>
     </row>
@@ -6671,12 +6700,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6684,7 +6713,7 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6692,17 +6721,17 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6710,32 +6739,32 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6743,7 +6772,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6751,12 +6780,12 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
     </row>
   </sheetData>
@@ -6787,177 +6816,177 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>156</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>349</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>350</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>351</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>144</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>42</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
   </sheetData>
@@ -6994,7 +7023,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7005,58 +7034,58 @@
         <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>141</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7085,22 +7114,22 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>66</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="L4" s="3" t="s">
         <v>151</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>45897</v>
@@ -7125,7 +7154,7 @@
         <v>No - SLA not met</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7154,22 +7183,22 @@
         <v>1</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>66</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>151</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="N5" s="4" t="n">
         <v>45897</v>
@@ -7194,7 +7223,7 @@
         <v>No - SLA not met</v>
       </c>
       <c r="T5" s="3" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7223,22 +7252,22 @@
         <v>1</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>66</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="L6" s="3" t="s">
         <v>151</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>45897</v>
@@ -7263,7 +7292,7 @@
         <v>No - SLA not met</v>
       </c>
       <c r="T6" s="3" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7292,22 +7321,22 @@
         <v>1</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>66</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="L7" s="3" t="s">
         <v>151</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="N7" s="4" t="n">
         <v>45897</v>
@@ -7332,7 +7361,7 @@
         <v>No - SLA not met</v>
       </c>
       <c r="T7" s="3" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7361,22 +7390,22 @@
         <v>1</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>66</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="L8" s="3" t="s">
         <v>151</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>45897</v>
@@ -7401,7 +7430,7 @@
         <v>No - SLA not met</v>
       </c>
       <c r="T8" s="3" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7430,22 +7459,22 @@
         <v>1</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>66</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>151</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="N9" s="4" t="n">
         <v>45897</v>
@@ -7470,12 +7499,12 @@
         <v>No - SLA not met</v>
       </c>
       <c r="T9" s="3" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="15"/>
@@ -7486,7 +7515,7 @@
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="B12" s="16"/>
       <c r="C12" s="16"/>
@@ -7504,7 +7533,7 @@
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
@@ -7522,7 +7551,7 @@
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="B14" s="16"/>
       <c r="C14" s="16"/>
@@ -7540,7 +7569,7 @@
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
@@ -7558,12 +7587,12 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="B18" s="17"/>
       <c r="C18" s="17"/>
@@ -7581,7 +7610,7 @@
     </row>
     <row r="19" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
@@ -7602,12 +7631,12 @@
     </row>
     <row r="20" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="B20" s="18"/>
       <c r="C20" s="18"/>
       <c r="D20" s="19" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="E20" s="19"/>
       <c r="F20" s="19"/>
@@ -7622,7 +7651,7 @@
     </row>
     <row r="21" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="B21" s="18"/>
       <c r="C21" s="18"/>
@@ -7648,7 +7677,7 @@
       <c r="B22" s="18"/>
       <c r="C22" s="18"/>
       <c r="D22" s="19" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="E22" s="19"/>
       <c r="F22" s="19"/>
@@ -7663,7 +7692,7 @@
     </row>
     <row r="23" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="B23" s="18"/>
       <c r="C23" s="18"/>
@@ -7689,7 +7718,7 @@
       <c r="B24" s="18"/>
       <c r="C24" s="18"/>
       <c r="D24" s="20" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="E24" s="20"/>
       <c r="F24" s="20"/>
@@ -7704,7 +7733,7 @@
     </row>
     <row r="25" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -7725,7 +7754,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="17" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="B27" s="17"/>
       <c r="C27" s="17"/>
@@ -7743,7 +7772,7 @@
     </row>
     <row r="28" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="18" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="B28" s="18"/>
       <c r="C28" s="18"/>
@@ -7764,12 +7793,12 @@
     </row>
     <row r="29" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="18" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="B29" s="18"/>
       <c r="C29" s="18"/>
       <c r="D29" s="19" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="E29" s="19"/>
       <c r="F29" s="19"/>
@@ -7784,7 +7813,7 @@
     </row>
     <row r="30" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="18" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="B30" s="18"/>
       <c r="C30" s="18"/>
@@ -7810,7 +7839,7 @@
       <c r="B31" s="18"/>
       <c r="C31" s="18"/>
       <c r="D31" s="19" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="E31" s="19"/>
       <c r="F31" s="19"/>
@@ -7825,7 +7854,7 @@
     </row>
     <row r="32" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="18" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="B32" s="18"/>
       <c r="C32" s="18"/>
@@ -7851,7 +7880,7 @@
       <c r="B33" s="18"/>
       <c r="C33" s="18"/>
       <c r="D33" s="20" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="E33" s="20"/>
       <c r="F33" s="20"/>
@@ -7866,7 +7895,7 @@
     </row>
     <row r="34" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="18" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B34" s="18"/>
       <c r="C34" s="18"/>
@@ -7887,7 +7916,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="17" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="B36" s="17"/>
       <c r="C36" s="17"/>
@@ -7905,7 +7934,7 @@
     </row>
     <row r="37" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="18" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="B37" s="18"/>
       <c r="C37" s="18"/>
@@ -7926,12 +7955,12 @@
     </row>
     <row r="38" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="18" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="B38" s="18"/>
       <c r="C38" s="18"/>
       <c r="D38" s="19" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="E38" s="19"/>
       <c r="F38" s="19"/>
@@ -7946,7 +7975,7 @@
     </row>
     <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="18" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="B39" s="18"/>
       <c r="C39" s="18"/>
@@ -7972,7 +8001,7 @@
       <c r="B40" s="18"/>
       <c r="C40" s="18"/>
       <c r="D40" s="19" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="E40" s="19"/>
       <c r="F40" s="19"/>
@@ -7987,7 +8016,7 @@
     </row>
     <row r="41" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="18" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="B41" s="18"/>
       <c r="C41" s="18"/>
@@ -8013,7 +8042,7 @@
       <c r="B42" s="18"/>
       <c r="C42" s="18"/>
       <c r="D42" s="20" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="E42" s="20"/>
       <c r="F42" s="20"/>
@@ -8028,7 +8057,7 @@
     </row>
     <row r="43" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="18" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B43" s="18"/>
       <c r="C43" s="18"/>
@@ -8049,7 +8078,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="17" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="B45" s="17"/>
       <c r="C45" s="17"/>
@@ -8067,7 +8096,7 @@
     </row>
     <row r="46" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="18" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="B46" s="18"/>
       <c r="C46" s="18"/>
@@ -8088,12 +8117,12 @@
     </row>
     <row r="47" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="18" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="B47" s="18"/>
       <c r="C47" s="18"/>
       <c r="D47" s="19" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="E47" s="19"/>
       <c r="F47" s="19"/>
@@ -8108,7 +8137,7 @@
     </row>
     <row r="48" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="18" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="B48" s="18"/>
       <c r="C48" s="18"/>
@@ -8134,7 +8163,7 @@
       <c r="B49" s="18"/>
       <c r="C49" s="18"/>
       <c r="D49" s="19" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="E49" s="19"/>
       <c r="F49" s="19"/>
@@ -8149,7 +8178,7 @@
     </row>
     <row r="50" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="18" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="B50" s="18"/>
       <c r="C50" s="18"/>
@@ -8175,7 +8204,7 @@
       <c r="B51" s="18"/>
       <c r="C51" s="18"/>
       <c r="D51" s="20" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="E51" s="20"/>
       <c r="F51" s="20"/>
@@ -8190,7 +8219,7 @@
     </row>
     <row r="52" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="18" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B52" s="18"/>
       <c r="C52" s="18"/>
@@ -8211,7 +8240,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="17" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="B54" s="17"/>
       <c r="C54" s="17"/>
@@ -8229,7 +8258,7 @@
     </row>
     <row r="55" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="18" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="B55" s="18"/>
       <c r="C55" s="18"/>
@@ -8250,12 +8279,12 @@
     </row>
     <row r="56" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="18" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="B56" s="18"/>
       <c r="C56" s="18"/>
       <c r="D56" s="19" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="E56" s="19"/>
       <c r="F56" s="19"/>
@@ -8270,7 +8299,7 @@
     </row>
     <row r="57" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="18" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="B57" s="18"/>
       <c r="C57" s="18"/>
@@ -8296,7 +8325,7 @@
       <c r="B58" s="18"/>
       <c r="C58" s="18"/>
       <c r="D58" s="19" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="E58" s="19"/>
       <c r="F58" s="19"/>
@@ -8311,7 +8340,7 @@
     </row>
     <row r="59" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="18" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="B59" s="18"/>
       <c r="C59" s="18"/>
@@ -8337,7 +8366,7 @@
       <c r="B60" s="18"/>
       <c r="C60" s="18"/>
       <c r="D60" s="20" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="E60" s="20"/>
       <c r="F60" s="20"/>
@@ -8352,7 +8381,7 @@
     </row>
     <row r="61" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="18" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B61" s="18"/>
       <c r="C61" s="18"/>
@@ -8373,7 +8402,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="17" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="B63" s="17"/>
       <c r="C63" s="17"/>
@@ -8391,7 +8420,7 @@
     </row>
     <row r="64" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="18" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="B64" s="18"/>
       <c r="C64" s="18"/>
@@ -8412,12 +8441,12 @@
     </row>
     <row r="65" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="18" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="B65" s="18"/>
       <c r="C65" s="18"/>
       <c r="D65" s="19" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="E65" s="19"/>
       <c r="F65" s="19"/>
@@ -8432,7 +8461,7 @@
     </row>
     <row r="66" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="18" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="B66" s="18"/>
       <c r="C66" s="18"/>
@@ -8458,7 +8487,7 @@
       <c r="B67" s="18"/>
       <c r="C67" s="18"/>
       <c r="D67" s="19" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="E67" s="19"/>
       <c r="F67" s="19"/>
@@ -8473,7 +8502,7 @@
     </row>
     <row r="68" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="18" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="B68" s="18"/>
       <c r="C68" s="18"/>
@@ -8499,7 +8528,7 @@
       <c r="B69" s="18"/>
       <c r="C69" s="18"/>
       <c r="D69" s="20" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="E69" s="20"/>
       <c r="F69" s="20"/>
@@ -8514,7 +8543,7 @@
     </row>
     <row r="70" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="18" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B70" s="18"/>
       <c r="C70" s="18"/>
@@ -8655,15 +8684,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8671,7 +8700,7 @@
         <v>45658</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8679,7 +8708,7 @@
         <v>45677</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8687,7 +8716,7 @@
         <v>45705</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8695,7 +8724,7 @@
         <v>45803</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8703,7 +8732,7 @@
         <v>45827</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8711,7 +8740,7 @@
         <v>45842</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8719,7 +8748,7 @@
         <v>45901</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8727,7 +8756,7 @@
         <v>45943</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8735,7 +8764,7 @@
         <v>45972</v>
       </c>
       <c r="B12" s="22" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8743,7 +8772,7 @@
         <v>45988</v>
       </c>
       <c r="B13" s="22" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8751,7 +8780,7 @@
         <v>46016</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8759,7 +8788,7 @@
         <v>46023</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8767,7 +8796,7 @@
         <v>46041</v>
       </c>
       <c r="B16" s="22" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8775,7 +8804,7 @@
         <v>46069</v>
       </c>
       <c r="B17" s="22" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8783,7 +8812,7 @@
         <v>46167</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8791,7 +8820,7 @@
         <v>46192</v>
       </c>
       <c r="B19" s="22" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8799,7 +8828,7 @@
         <v>46206</v>
       </c>
       <c r="B20" s="22" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8807,7 +8836,7 @@
         <v>46272</v>
       </c>
       <c r="B21" s="22" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8815,7 +8844,7 @@
         <v>46307</v>
       </c>
       <c r="B22" s="22" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8823,7 +8852,7 @@
         <v>46337</v>
       </c>
       <c r="B23" s="22" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rework SLA test for the 6 supplemental accounts per IAM Standard and PAM procedure
The 30-business-day review SLA (SUS.IAMS.4.2.5.21) is only triggered by
a Revoked decision, so A6 is N/A for the six approved accounts and the
earlier 'SLA not met' result is withdrawn. The exception is kept under
A5 (PAM Procedure step 9 requires revocation for terminated users), and
the leaver SLA (SUS.IAMS.4.2.4.3) is recorded as an observation pending
HR confirmation. Adds policy citations and a draft reply to the process
owner.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015rwvi2ZZV7Ac5SymUE9zfu
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7.06 Sample Response Evaluation - 2026 Q2.xlsx
+++ b/BSI.IT.27.C7.06 Sample Response Evaluation - 2026 Q2.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1358" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1404" uniqueCount="483">
   <si>
     <t xml:space="preserve">BSI.IT.27.C7 - evaluation of the management response (C7.Sample.xlsx) to the A6 / A5 sample request - 10 accounts</t>
   </si>
@@ -1142,6 +1142,33 @@
     <t xml:space="preserve">a6eee02a47888234ca2afd7662f0fd49</t>
   </si>
   <si>
+    <t xml:space="preserve">CUSO Identity and Access Management Standard v11.0 (BSIIT21.PDF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sec. 4.2.4, 4.2.5, Appendix G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved 07/28/2026; SUS.IAMS.4.2.4.2 / 4.2.4.3 leaver SLAs (1 / 30 business days from termination); 4.2.5.7 / 4.2.5.21 review revocation SLA (30 business days from close of review)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which SLA applies (tab 7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35484fd4951ac6439d9e4aee56437c38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAM_Recertification_Procedure_BSI_04.22.26.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sec. 3, 4.1.1, 8 step 9-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v2.0 approved 04/22/2026; revocation tickets for reject decisions or terminated users; process ends when manager approves</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9eaef168c42e8bd6bdd088432f6bf75a</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sample step taken.docx</t>
   </si>
   <si>
@@ -1154,10 +1181,107 @@
     <t xml:space="preserve">478b98cad0b66e5989c71e3ee9f1bef3</t>
   </si>
   <si>
-    <t xml:space="preserve">Re-performance - 30-business-day SLA for the 6 supplemental accounts (Ivan Ramirez Gonzalez, Jefferson Paez Venegas, David Serrano Aguirre, Maiko Vazquez Arias, Richard Harris, Kevin Ackley)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Identity (SanIAM)</t>
+    <t xml:space="preserve">SLA re-performance for the 6 supplemental accounts, based on the IAM Standard and the PAM Recertification Procedure (responds to the process owner's challenge)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A. Process owner's challenge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"If the access is approved, what SLA is being measured? The SLA only starts if the access is revoked. Approved access has no action; only revoked access needs action. The workpaper says none of the 6 accounts was revoked, so the SLA clock never started, but then concludes 'No - SLA not met' using the first review after termination as the trigger date."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B. Policy analysis - which SLA applies to the 6 accounts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Question</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Policy text (exact)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the 30-business-day review SLA apply to access that was approved?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Any revocation of privileged access rights resulting from the privileged access review outcomes must be completed within 30 business days of the close of the review per the SLA." (4.2.5.21)
+"Any revocations of access rights must be completed within 30 business days per the SLA." (4.2.5.7)
+"When all assignees have completed their decisions, if the manager approves the user access, the process ends." (PAM step 9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CUSO Identity and Access Management Standard v11.0 (approved 07/28/2026) SUS.IAMS.4.2.5.21 (p.22), SUS.IAMS.4.2.5.7 (p.18); BSI PAM Recertification Procedure v2.0 (approved 04/22/2026) sec. 4.1.1 C3-C4 (p.6), sec. 8 step 9 (p.10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. The 30-business-day clock starts at the close of the review and only for a revocation that results from the review outcome. All 6 accounts were Approved in every review, so no revocation was raised and no SLA clock started.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Process owner is CORRECT. The prior "No - SLA not met (211 business days)" result is WITHDRAWN. A6 (revocation within SLA) = N/A for the 6 accounts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Did the procedure still require these accounts to be revoked at the review?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"If access is revoked, the PAM team submits revocation tickets for any 'reject' decision or terminated users." (PAM step 9)
+"The recertification process must be performed as a formal review of information assets to confirm that all granted access rights entitlements remain valid" (4.2.5.1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSI PAM Recertification Procedure v2.0 (approved 04/22/2026) sec. 8 step 9 (p.10), sec. 3 PAM US Team; CUSO Identity and Access Management Standard v11.0 (approved 07/28/2026) SUS.IAMS.4.2.5.1 (p.14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes, if the identities were terminated. Step 9 names terminated users alongside reject decisions as a revocation trigger, and 4.2.5.1 requires the review to confirm access remains valid. IAMS shows Termination Date 12/31/2024 for all 6; the reviewer approved and PAM raised no revocation ticket in 2025 Q3, 2026 Q1 or 2026 Q2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exception stands as A5 (appropriateness / control execution), NOT as an SLA (A6) failure: the review did not identify and revoke access of terminated identities.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is there an SLA for terminated users that does not depend on a Revoked decision?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Network Access for terminated users must be in line with the SLAs defined in the SLA matrix" (4.2.4.2) - Appendix G: disable AD access, 1 business day.
+"Privileged access and control plane access for terminated users must be in line with the SLAs defined in the SLA matrix ... If ... the SLA is missed, initiate a look-back assessment" (4.2.4.3) - Appendix G: 30 business days.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CUSO Identity and Access Management Standard v11.0 (approved 07/28/2026) SUS.IAMS.4.2.4.2 and 4.2.4.3 (p.12-13), Appendix G SLA Matrix (p.46, 53)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes, but it is the leaver (de-provisioning) SLA, triggered by the termination date and owned by IAM/PAM under 4.2.4 - not by the C7 review. If the 12/31/2024 termination is confirmed, the deadlines were 01/02/2025 (AD) and 02/13/2025 (privileged access) and both were missed; a look-back of use after termination is required.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not rated in C7 A6. Report as an observation and refer to the leaver / de-provisioning control owner, pending HR confirmation (item 4).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the 12/31/2024 termination real?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAMS: Termination Date 12/31/2024, Identity Inactive = FALSE, Assignee Employee Status = A (2026 Q2 exports). AD: expiration 01/01/2026 then 06/01/2026, logons in Nov 2025 (walkthrough). CyberArk safes are named Alero_Consultant_* / Alero_Protect-* (external consultants).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7.Sample.xlsx 2026 Q2 Manager tabs; walkthrough 4_Item Detail, 7_Evidence Status #4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not confirmed. The data suggest consultants whose contract end date was not updated in IAMS after an extension. HR / vendor contract evidence is still outstanding.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If contracts were active: items 2-3 become an IAMS data-quality observation, except MIA25103 (below). If terminated: A5 exception + leaver SLA observation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MIA25103 (Ivan Ramirez Gonzalez) - AD disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AD enabled = FALSE on 11/25/2025, 05/15/2026 and 10/10/2026; last logon 10/15/2023. Still a member of Cisco Network Administrators / ISEAdmin and approved on 7/27/2026 and 8/17/2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7.Sample.xlsx Oct10_2026Users row 1598; Sox-Manager rows 86-88; CyberArk-Manager rows 419-421</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disabled account kept privileged network group membership and was re-approved. The review SLA does not apply (no revocation), but the review failed to identify an inactive account.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exception A5 (E1) stands regardless of the HR outcome.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C. Re-performance per account - three tests (formulas in green-shaded result columns)</t>
   </si>
   <si>
     <t xml:space="preserve">IAMS Termination Date</t>
@@ -1169,91 +1293,85 @@
     <t xml:space="preserve">AD enabled 05/15/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">2025 Q3 decision</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 Q1 decision</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 Q2 SOX Manager decision</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 Q2 CyberArk Manager decision</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Revocation raised in any review?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Access removal date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLA trigger date (first review after termination)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLA deadline (trigger + 30 business days)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deadline if measured from termination date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Access still held on (latest evidence)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Business days past SLA deadline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLA followed?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference (file / tab / rows)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Approved 08/28/2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Approved 7/27/26, 12:45 PM (Borges, Dayam)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Approved 8/17/26, 9:23 AM (Borges, Dayam)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">None - access not removed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A72 (screenshots at A73 and A79); 2026Q2PamBsiSox-Manager rows 86-88; 2026Q2BsiPamCyberark-Manager rows 419-421; Oct10_2026Users row 1598. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 15, 2025 Q3 ISEAdmin row 53, 2026 Q1 CISCO Network Administrators row 103, 2026 Q1 ISEAdmin row 126; 5_Exceptions row 4. This workbook: 2_Item Detail.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A86 (screenshots at A87 and A93); 2026Q2PamBsiSox-Manager rows 89-91; 2026Q2BsiPamCyberark-Manager rows 422-424; Oct10_2026Users row 1596. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 16, 2025 Q3 ISEAdmin row 54, 2026 Q1 CISCO Network Administrators row 104, 2026 Q1 ISEAdmin row 127; 5_Exceptions row 5. This workbook: 2_Item Detail.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A100 (screenshots at A101 and A107); 2026Q2PamBsiSox-Manager rows 92-94; 2026Q2BsiPamCyberark-Manager rows 425-427; Oct10_2026Users row 1599. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 17, 2025 Q3 ISEAdmin row 55, 2026 Q1 CISCO Network Administrators row 105, 2026 Q1 ISEAdmin row 128; 5_Exceptions row 6. This workbook: 2_Item Detail.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A114 (screenshots at A115 and A121); 2026Q2PamBsiSox-Manager rows 95-97; 2026Q2BsiPamCyberark-Manager rows 428-430; Oct10_2026Users row 1597. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 18, 2025 Q3 ISEAdmin row 56, 2026 Q1 CISCO Network Administrators row 106, 2026 Q1 ISEAdmin row 129; 5_Exceptions row 7. This workbook: 2_Item Detail.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A128 (screenshots at A129 and A135); 2026Q2PamBsiSox-Manager rows 104-106; 2026Q2BsiPamCyberark-Manager rows 437-439; Oct10_2026Users row 1787. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 23, 2025 Q3 ISEAdmin row 58, 2026 Q1 CISCO Network Administrators row 110, 2026 Q1 ISEAdmin row 133; 5_Exceptions row 11. This workbook: 2_Item Detail.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A142 (screenshots at A143 and A149); 2026Q2PamBsiSox-Manager rows 101-103; 2026Q2BsiPamCyberark-Manager rows 434-436; Oct10_2026Users row 1785. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 24, 2025 Q3 ISEAdmin row 59, 2026 Q1 CISCO Network Administrators row 111, 2026 Q1 ISEAdmin row 134; 5_Exceptions row 12. This workbook: 2_Item Detail.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Accounts not following the SLA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">How the SLA was measured: none of the 6 accounts was revoked, so the SLA clock never started from a "Revoked" decision. Under PAM Recertification Procedure sec. 8 step 9 (revocation for rejects or terminated users) and IAM Standard SUS.IAMS.4.2.5.7 / 4.2.5.21, access of a terminated identity must be revoked at the review and removed within 30 business days.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The trigger is therefore the first certification decision after the IAMS termination date (12/31/2024): the 2025 Q3 decision on 08/28/2025, giving a deadline of 10/10/2025. Column P shows the stricter deadline counted from the termination date itself.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Access still held on: 08/17/2026 = the latest certification in C7.Sample.xlsx (2026 Q2 CyberArk Manager) in which each account is still listed with Cisco Network Administrators / ISEAdmin and Approved. The 10/10/2026 AD export has no group data, so membership after 08/17/2026 is not evidenced.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blue text = inputs (dates from the certification exports / walkthrough). Columns O, P, R, S are formulas over the Holidays tab.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Answer to the test step, per account (with reference)</t>
+    <t xml:space="preserve">Revoked decision in any review?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decisions (2025 Q3 / 2026 Q1 / 2026 Q2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEST 1 - Review revocation SLA (4.2.5.21, 30 bd from close of review)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEST 2 - Terminated-user revocation at review (PAM step 9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revocation ticket raised?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leaver deadline - AD disable (4.2.4.2, 1 bd)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leaver deadline - privileged access (4.2.4.3, 30 bd)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Privileged access still held on</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Business days past leaver deadline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEST 3 - Leaver SLA (4.2.4.3) - if termination confirmed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overall result</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved 08/28/2025 / Approved 04/30/2026 / Approved 7/27/26, 12:45 PM (SOX) and 8/17/26, 9:23 AM (CyberArk)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No - none in any tab (WorkItemID blank)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exception A5 (E1, E2) - disabled and IAMS-terminated account approved; no revocation ticket. A6 N/A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A72 (screenshots A73, A79); 2026Q2PamBsiSox-Manager rows 86-88; 2026Q2BsiPamCyberark-Manager rows 419-421; Oct10_2026Users row 1598. Walkthrough: 4_Item Detail 2025 Q3 CISCO Network Administrators row 15, 2025 Q3 ISEAdmin row 53, 2026 Q1 CISCO Network Administrators row 103, 2026 Q1 ISEAdmin row 126; 5_Exceptions row 4. Policy: section B above.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exception A5 (E2) - IAMS-terminated identity approved; no revocation ticket. A6 N/A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A86 (screenshots A87, A93); 2026Q2PamBsiSox-Manager rows 89-91; 2026Q2BsiPamCyberark-Manager rows 422-424; Oct10_2026Users row 1596. Walkthrough: 4_Item Detail 2025 Q3 CISCO Network Administrators row 16, 2025 Q3 ISEAdmin row 54, 2026 Q1 CISCO Network Administrators row 104, 2026 Q1 ISEAdmin row 127; 5_Exceptions row 5. Policy: section B above.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A100 (screenshots A101, A107); 2026Q2PamBsiSox-Manager rows 92-94; 2026Q2BsiPamCyberark-Manager rows 425-427; Oct10_2026Users row 1599. Walkthrough: 4_Item Detail 2025 Q3 CISCO Network Administrators row 17, 2025 Q3 ISEAdmin row 55, 2026 Q1 CISCO Network Administrators row 105, 2026 Q1 ISEAdmin row 128; 5_Exceptions row 6. Policy: section B above.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A114 (screenshots A115, A121); 2026Q2PamBsiSox-Manager rows 95-97; 2026Q2BsiPamCyberark-Manager rows 428-430; Oct10_2026Users row 1597. Walkthrough: 4_Item Detail 2025 Q3 CISCO Network Administrators row 18, 2025 Q3 ISEAdmin row 56, 2026 Q1 CISCO Network Administrators row 106, 2026 Q1 ISEAdmin row 129; 5_Exceptions row 7. Policy: section B above.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exception A5 (E1, E2) - re-enabled after 05/15/2026; IAMS-terminated identity approved; no revocation ticket. A6 N/A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A128 (screenshots A129, A135); 2026Q2PamBsiSox-Manager rows 104-106; 2026Q2BsiPamCyberark-Manager rows 437-439; Oct10_2026Users row 1787. Walkthrough: 4_Item Detail 2025 Q3 CISCO Network Administrators row 23, 2025 Q3 ISEAdmin row 58, 2026 Q1 CISCO Network Administrators row 110, 2026 Q1 ISEAdmin row 133; 5_Exceptions row 11. Policy: section B above.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7.Sample.xlsx: SAMPLE!A142 (screenshots A143, A149); 2026Q2PamBsiSox-Manager rows 101-103; 2026Q2BsiPamCyberark-Manager rows 434-436; Oct10_2026Users row 1785. Walkthrough: 4_Item Detail 2025 Q3 CISCO Network Administrators row 24, 2025 Q3 ISEAdmin row 59, 2026 Q1 CISCO Network Administrators row 111, 2026 Q1 ISEAdmin row 134; 5_Exceptions row 12. Policy: section B above.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEST 1 - accounts failing the 30-business-day review SLA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEST 2 - accounts failing terminated-user revocation at review (A5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEST 3 - leaver SLA missed if termination is confirmed (observation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue = inputs: IAMS Termination Date from the 2026 Q2 Manager certifications; 08/17/2026 = latest certification (2026 Q2 CyberArk Manager) in which each account still holds Cisco Network Administrators / ISEAdmin. The 10/10/2026 AD export has no group data, so membership after 08/17/2026 is not evidenced. Business days exclude the US bank holidays on the Holidays tab.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D. Answer to the test step, per account (with reference)</t>
   </si>
   <si>
     <t xml:space="preserve">Ivan Ramirez Gonzalez (MIA25103)</t>
@@ -1265,28 +1383,28 @@
     <t xml:space="preserve">Date access was removed (if revoked)</t>
   </si>
   <si>
-    <t xml:space="preserve">Not removed. No revocation was raised, and the account is still listed with Cisco Network Administrators, ISEAdmin and CYBERARK_ALERO_USERS in the 2026 Q2 certifications.</t>
+    <t xml:space="preserve">N/A - not revoked. The account still holds Cisco Network Administrators, ISEAdmin and CYBERARK_ALERO_USERS in the 2026 Q2 certifications.</t>
   </si>
   <si>
     <t xml:space="preserve">Removal within the 30-business-day SLA?</t>
   </si>
   <si>
-    <t xml:space="preserve">N/A - access was never removed and no remediation is evidenced.</t>
+    <t xml:space="preserve">N/A - the 30-business-day SLA (SUS.IAMS.4.2.5.21; PAM Procedure 4.1.1 C3-C4) starts only from a Revoked decision at the close of the review. No revocation was decided, so no SLA was triggered and A6 is not rated for this account.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/A - access was never removed.</t>
   </si>
   <si>
     <t xml:space="preserve">Supporting evidence</t>
   </si>
   <si>
-    <t xml:space="preserve">Exception - A5 (terminated identity approved) and A6 (access not removed within SLA). The AD account is also disabled (11/25/2025, 05/15/2026, 10/10/2026) yet still holds and is re-approved for privileged network access. Root cause: the reviewer approved instead of revoking, so the PAM/IAM revocation and SLA process was never triggered.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference</t>
+    <t xml:space="preserve">Exception A5 - not an SLA exception. IAMS shows termination 12/31/2024; under PAM Procedure sec. 8 step 9 terminated users require a PAM revocation ticket, but the reviewer approved and none was raised. The AD account is disabled (11/25/2025, 05/15/2026, 10/10/2026) yet keeps and is re-approved for privileged network access - E1 stands even if the contract was active. If HR confirms the termination, the leaver SLA (SUS.IAMS.4.2.4.3, 30 business days from termination) was also missed - refer to the leaver control owner and request a look-back.</t>
   </si>
   <si>
     <t xml:space="preserve">Jefferson Paez Venegas (MIA25104)</t>
   </si>
   <si>
-    <t xml:space="preserve">Exception - A5 (terminated identity approved) and A6 (access not removed within SLA). Root cause: the reviewer approved instead of revoking, so the PAM/IAM revocation and SLA process was never triggered.</t>
+    <t xml:space="preserve">Exception A5 - not an SLA exception. IAMS shows termination 12/31/2024; under PAM Procedure sec. 8 step 9 terminated users require a PAM revocation ticket, but the reviewer approved and none was raised. If HR confirms the termination, the leaver SLA (SUS.IAMS.4.2.4.3, 30 business days from termination) was also missed - refer to the leaver control owner and request a look-back.</t>
   </si>
   <si>
     <t xml:space="preserve">David Serrano Aguirre (MIA25105)</t>
@@ -1298,13 +1416,28 @@
     <t xml:space="preserve">Richard Harris (MIA25249)</t>
   </si>
   <si>
-    <t xml:space="preserve">Exception - A5 (terminated identity approved) and A6 (access not removed within SLA). AD shows the account disabled on 05/15/2026 and enabled again on 10/10/2026, with no request or audit event provided. Root cause: the reviewer approved instead of revoking, so the PAM/IAM revocation and SLA process was never triggered.</t>
+    <t xml:space="preserve">Exception A5 - not an SLA exception. IAMS shows termination 12/31/2024; under PAM Procedure sec. 8 step 9 terminated users require a PAM revocation ticket, but the reviewer approved and none was raised. AD shows the account disabled on 05/15/2026 and enabled again on 10/10/2026, with no request or audit event provided. If HR confirms the termination, the leaver SLA (SUS.IAMS.4.2.4.3, 30 business days from termination) was also missed - refer to the leaver control owner and request a look-back.</t>
   </si>
   <si>
     <t xml:space="preserve">Kevin Ackley (MIA25250)</t>
   </si>
   <si>
-    <t xml:space="preserve">Exception - A5 (terminated identity approved) and A6 (access not removed within SLA). AD shows the account disabled on 05/15/2026 and enabled again on 10/10/2026, with no request or audit event provided. AD employeeID / employeeNumber are blank, so the SAMPLE tab hard-codes identity 100592068. Root cause: the reviewer approved instead of revoking, so the PAM/IAM revocation and SLA process was never triggered.</t>
+    <t xml:space="preserve">Exception A5 - not an SLA exception. IAMS shows termination 12/31/2024; under PAM Procedure sec. 8 step 9 terminated users require a PAM revocation ticket, but the reviewer approved and none was raised. AD shows the account disabled on 05/15/2026 and enabled again on 10/10/2026, with no request or audit event provided. AD employeeID / employeeNumber are blank, so the SAMPLE tab hard-codes identity 100592068. If HR confirms the termination, the leaver SLA (SUS.IAMS.4.2.4.3, 30 business days from termination) was also missed - refer to the leaver control owner and request a look-back.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E. Draft response to the process owner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We agree. Under SUS.IAMS.4.2.5.21 the 30-business-day SLA applies to "any revocation of privileged access rights resulting from the privileged access review outcomes", measured from the close of the review, and PAM Procedure step 9 ends the process when the manager approves. None of the 6 accounts (MIA25103, MIA25104, MIA25105, MIA25106, MIA25249, MIA25250) was revoked, so no SLA was triggered. We have withdrawn the "SLA not met" result, and these accounts are no longer rated under A6 (revocation within SLA).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The exception remains, but under A5 (appropriateness of the review outcome). PAM Procedure sec. 8 step 9 requires the PAM team to submit revocation tickets "for any 'reject' decision or terminated users", and SUS.IAMS.4.2.5.1 requires the review to confirm that access remains valid. All 6 identities show IAMS Termination Date 12/31/2024, and MIA25103 is disabled in AD. All were approved in 2025 Q3, 2026 Q1 and 2026 Q2, and no revocation ticket was raised.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Separately, SUS.IAMS.4.2.4.2 / 4.2.4.3 and Appendix G set leaver SLAs from the termination date (1 business day to disable AD; 30 business days to revoke privileged access), with a look-back if missed. We are not rating that in C7. If HR confirms the terminations, we will refer it to the de-provisioning control owner.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To close the point, please provide: (1) HR / vendor contract evidence of the engagement status for the 6 accounts on 08/28/2025, 04/30/2026 and 07/27/2026, and why IAMS still shows 12/31/2024; (2) the reason MIA25103 (AD-disabled) kept and was re-approved for privileged network access; (3) the request / approval for re-enabling MIA25249 and MIA25250 after 05/15/2026.</t>
   </si>
   <si>
     <t xml:space="preserve">US bank holidays (Federal Reserve) used for the 30-business-day SLA</t>
@@ -1361,7 +1494,7 @@
     <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="166" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1421,6 +1554,20 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -1508,7 +1655,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1565,6 +1712,14 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1586,10 +1741,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6804,7 +6955,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -6972,21 +7123,55 @@
         <v>369</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
         <v>370</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>372</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>371</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>372</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>373</v>
+      <c r="C14" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>382</v>
       </c>
     </row>
   </sheetData>
@@ -7005,801 +7190,726 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T70"/>
+  <dimension ref="A1:R87"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="10" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="14" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="12" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="14" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="15" t="s">
+        <v>385</v>
+      </c>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="J8" s="3"/>
+      <c r="K8" s="12" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="J9" s="3"/>
+      <c r="K9" s="6" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="J10" s="3"/>
+      <c r="K10" s="7" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="J11" s="3"/>
+      <c r="K11" s="7" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="J12" s="3"/>
+      <c r="K12" s="6" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="14" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B15" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>375</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>376</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="G3" s="2" t="s">
+      <c r="C15" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>379</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>381</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>382</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>385</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>386</v>
-      </c>
-      <c r="P3" s="2" t="s">
-        <v>387</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>388</v>
-      </c>
-      <c r="R3" s="2" t="s">
+      <c r="G15" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="O15" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="P15" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="Q15" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="R15" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="S3" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B16" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C4" s="3" t="n">
-        <v>100531048</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="C16" s="4" t="n">
         <v>45657</v>
       </c>
-      <c r="E4" s="14" t="b">
+      <c r="D16" s="16" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="F4" s="14" t="b">
+      <c r="E16" s="16" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G4" s="14" t="b">
+      <c r="F16" s="16" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H4" s="3" t="s">
-        <v>392</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>394</v>
-      </c>
-      <c r="L4" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="M4" s="3" t="s">
-        <v>395</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>45897</v>
-      </c>
-      <c r="O4" s="5" t="n">
-        <f aca="false">WORKDAY(N4,30,Holidays!$A$4:$A$23)</f>
-        <v>45940</v>
-      </c>
-      <c r="P4" s="5" t="n">
-        <f aca="false">WORKDAY(D4,30,Holidays!$A$4:$A$23)</f>
+      <c r="H16" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="I16" s="12" t="str">
+        <f aca="false">IF(G16="No","N/A - not triggered: no Revoked decision, no SLA clock","Measure from close of review")</f>
+        <v>N/A - not triggered: no Revoked decision, no SLA clock</v>
+      </c>
+      <c r="J16" s="6" t="str">
+        <f aca="false">IF(AND(C16&lt;&gt;"",K16="No - none in any tab (WorkItemID blank)"),"FAIL - IAMS-terminated identity ("&amp;TEXT(C16,"mm/dd/yyyy")&amp;") approved; PAM raised no revocation ticket","Pass")</f>
+        <v>FAIL - IAMS-terminated identity (12/31/2024) approved; PAM raised no revocation ticket</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="L16" s="5" t="n">
+        <f aca="false">WORKDAY(C16,1,Holidays!$A$4:$A$23)</f>
+        <v>45659</v>
+      </c>
+      <c r="M16" s="5" t="n">
+        <f aca="false">WORKDAY(C16,30,Holidays!$A$4:$A$23)</f>
         <v>45701</v>
       </c>
-      <c r="Q4" s="4" t="n">
+      <c r="N16" s="4" t="n">
         <v>46251</v>
       </c>
-      <c r="R4" s="3" t="n">
-        <f aca="false">IF(Q4&gt;O4,NETWORKDAYS(O4+1,Q4,Holidays!$A$4:$A$23),0)</f>
-        <v>211</v>
-      </c>
-      <c r="S4" s="6" t="str">
-        <f aca="false">IF(AND(L4="No",Q4&gt;O4),"No - SLA not met",IF(R4=0,"Yes","No - late"))</f>
-        <v>No - SLA not met</v>
-      </c>
-      <c r="T4" s="3" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="O16" s="3" t="n">
+        <f aca="false">IF(N16&gt;M16,NETWORKDAYS(M16+1,N16,Holidays!$A$4:$A$23),0)</f>
+        <v>377</v>
+      </c>
+      <c r="P16" s="7" t="str">
+        <f aca="false">IF(O16&gt;0,"Missed by "&amp;O16&amp;" business days IF termination is confirmed - leaver control observation, look-back required (4.2.4.3)","Met")</f>
+        <v>Missed by 377 business days IF termination is confirmed - leaver control observation, look-back required (4.2.4.3)</v>
+      </c>
+      <c r="Q16" s="6" t="s">
+        <v>432</v>
+      </c>
+      <c r="R16" s="3" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B17" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C5" s="3" t="n">
-        <v>100531049</v>
-      </c>
-      <c r="D5" s="4" t="n">
+      <c r="C17" s="4" t="n">
         <v>45657</v>
       </c>
-      <c r="E5" s="11" t="b">
+      <c r="D17" s="11" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="F5" s="11" t="b">
+      <c r="E17" s="11" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="G5" s="11" t="b">
+      <c r="F17" s="11" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H5" s="3" t="s">
-        <v>392</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>394</v>
-      </c>
-      <c r="L5" s="3" t="s">
+      <c r="G17" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="M5" s="3" t="s">
-        <v>395</v>
-      </c>
-      <c r="N5" s="4" t="n">
-        <v>45897</v>
-      </c>
-      <c r="O5" s="5" t="n">
-        <f aca="false">WORKDAY(N5,30,Holidays!$A$4:$A$23)</f>
-        <v>45940</v>
-      </c>
-      <c r="P5" s="5" t="n">
-        <f aca="false">WORKDAY(D5,30,Holidays!$A$4:$A$23)</f>
+      <c r="H17" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="I17" s="12" t="str">
+        <f aca="false">IF(G17="No","N/A - not triggered: no Revoked decision, no SLA clock","Measure from close of review")</f>
+        <v>N/A - not triggered: no Revoked decision, no SLA clock</v>
+      </c>
+      <c r="J17" s="6" t="str">
+        <f aca="false">IF(AND(C17&lt;&gt;"",K17="No - none in any tab (WorkItemID blank)"),"FAIL - IAMS-terminated identity ("&amp;TEXT(C17,"mm/dd/yyyy")&amp;") approved; PAM raised no revocation ticket","Pass")</f>
+        <v>FAIL - IAMS-terminated identity (12/31/2024) approved; PAM raised no revocation ticket</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="L17" s="5" t="n">
+        <f aca="false">WORKDAY(C17,1,Holidays!$A$4:$A$23)</f>
+        <v>45659</v>
+      </c>
+      <c r="M17" s="5" t="n">
+        <f aca="false">WORKDAY(C17,30,Holidays!$A$4:$A$23)</f>
         <v>45701</v>
       </c>
-      <c r="Q5" s="4" t="n">
+      <c r="N17" s="4" t="n">
         <v>46251</v>
       </c>
-      <c r="R5" s="3" t="n">
-        <f aca="false">IF(Q5&gt;O5,NETWORKDAYS(O5+1,Q5,Holidays!$A$4:$A$23),0)</f>
-        <v>211</v>
-      </c>
-      <c r="S5" s="6" t="str">
-        <f aca="false">IF(AND(L5="No",Q5&gt;O5),"No - SLA not met",IF(R5=0,"Yes","No - late"))</f>
-        <v>No - SLA not met</v>
-      </c>
-      <c r="T5" s="3" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="O17" s="3" t="n">
+        <f aca="false">IF(N17&gt;M17,NETWORKDAYS(M17+1,N17,Holidays!$A$4:$A$23),0)</f>
+        <v>377</v>
+      </c>
+      <c r="P17" s="7" t="str">
+        <f aca="false">IF(O17&gt;0,"Missed by "&amp;O17&amp;" business days IF termination is confirmed - leaver control observation, look-back required (4.2.4.3)","Met")</f>
+        <v>Missed by 377 business days IF termination is confirmed - leaver control observation, look-back required (4.2.4.3)</v>
+      </c>
+      <c r="Q17" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="R17" s="3" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B18" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C6" s="3" t="n">
-        <v>100531050</v>
-      </c>
-      <c r="D6" s="4" t="n">
+      <c r="C18" s="4" t="n">
         <v>45657</v>
       </c>
-      <c r="E6" s="11" t="b">
+      <c r="D18" s="11" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="F6" s="11" t="b">
+      <c r="E18" s="11" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="G6" s="11" t="b">
+      <c r="F18" s="11" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H6" s="3" t="s">
-        <v>392</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>394</v>
-      </c>
-      <c r="L6" s="3" t="s">
+      <c r="G18" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="M6" s="3" t="s">
-        <v>395</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>45897</v>
-      </c>
-      <c r="O6" s="5" t="n">
-        <f aca="false">WORKDAY(N6,30,Holidays!$A$4:$A$23)</f>
-        <v>45940</v>
-      </c>
-      <c r="P6" s="5" t="n">
-        <f aca="false">WORKDAY(D6,30,Holidays!$A$4:$A$23)</f>
+      <c r="H18" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="I18" s="12" t="str">
+        <f aca="false">IF(G18="No","N/A - not triggered: no Revoked decision, no SLA clock","Measure from close of review")</f>
+        <v>N/A - not triggered: no Revoked decision, no SLA clock</v>
+      </c>
+      <c r="J18" s="6" t="str">
+        <f aca="false">IF(AND(C18&lt;&gt;"",K18="No - none in any tab (WorkItemID blank)"),"FAIL - IAMS-terminated identity ("&amp;TEXT(C18,"mm/dd/yyyy")&amp;") approved; PAM raised no revocation ticket","Pass")</f>
+        <v>FAIL - IAMS-terminated identity (12/31/2024) approved; PAM raised no revocation ticket</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="L18" s="5" t="n">
+        <f aca="false">WORKDAY(C18,1,Holidays!$A$4:$A$23)</f>
+        <v>45659</v>
+      </c>
+      <c r="M18" s="5" t="n">
+        <f aca="false">WORKDAY(C18,30,Holidays!$A$4:$A$23)</f>
         <v>45701</v>
       </c>
-      <c r="Q6" s="4" t="n">
+      <c r="N18" s="4" t="n">
         <v>46251</v>
       </c>
-      <c r="R6" s="3" t="n">
-        <f aca="false">IF(Q6&gt;O6,NETWORKDAYS(O6+1,Q6,Holidays!$A$4:$A$23),0)</f>
-        <v>211</v>
-      </c>
-      <c r="S6" s="6" t="str">
-        <f aca="false">IF(AND(L6="No",Q6&gt;O6),"No - SLA not met",IF(R6=0,"Yes","No - late"))</f>
-        <v>No - SLA not met</v>
-      </c>
-      <c r="T6" s="3" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="O18" s="3" t="n">
+        <f aca="false">IF(N18&gt;M18,NETWORKDAYS(M18+1,N18,Holidays!$A$4:$A$23),0)</f>
+        <v>377</v>
+      </c>
+      <c r="P18" s="7" t="str">
+        <f aca="false">IF(O18&gt;0,"Missed by "&amp;O18&amp;" business days IF termination is confirmed - leaver control observation, look-back required (4.2.4.3)","Met")</f>
+        <v>Missed by 377 business days IF termination is confirmed - leaver control observation, look-back required (4.2.4.3)</v>
+      </c>
+      <c r="Q18" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="R18" s="3" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B19" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C7" s="3" t="n">
-        <v>100531051</v>
-      </c>
-      <c r="D7" s="4" t="n">
+      <c r="C19" s="4" t="n">
         <v>45657</v>
       </c>
-      <c r="E7" s="11" t="b">
+      <c r="D19" s="11" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="F7" s="11" t="b">
+      <c r="E19" s="11" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="G7" s="11" t="b">
+      <c r="F19" s="11" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H7" s="3" t="s">
-        <v>392</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>394</v>
-      </c>
-      <c r="L7" s="3" t="s">
+      <c r="G19" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="M7" s="3" t="s">
-        <v>395</v>
-      </c>
-      <c r="N7" s="4" t="n">
-        <v>45897</v>
-      </c>
-      <c r="O7" s="5" t="n">
-        <f aca="false">WORKDAY(N7,30,Holidays!$A$4:$A$23)</f>
-        <v>45940</v>
-      </c>
-      <c r="P7" s="5" t="n">
-        <f aca="false">WORKDAY(D7,30,Holidays!$A$4:$A$23)</f>
+      <c r="H19" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="I19" s="12" t="str">
+        <f aca="false">IF(G19="No","N/A - not triggered: no Revoked decision, no SLA clock","Measure from close of review")</f>
+        <v>N/A - not triggered: no Revoked decision, no SLA clock</v>
+      </c>
+      <c r="J19" s="6" t="str">
+        <f aca="false">IF(AND(C19&lt;&gt;"",K19="No - none in any tab (WorkItemID blank)"),"FAIL - IAMS-terminated identity ("&amp;TEXT(C19,"mm/dd/yyyy")&amp;") approved; PAM raised no revocation ticket","Pass")</f>
+        <v>FAIL - IAMS-terminated identity (12/31/2024) approved; PAM raised no revocation ticket</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="L19" s="5" t="n">
+        <f aca="false">WORKDAY(C19,1,Holidays!$A$4:$A$23)</f>
+        <v>45659</v>
+      </c>
+      <c r="M19" s="5" t="n">
+        <f aca="false">WORKDAY(C19,30,Holidays!$A$4:$A$23)</f>
         <v>45701</v>
       </c>
-      <c r="Q7" s="4" t="n">
+      <c r="N19" s="4" t="n">
         <v>46251</v>
       </c>
-      <c r="R7" s="3" t="n">
-        <f aca="false">IF(Q7&gt;O7,NETWORKDAYS(O7+1,Q7,Holidays!$A$4:$A$23),0)</f>
-        <v>211</v>
-      </c>
-      <c r="S7" s="6" t="str">
-        <f aca="false">IF(AND(L7="No",Q7&gt;O7),"No - SLA not met",IF(R7=0,"Yes","No - late"))</f>
-        <v>No - SLA not met</v>
-      </c>
-      <c r="T7" s="3" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="O19" s="3" t="n">
+        <f aca="false">IF(N19&gt;M19,NETWORKDAYS(M19+1,N19,Holidays!$A$4:$A$23),0)</f>
+        <v>377</v>
+      </c>
+      <c r="P19" s="7" t="str">
+        <f aca="false">IF(O19&gt;0,"Missed by "&amp;O19&amp;" business days IF termination is confirmed - leaver control observation, look-back required (4.2.4.3)","Met")</f>
+        <v>Missed by 377 business days IF termination is confirmed - leaver control observation, look-back required (4.2.4.3)</v>
+      </c>
+      <c r="Q19" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="R19" s="3" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B20" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="C8" s="3" t="n">
-        <v>100592069</v>
-      </c>
-      <c r="D8" s="4" t="n">
+      <c r="C20" s="4" t="n">
         <v>45657</v>
       </c>
-      <c r="E8" s="11" t="b">
+      <c r="D20" s="11" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="F8" s="14" t="b">
+      <c r="E20" s="16" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G8" s="11" t="b">
+      <c r="F20" s="11" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H8" s="3" t="s">
-        <v>392</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>394</v>
-      </c>
-      <c r="L8" s="3" t="s">
+      <c r="G20" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="M8" s="3" t="s">
-        <v>395</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>45897</v>
-      </c>
-      <c r="O8" s="5" t="n">
-        <f aca="false">WORKDAY(N8,30,Holidays!$A$4:$A$23)</f>
-        <v>45940</v>
-      </c>
-      <c r="P8" s="5" t="n">
-        <f aca="false">WORKDAY(D8,30,Holidays!$A$4:$A$23)</f>
+      <c r="H20" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="I20" s="12" t="str">
+        <f aca="false">IF(G20="No","N/A - not triggered: no Revoked decision, no SLA clock","Measure from close of review")</f>
+        <v>N/A - not triggered: no Revoked decision, no SLA clock</v>
+      </c>
+      <c r="J20" s="6" t="str">
+        <f aca="false">IF(AND(C20&lt;&gt;"",K20="No - none in any tab (WorkItemID blank)"),"FAIL - IAMS-terminated identity ("&amp;TEXT(C20,"mm/dd/yyyy")&amp;") approved; PAM raised no revocation ticket","Pass")</f>
+        <v>FAIL - IAMS-terminated identity (12/31/2024) approved; PAM raised no revocation ticket</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="L20" s="5" t="n">
+        <f aca="false">WORKDAY(C20,1,Holidays!$A$4:$A$23)</f>
+        <v>45659</v>
+      </c>
+      <c r="M20" s="5" t="n">
+        <f aca="false">WORKDAY(C20,30,Holidays!$A$4:$A$23)</f>
         <v>45701</v>
       </c>
-      <c r="Q8" s="4" t="n">
+      <c r="N20" s="4" t="n">
         <v>46251</v>
       </c>
-      <c r="R8" s="3" t="n">
-        <f aca="false">IF(Q8&gt;O8,NETWORKDAYS(O8+1,Q8,Holidays!$A$4:$A$23),0)</f>
-        <v>211</v>
-      </c>
-      <c r="S8" s="6" t="str">
-        <f aca="false">IF(AND(L8="No",Q8&gt;O8),"No - SLA not met",IF(R8=0,"Yes","No - late"))</f>
-        <v>No - SLA not met</v>
-      </c>
-      <c r="T8" s="3" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="O20" s="3" t="n">
+        <f aca="false">IF(N20&gt;M20,NETWORKDAYS(M20+1,N20,Holidays!$A$4:$A$23),0)</f>
+        <v>377</v>
+      </c>
+      <c r="P20" s="7" t="str">
+        <f aca="false">IF(O20&gt;0,"Missed by "&amp;O20&amp;" business days IF termination is confirmed - leaver control observation, look-back required (4.2.4.3)","Met")</f>
+        <v>Missed by 377 business days IF termination is confirmed - leaver control observation, look-back required (4.2.4.3)</v>
+      </c>
+      <c r="Q20" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="R20" s="3" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B21" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="C9" s="3" t="n">
-        <v>100592068</v>
-      </c>
-      <c r="D9" s="4" t="n">
+      <c r="C21" s="4" t="n">
         <v>45657</v>
       </c>
-      <c r="E9" s="11" t="b">
+      <c r="D21" s="11" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="F9" s="14" t="b">
+      <c r="E21" s="16" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G9" s="11" t="b">
+      <c r="F21" s="11" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H9" s="3" t="s">
-        <v>392</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>394</v>
-      </c>
-      <c r="L9" s="3" t="s">
+      <c r="G21" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="M9" s="3" t="s">
-        <v>395</v>
-      </c>
-      <c r="N9" s="4" t="n">
-        <v>45897</v>
-      </c>
-      <c r="O9" s="5" t="n">
-        <f aca="false">WORKDAY(N9,30,Holidays!$A$4:$A$23)</f>
-        <v>45940</v>
-      </c>
-      <c r="P9" s="5" t="n">
-        <f aca="false">WORKDAY(D9,30,Holidays!$A$4:$A$23)</f>
+      <c r="H21" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="I21" s="12" t="str">
+        <f aca="false">IF(G21="No","N/A - not triggered: no Revoked decision, no SLA clock","Measure from close of review")</f>
+        <v>N/A - not triggered: no Revoked decision, no SLA clock</v>
+      </c>
+      <c r="J21" s="6" t="str">
+        <f aca="false">IF(AND(C21&lt;&gt;"",K21="No - none in any tab (WorkItemID blank)"),"FAIL - IAMS-terminated identity ("&amp;TEXT(C21,"mm/dd/yyyy")&amp;") approved; PAM raised no revocation ticket","Pass")</f>
+        <v>FAIL - IAMS-terminated identity (12/31/2024) approved; PAM raised no revocation ticket</v>
+      </c>
+      <c r="K21" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="L21" s="5" t="n">
+        <f aca="false">WORKDAY(C21,1,Holidays!$A$4:$A$23)</f>
+        <v>45659</v>
+      </c>
+      <c r="M21" s="5" t="n">
+        <f aca="false">WORKDAY(C21,30,Holidays!$A$4:$A$23)</f>
         <v>45701</v>
       </c>
-      <c r="Q9" s="4" t="n">
+      <c r="N21" s="4" t="n">
         <v>46251</v>
       </c>
-      <c r="R9" s="3" t="n">
-        <f aca="false">IF(Q9&gt;O9,NETWORKDAYS(O9+1,Q9,Holidays!$A$4:$A$23),0)</f>
-        <v>211</v>
-      </c>
-      <c r="S9" s="6" t="str">
-        <f aca="false">IF(AND(L9="No",Q9&gt;O9),"No - SLA not met",IF(R9=0,"Yes","No - late"))</f>
-        <v>No - SLA not met</v>
-      </c>
-      <c r="T9" s="3" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
-        <v>402</v>
-      </c>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="9" t="str">
-        <f aca="false">COUNTIF(S4:S9,"No*")&amp;" of "&amp;COUNTA(A4:A9)</f>
+      <c r="O21" s="3" t="n">
+        <f aca="false">IF(N21&gt;M21,NETWORKDAYS(M21+1,N21,Holidays!$A$4:$A$23),0)</f>
+        <v>377</v>
+      </c>
+      <c r="P21" s="7" t="str">
+        <f aca="false">IF(O21&gt;0,"Missed by "&amp;O21&amp;" business days IF termination is confirmed - leaver control observation, look-back required (4.2.4.3)","Met")</f>
+        <v>Missed by 377 business days IF termination is confirmed - leaver control observation, look-back required (4.2.4.3)</v>
+      </c>
+      <c r="Q21" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="R21" s="3" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="17" t="s">
+        <v>441</v>
+      </c>
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="9" t="str">
+        <f aca="false">COUNTIF(I16:I21,"Fail*")&amp;" of "&amp;COUNTA(A16:A21)&amp;" (SLA not triggered)"</f>
+        <v>0 of 6 (SLA not triggered)</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="17" t="s">
+        <v>442</v>
+      </c>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="9" t="str">
+        <f aca="false">COUNTIF(J16:J21,"FAIL*")&amp;" of "&amp;COUNTA(A16:A21)</f>
         <v>6 of 6</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="16" t="s">
-        <v>403</v>
-      </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="16"/>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="16"/>
-    </row>
-    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="16" t="s">
-        <v>404</v>
-      </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
-      <c r="I13" s="16"/>
-      <c r="J13" s="16"/>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="16"/>
-    </row>
-    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="16" t="s">
-        <v>405</v>
-      </c>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
-      <c r="I14" s="16"/>
-      <c r="J14" s="16"/>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
-      <c r="N14" s="16"/>
-    </row>
-    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="16" t="s">
-        <v>406</v>
-      </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
-      <c r="I15" s="16"/>
-      <c r="J15" s="16"/>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
-      <c r="N15" s="16"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17" t="s">
-        <v>408</v>
-      </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="17"/>
-      <c r="L18" s="17"/>
-      <c r="M18" s="17"/>
-      <c r="N18" s="17"/>
-    </row>
-    <row r="19" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="18" t="s">
-        <v>409</v>
-      </c>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="19" t="str">
-        <f aca="false">"Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), "&amp;J4&amp;", "&amp;K4&amp;". No Revoked decision in any review."</f>
-        <v>Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), Approved 7/27/26, 12:45 PM (Borges, Dayam), Approved 8/17/26, 9:23 AM (Borges, Dayam). No Revoked decision in any review.</v>
-      </c>
-      <c r="E19" s="19"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="19"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
-      <c r="J19" s="19"/>
-      <c r="K19" s="19"/>
-      <c r="L19" s="19"/>
-      <c r="M19" s="19"/>
-      <c r="N19" s="19"/>
-    </row>
-    <row r="20" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="18" t="s">
-        <v>410</v>
-      </c>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="19" t="s">
-        <v>411</v>
-      </c>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="19"/>
-      <c r="J20" s="19"/>
-      <c r="K20" s="19"/>
-      <c r="L20" s="19"/>
-      <c r="M20" s="19"/>
-      <c r="N20" s="19"/>
-    </row>
-    <row r="21" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="18" t="s">
-        <v>412</v>
-      </c>
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="20" t="str">
-        <f aca="false">"NO - SLA not met. IAMS termination date "&amp;TEXT(D4,"mm/dd/yyyy")&amp;"; removal was due by "&amp;TEXT(O4,"mm/dd/yyyy")&amp;" (30 business days after the 08/28/2025 review) and access was still held on "&amp;TEXT(Q4,"mm/dd/yyyy")&amp;", "&amp;R4&amp;" business days past the deadline."</f>
-        <v>NO - SLA not met. IAMS termination date 12/31/2024; removal was due by 10/10/2025 (30 business days after the 08/28/2025 review) and access was still held on 08/17/2026, 211 business days past the deadline.</v>
-      </c>
-      <c r="E21" s="20"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="20"/>
-      <c r="H21" s="20"/>
-      <c r="I21" s="20"/>
-      <c r="J21" s="20"/>
-      <c r="K21" s="20"/>
-      <c r="L21" s="20"/>
-      <c r="M21" s="20"/>
-      <c r="N21" s="20"/>
-    </row>
-    <row r="22" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B22" s="18"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="19" t="s">
-        <v>413</v>
-      </c>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="19"/>
-      <c r="H22" s="19"/>
-      <c r="I22" s="19"/>
-      <c r="J22" s="19"/>
-      <c r="K22" s="19"/>
-      <c r="L22" s="19"/>
-      <c r="M22" s="19"/>
-      <c r="N22" s="19"/>
-    </row>
-    <row r="23" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18" t="s">
-        <v>414</v>
-      </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="19" t="str">
-        <f aca="false">"C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = "&amp;IF(G4,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
-        <v>C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = FALSE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
-      </c>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="19"/>
-      <c r="J23" s="19"/>
-      <c r="K23" s="19"/>
-      <c r="L23" s="19"/>
-      <c r="M23" s="19"/>
-      <c r="N23" s="19"/>
-    </row>
-    <row r="24" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="20" t="s">
-        <v>415</v>
-      </c>
-      <c r="E24" s="20"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="20"/>
-      <c r="H24" s="20"/>
-      <c r="I24" s="20"/>
-      <c r="J24" s="20"/>
-      <c r="K24" s="20"/>
-      <c r="L24" s="20"/>
-      <c r="M24" s="20"/>
-      <c r="N24" s="20"/>
-    </row>
-    <row r="25" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="18" t="s">
-        <v>416</v>
-      </c>
-      <c r="B25" s="18"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="19" t="str">
-        <f aca="false">T4</f>
-        <v>C7.Sample.xlsx: SAMPLE!A72 (screenshots at A73 and A79); 2026Q2PamBsiSox-Manager rows 86-88; 2026Q2BsiPamCyberark-Manager rows 419-421; Oct10_2026Users row 1598. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 15, 2025 Q3 ISEAdmin row 53, 2026 Q1 CISCO Network Administrators row 103, 2026 Q1 ISEAdmin row 126; 5_Exceptions row 4. This workbook: 2_Item Detail.</v>
-      </c>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19"/>
-      <c r="H25" s="19"/>
-      <c r="I25" s="19"/>
-      <c r="J25" s="19"/>
-      <c r="K25" s="19"/>
-      <c r="L25" s="19"/>
-      <c r="M25" s="19"/>
-      <c r="N25" s="19"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="17" t="s">
-        <v>417</v>
-      </c>
-      <c r="B27" s="17"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
-      <c r="G27" s="17"/>
-      <c r="H27" s="17"/>
-      <c r="I27" s="17"/>
-      <c r="J27" s="17"/>
-      <c r="K27" s="17"/>
-      <c r="L27" s="17"/>
-      <c r="M27" s="17"/>
-      <c r="N27" s="17"/>
-    </row>
-    <row r="28" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="18" t="s">
-        <v>409</v>
-      </c>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="19" t="str">
-        <f aca="false">"Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), "&amp;J5&amp;", "&amp;K5&amp;". No Revoked decision in any review."</f>
-        <v>Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), Approved 7/27/26, 12:45 PM (Borges, Dayam), Approved 8/17/26, 9:23 AM (Borges, Dayam). No Revoked decision in any review.</v>
-      </c>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="19"/>
-      <c r="I28" s="19"/>
-      <c r="J28" s="19"/>
-      <c r="K28" s="19"/>
-      <c r="L28" s="19"/>
-      <c r="M28" s="19"/>
-      <c r="N28" s="19"/>
-    </row>
-    <row r="29" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="18" t="s">
-        <v>410</v>
-      </c>
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="19" t="s">
-        <v>411</v>
-      </c>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="17" t="s">
+        <v>443</v>
+      </c>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="9" t="str">
+        <f aca="false">COUNTIF(P16:P21,"Missed*")&amp;" of "&amp;COUNTA(A16:A21)</f>
+        <v>6 of 6</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="18" t="s">
+        <v>444</v>
+      </c>
+      <c r="B26" s="18"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="18"/>
+      <c r="I26" s="18"/>
+      <c r="J26" s="18"/>
+      <c r="K26" s="18"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="14" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="19" t="s">
+        <v>446</v>
+      </c>
+      <c r="B29" s="19"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
       <c r="E29" s="19"/>
       <c r="F29" s="19"/>
       <c r="G29" s="19"/>
@@ -7807,161 +7917,136 @@
       <c r="I29" s="19"/>
       <c r="J29" s="19"/>
       <c r="K29" s="19"/>
-      <c r="L29" s="19"/>
-      <c r="M29" s="19"/>
-      <c r="N29" s="19"/>
-    </row>
-    <row r="30" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="18" t="s">
-        <v>412</v>
-      </c>
-      <c r="B30" s="18"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="20" t="str">
-        <f aca="false">"NO - SLA not met. IAMS termination date "&amp;TEXT(D5,"mm/dd/yyyy")&amp;"; removal was due by "&amp;TEXT(O5,"mm/dd/yyyy")&amp;" (30 business days after the 08/28/2025 review) and access was still held on "&amp;TEXT(Q5,"mm/dd/yyyy")&amp;", "&amp;R5&amp;" business days past the deadline."</f>
-        <v>NO - SLA not met. IAMS termination date 12/31/2024; removal was due by 10/10/2025 (30 business days after the 08/28/2025 review) and access was still held on 08/17/2026, 211 business days past the deadline.</v>
-      </c>
-      <c r="E30" s="20"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="20"/>
-      <c r="H30" s="20"/>
-      <c r="I30" s="20"/>
-      <c r="J30" s="20"/>
-      <c r="K30" s="20"/>
-      <c r="L30" s="20"/>
-      <c r="M30" s="20"/>
-      <c r="N30" s="20"/>
-    </row>
-    <row r="31" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="18" t="s">
+    </row>
+    <row r="30" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="20" t="s">
+        <v>447</v>
+      </c>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="3" t="str">
+        <f aca="false">H16&amp;". No Revoked decision in any review (reviewer: Borges, Dayam)."</f>
+        <v>Approved 08/28/2025 / Approved 04/30/2026 / Approved 7/27/26, 12:45 PM (SOX) and 8/17/26, 9:23 AM (CyberArk). No Revoked decision in any review (reviewer: Borges, Dayam).</v>
+      </c>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+      <c r="K30" s="3"/>
+    </row>
+    <row r="31" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="B31" s="20"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="3"/>
+      <c r="K31" s="3"/>
+    </row>
+    <row r="32" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="20" t="s">
+        <v>450</v>
+      </c>
+      <c r="B32" s="20"/>
+      <c r="C32" s="20"/>
+      <c r="D32" s="12" t="s">
+        <v>451</v>
+      </c>
+      <c r="E32" s="12"/>
+      <c r="F32" s="12"/>
+      <c r="G32" s="12"/>
+      <c r="H32" s="12"/>
+      <c r="I32" s="12"/>
+      <c r="J32" s="12"/>
+      <c r="K32" s="12"/>
+    </row>
+    <row r="33" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="19" t="s">
-        <v>413</v>
-      </c>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
-      <c r="G31" s="19"/>
-      <c r="H31" s="19"/>
-      <c r="I31" s="19"/>
-      <c r="J31" s="19"/>
-      <c r="K31" s="19"/>
-      <c r="L31" s="19"/>
-      <c r="M31" s="19"/>
-      <c r="N31" s="19"/>
-    </row>
-    <row r="32" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="18" t="s">
-        <v>414</v>
-      </c>
-      <c r="B32" s="18"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="19" t="str">
-        <f aca="false">"C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = "&amp;IF(G5,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
-        <v>C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = TRUE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
-      </c>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
-      <c r="G32" s="19"/>
-      <c r="H32" s="19"/>
-      <c r="I32" s="19"/>
-      <c r="J32" s="19"/>
-      <c r="K32" s="19"/>
-      <c r="L32" s="19"/>
-      <c r="M32" s="19"/>
-      <c r="N32" s="19"/>
-    </row>
-    <row r="33" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="18" t="s">
+      <c r="B33" s="20"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="3"/>
+      <c r="K33" s="3"/>
+    </row>
+    <row r="34" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="20" t="s">
+        <v>453</v>
+      </c>
+      <c r="B34" s="20"/>
+      <c r="C34" s="20"/>
+      <c r="D34" s="3" t="str">
+        <f aca="false">"C7.Sample.xlsx certification exports (all Approved, WorkItemID blank) and AD export (enabled 10/10/2026 = "&amp;IF(F16,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
+        <v>C7.Sample.xlsx certification exports (all Approved, WorkItemID blank) and AD export (enabled 10/10/2026 = FALSE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
+      </c>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="3"/>
+      <c r="K34" s="3"/>
+    </row>
+    <row r="35" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="B33" s="18"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="20" t="s">
-        <v>418</v>
-      </c>
-      <c r="E33" s="20"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="20"/>
-      <c r="H33" s="20"/>
-      <c r="I33" s="20"/>
-      <c r="J33" s="20"/>
-      <c r="K33" s="20"/>
-      <c r="L33" s="20"/>
-      <c r="M33" s="20"/>
-      <c r="N33" s="20"/>
-    </row>
-    <row r="34" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="18" t="s">
-        <v>416</v>
-      </c>
-      <c r="B34" s="18"/>
-      <c r="C34" s="18"/>
-      <c r="D34" s="19" t="str">
-        <f aca="false">T5</f>
-        <v>C7.Sample.xlsx: SAMPLE!A86 (screenshots at A87 and A93); 2026Q2PamBsiSox-Manager rows 89-91; 2026Q2BsiPamCyberark-Manager rows 422-424; Oct10_2026Users row 1596. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 16, 2025 Q3 ISEAdmin row 54, 2026 Q1 CISCO Network Administrators row 104, 2026 Q1 ISEAdmin row 127; 5_Exceptions row 5. This workbook: 2_Item Detail.</v>
-      </c>
-      <c r="E34" s="19"/>
-      <c r="F34" s="19"/>
-      <c r="G34" s="19"/>
-      <c r="H34" s="19"/>
-      <c r="I34" s="19"/>
-      <c r="J34" s="19"/>
-      <c r="K34" s="19"/>
-      <c r="L34" s="19"/>
-      <c r="M34" s="19"/>
-      <c r="N34" s="19"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="17" t="s">
-        <v>419</v>
-      </c>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="17"/>
-      <c r="F36" s="17"/>
-      <c r="G36" s="17"/>
-      <c r="H36" s="17"/>
-      <c r="I36" s="17"/>
-      <c r="J36" s="17"/>
-      <c r="K36" s="17"/>
-      <c r="L36" s="17"/>
-      <c r="M36" s="17"/>
-      <c r="N36" s="17"/>
-    </row>
-    <row r="37" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="18" t="s">
-        <v>409</v>
-      </c>
-      <c r="B37" s="18"/>
-      <c r="C37" s="18"/>
-      <c r="D37" s="19" t="str">
-        <f aca="false">"Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), "&amp;J6&amp;", "&amp;K6&amp;". No Revoked decision in any review."</f>
-        <v>Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), Approved 7/27/26, 12:45 PM (Borges, Dayam), Approved 8/17/26, 9:23 AM (Borges, Dayam). No Revoked decision in any review.</v>
-      </c>
-      <c r="E37" s="19"/>
-      <c r="F37" s="19"/>
-      <c r="G37" s="19"/>
-      <c r="H37" s="19"/>
-      <c r="I37" s="19"/>
-      <c r="J37" s="19"/>
-      <c r="K37" s="19"/>
-      <c r="L37" s="19"/>
-      <c r="M37" s="19"/>
-      <c r="N37" s="19"/>
-    </row>
-    <row r="38" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="18" t="s">
-        <v>410</v>
-      </c>
-      <c r="B38" s="18"/>
-      <c r="C38" s="18"/>
-      <c r="D38" s="19" t="s">
-        <v>411</v>
-      </c>
+      <c r="B35" s="20"/>
+      <c r="C35" s="20"/>
+      <c r="D35" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="6"/>
+      <c r="H35" s="6"/>
+      <c r="I35" s="6"/>
+      <c r="J35" s="6"/>
+      <c r="K35" s="6"/>
+    </row>
+    <row r="36" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="20" t="s">
+        <v>389</v>
+      </c>
+      <c r="B36" s="20"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="3" t="str">
+        <f aca="false">R16</f>
+        <v>C7.Sample.xlsx: SAMPLE!A72 (screenshots A73, A79); 2026Q2PamBsiSox-Manager rows 86-88; 2026Q2BsiPamCyberark-Manager rows 419-421; Oct10_2026Users row 1598. Walkthrough: 4_Item Detail 2025 Q3 CISCO Network Administrators row 15, 2025 Q3 ISEAdmin row 53, 2026 Q1 CISCO Network Administrators row 103, 2026 Q1 ISEAdmin row 126; 5_Exceptions row 4. Policy: section B above.</v>
+      </c>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
+      <c r="J36" s="3"/>
+      <c r="K36" s="3"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="19" t="s">
+        <v>455</v>
+      </c>
+      <c r="B38" s="19"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19"/>
       <c r="E38" s="19"/>
       <c r="F38" s="19"/>
       <c r="G38" s="19"/>
@@ -7969,161 +8054,136 @@
       <c r="I38" s="19"/>
       <c r="J38" s="19"/>
       <c r="K38" s="19"/>
-      <c r="L38" s="19"/>
-      <c r="M38" s="19"/>
-      <c r="N38" s="19"/>
-    </row>
-    <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="18" t="s">
-        <v>412</v>
-      </c>
-      <c r="B39" s="18"/>
-      <c r="C39" s="18"/>
-      <c r="D39" s="20" t="str">
-        <f aca="false">"NO - SLA not met. IAMS termination date "&amp;TEXT(D6,"mm/dd/yyyy")&amp;"; removal was due by "&amp;TEXT(O6,"mm/dd/yyyy")&amp;" (30 business days after the 08/28/2025 review) and access was still held on "&amp;TEXT(Q6,"mm/dd/yyyy")&amp;", "&amp;R6&amp;" business days past the deadline."</f>
-        <v>NO - SLA not met. IAMS termination date 12/31/2024; removal was due by 10/10/2025 (30 business days after the 08/28/2025 review) and access was still held on 08/17/2026, 211 business days past the deadline.</v>
-      </c>
-      <c r="E39" s="20"/>
-      <c r="F39" s="20"/>
-      <c r="G39" s="20"/>
-      <c r="H39" s="20"/>
-      <c r="I39" s="20"/>
-      <c r="J39" s="20"/>
-      <c r="K39" s="20"/>
-      <c r="L39" s="20"/>
-      <c r="M39" s="20"/>
-      <c r="N39" s="20"/>
-    </row>
-    <row r="40" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="18" t="s">
+    </row>
+    <row r="39" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="20" t="s">
+        <v>447</v>
+      </c>
+      <c r="B39" s="20"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="3" t="str">
+        <f aca="false">H17&amp;". No Revoked decision in any review (reviewer: Borges, Dayam)."</f>
+        <v>Approved 08/28/2025 / Approved 04/30/2026 / Approved 7/27/26, 12:45 PM (SOX) and 8/17/26, 9:23 AM (CyberArk). No Revoked decision in any review (reviewer: Borges, Dayam).</v>
+      </c>
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
+      <c r="I39" s="3"/>
+      <c r="J39" s="3"/>
+      <c r="K39" s="3"/>
+    </row>
+    <row r="40" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="B40" s="20"/>
+      <c r="C40" s="20"/>
+      <c r="D40" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+      <c r="I40" s="3"/>
+      <c r="J40" s="3"/>
+      <c r="K40" s="3"/>
+    </row>
+    <row r="41" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="20" t="s">
+        <v>450</v>
+      </c>
+      <c r="B41" s="20"/>
+      <c r="C41" s="20"/>
+      <c r="D41" s="12" t="s">
+        <v>451</v>
+      </c>
+      <c r="E41" s="12"/>
+      <c r="F41" s="12"/>
+      <c r="G41" s="12"/>
+      <c r="H41" s="12"/>
+      <c r="I41" s="12"/>
+      <c r="J41" s="12"/>
+      <c r="K41" s="12"/>
+    </row>
+    <row r="42" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B40" s="18"/>
-      <c r="C40" s="18"/>
-      <c r="D40" s="19" t="s">
-        <v>413</v>
-      </c>
-      <c r="E40" s="19"/>
-      <c r="F40" s="19"/>
-      <c r="G40" s="19"/>
-      <c r="H40" s="19"/>
-      <c r="I40" s="19"/>
-      <c r="J40" s="19"/>
-      <c r="K40" s="19"/>
-      <c r="L40" s="19"/>
-      <c r="M40" s="19"/>
-      <c r="N40" s="19"/>
-    </row>
-    <row r="41" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="18" t="s">
-        <v>414</v>
-      </c>
-      <c r="B41" s="18"/>
-      <c r="C41" s="18"/>
-      <c r="D41" s="19" t="str">
-        <f aca="false">"C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = "&amp;IF(G6,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
-        <v>C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = TRUE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
-      </c>
-      <c r="E41" s="19"/>
-      <c r="F41" s="19"/>
-      <c r="G41" s="19"/>
-      <c r="H41" s="19"/>
-      <c r="I41" s="19"/>
-      <c r="J41" s="19"/>
-      <c r="K41" s="19"/>
-      <c r="L41" s="19"/>
-      <c r="M41" s="19"/>
-      <c r="N41" s="19"/>
-    </row>
-    <row r="42" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="18" t="s">
+      <c r="B42" s="20"/>
+      <c r="C42" s="20"/>
+      <c r="D42" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="E42" s="3"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
+      <c r="I42" s="3"/>
+      <c r="J42" s="3"/>
+      <c r="K42" s="3"/>
+    </row>
+    <row r="43" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="20" t="s">
+        <v>453</v>
+      </c>
+      <c r="B43" s="20"/>
+      <c r="C43" s="20"/>
+      <c r="D43" s="3" t="str">
+        <f aca="false">"C7.Sample.xlsx certification exports (all Approved, WorkItemID blank) and AD export (enabled 10/10/2026 = "&amp;IF(F17,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
+        <v>C7.Sample.xlsx certification exports (all Approved, WorkItemID blank) and AD export (enabled 10/10/2026 = TRUE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
+      </c>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+      <c r="I43" s="3"/>
+      <c r="J43" s="3"/>
+      <c r="K43" s="3"/>
+    </row>
+    <row r="44" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="B42" s="18"/>
-      <c r="C42" s="18"/>
-      <c r="D42" s="20" t="s">
-        <v>418</v>
-      </c>
-      <c r="E42" s="20"/>
-      <c r="F42" s="20"/>
-      <c r="G42" s="20"/>
-      <c r="H42" s="20"/>
-      <c r="I42" s="20"/>
-      <c r="J42" s="20"/>
-      <c r="K42" s="20"/>
-      <c r="L42" s="20"/>
-      <c r="M42" s="20"/>
-      <c r="N42" s="20"/>
-    </row>
-    <row r="43" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="18" t="s">
-        <v>416</v>
-      </c>
-      <c r="B43" s="18"/>
-      <c r="C43" s="18"/>
-      <c r="D43" s="19" t="str">
-        <f aca="false">T6</f>
-        <v>C7.Sample.xlsx: SAMPLE!A100 (screenshots at A101 and A107); 2026Q2PamBsiSox-Manager rows 92-94; 2026Q2BsiPamCyberark-Manager rows 425-427; Oct10_2026Users row 1599. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 17, 2025 Q3 ISEAdmin row 55, 2026 Q1 CISCO Network Administrators row 105, 2026 Q1 ISEAdmin row 128; 5_Exceptions row 6. This workbook: 2_Item Detail.</v>
-      </c>
-      <c r="E43" s="19"/>
-      <c r="F43" s="19"/>
-      <c r="G43" s="19"/>
-      <c r="H43" s="19"/>
-      <c r="I43" s="19"/>
-      <c r="J43" s="19"/>
-      <c r="K43" s="19"/>
-      <c r="L43" s="19"/>
-      <c r="M43" s="19"/>
-      <c r="N43" s="19"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="17" t="s">
-        <v>420</v>
-      </c>
-      <c r="B45" s="17"/>
-      <c r="C45" s="17"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="17"/>
-      <c r="F45" s="17"/>
-      <c r="G45" s="17"/>
-      <c r="H45" s="17"/>
-      <c r="I45" s="17"/>
-      <c r="J45" s="17"/>
-      <c r="K45" s="17"/>
-      <c r="L45" s="17"/>
-      <c r="M45" s="17"/>
-      <c r="N45" s="17"/>
-    </row>
-    <row r="46" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="18" t="s">
-        <v>409</v>
-      </c>
-      <c r="B46" s="18"/>
-      <c r="C46" s="18"/>
-      <c r="D46" s="19" t="str">
-        <f aca="false">"Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), "&amp;J7&amp;", "&amp;K7&amp;". No Revoked decision in any review."</f>
-        <v>Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), Approved 7/27/26, 12:45 PM (Borges, Dayam), Approved 8/17/26, 9:23 AM (Borges, Dayam). No Revoked decision in any review.</v>
-      </c>
-      <c r="E46" s="19"/>
-      <c r="F46" s="19"/>
-      <c r="G46" s="19"/>
-      <c r="H46" s="19"/>
-      <c r="I46" s="19"/>
-      <c r="J46" s="19"/>
-      <c r="K46" s="19"/>
-      <c r="L46" s="19"/>
-      <c r="M46" s="19"/>
-      <c r="N46" s="19"/>
-    </row>
-    <row r="47" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="18" t="s">
-        <v>410</v>
-      </c>
-      <c r="B47" s="18"/>
-      <c r="C47" s="18"/>
-      <c r="D47" s="19" t="s">
-        <v>411</v>
-      </c>
+      <c r="B44" s="20"/>
+      <c r="C44" s="20"/>
+      <c r="D44" s="6" t="s">
+        <v>456</v>
+      </c>
+      <c r="E44" s="6"/>
+      <c r="F44" s="6"/>
+      <c r="G44" s="6"/>
+      <c r="H44" s="6"/>
+      <c r="I44" s="6"/>
+      <c r="J44" s="6"/>
+      <c r="K44" s="6"/>
+    </row>
+    <row r="45" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="20" t="s">
+        <v>389</v>
+      </c>
+      <c r="B45" s="20"/>
+      <c r="C45" s="20"/>
+      <c r="D45" s="3" t="str">
+        <f aca="false">R17</f>
+        <v>C7.Sample.xlsx: SAMPLE!A86 (screenshots A87, A93); 2026Q2PamBsiSox-Manager rows 89-91; 2026Q2BsiPamCyberark-Manager rows 422-424; Oct10_2026Users row 1596. Walkthrough: 4_Item Detail 2025 Q3 CISCO Network Administrators row 16, 2025 Q3 ISEAdmin row 54, 2026 Q1 CISCO Network Administrators row 104, 2026 Q1 ISEAdmin row 127; 5_Exceptions row 5. Policy: section B above.</v>
+      </c>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
+      <c r="K45" s="3"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="19" t="s">
+        <v>457</v>
+      </c>
+      <c r="B47" s="19"/>
+      <c r="C47" s="19"/>
+      <c r="D47" s="19"/>
       <c r="E47" s="19"/>
       <c r="F47" s="19"/>
       <c r="G47" s="19"/>
@@ -8131,161 +8191,136 @@
       <c r="I47" s="19"/>
       <c r="J47" s="19"/>
       <c r="K47" s="19"/>
-      <c r="L47" s="19"/>
-      <c r="M47" s="19"/>
-      <c r="N47" s="19"/>
-    </row>
-    <row r="48" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="18" t="s">
-        <v>412</v>
-      </c>
-      <c r="B48" s="18"/>
-      <c r="C48" s="18"/>
-      <c r="D48" s="20" t="str">
-        <f aca="false">"NO - SLA not met. IAMS termination date "&amp;TEXT(D7,"mm/dd/yyyy")&amp;"; removal was due by "&amp;TEXT(O7,"mm/dd/yyyy")&amp;" (30 business days after the 08/28/2025 review) and access was still held on "&amp;TEXT(Q7,"mm/dd/yyyy")&amp;", "&amp;R7&amp;" business days past the deadline."</f>
-        <v>NO - SLA not met. IAMS termination date 12/31/2024; removal was due by 10/10/2025 (30 business days after the 08/28/2025 review) and access was still held on 08/17/2026, 211 business days past the deadline.</v>
-      </c>
-      <c r="E48" s="20"/>
-      <c r="F48" s="20"/>
-      <c r="G48" s="20"/>
-      <c r="H48" s="20"/>
-      <c r="I48" s="20"/>
-      <c r="J48" s="20"/>
-      <c r="K48" s="20"/>
-      <c r="L48" s="20"/>
-      <c r="M48" s="20"/>
-      <c r="N48" s="20"/>
-    </row>
-    <row r="49" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="18" t="s">
+    </row>
+    <row r="48" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="20" t="s">
+        <v>447</v>
+      </c>
+      <c r="B48" s="20"/>
+      <c r="C48" s="20"/>
+      <c r="D48" s="3" t="str">
+        <f aca="false">H18&amp;". No Revoked decision in any review (reviewer: Borges, Dayam)."</f>
+        <v>Approved 08/28/2025 / Approved 04/30/2026 / Approved 7/27/26, 12:45 PM (SOX) and 8/17/26, 9:23 AM (CyberArk). No Revoked decision in any review (reviewer: Borges, Dayam).</v>
+      </c>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+      <c r="I48" s="3"/>
+      <c r="J48" s="3"/>
+      <c r="K48" s="3"/>
+    </row>
+    <row r="49" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="B49" s="20"/>
+      <c r="C49" s="20"/>
+      <c r="D49" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+      <c r="I49" s="3"/>
+      <c r="J49" s="3"/>
+      <c r="K49" s="3"/>
+    </row>
+    <row r="50" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="20" t="s">
+        <v>450</v>
+      </c>
+      <c r="B50" s="20"/>
+      <c r="C50" s="20"/>
+      <c r="D50" s="12" t="s">
+        <v>451</v>
+      </c>
+      <c r="E50" s="12"/>
+      <c r="F50" s="12"/>
+      <c r="G50" s="12"/>
+      <c r="H50" s="12"/>
+      <c r="I50" s="12"/>
+      <c r="J50" s="12"/>
+      <c r="K50" s="12"/>
+    </row>
+    <row r="51" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B49" s="18"/>
-      <c r="C49" s="18"/>
-      <c r="D49" s="19" t="s">
-        <v>413</v>
-      </c>
-      <c r="E49" s="19"/>
-      <c r="F49" s="19"/>
-      <c r="G49" s="19"/>
-      <c r="H49" s="19"/>
-      <c r="I49" s="19"/>
-      <c r="J49" s="19"/>
-      <c r="K49" s="19"/>
-      <c r="L49" s="19"/>
-      <c r="M49" s="19"/>
-      <c r="N49" s="19"/>
-    </row>
-    <row r="50" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="18" t="s">
-        <v>414</v>
-      </c>
-      <c r="B50" s="18"/>
-      <c r="C50" s="18"/>
-      <c r="D50" s="19" t="str">
-        <f aca="false">"C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = "&amp;IF(G7,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
-        <v>C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = TRUE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
-      </c>
-      <c r="E50" s="19"/>
-      <c r="F50" s="19"/>
-      <c r="G50" s="19"/>
-      <c r="H50" s="19"/>
-      <c r="I50" s="19"/>
-      <c r="J50" s="19"/>
-      <c r="K50" s="19"/>
-      <c r="L50" s="19"/>
-      <c r="M50" s="19"/>
-      <c r="N50" s="19"/>
-    </row>
-    <row r="51" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="18" t="s">
+      <c r="B51" s="20"/>
+      <c r="C51" s="20"/>
+      <c r="D51" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="3"/>
+      <c r="J51" s="3"/>
+      <c r="K51" s="3"/>
+    </row>
+    <row r="52" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="20" t="s">
+        <v>453</v>
+      </c>
+      <c r="B52" s="20"/>
+      <c r="C52" s="20"/>
+      <c r="D52" s="3" t="str">
+        <f aca="false">"C7.Sample.xlsx certification exports (all Approved, WorkItemID blank) and AD export (enabled 10/10/2026 = "&amp;IF(F18,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
+        <v>C7.Sample.xlsx certification exports (all Approved, WorkItemID blank) and AD export (enabled 10/10/2026 = TRUE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
+      </c>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="3"/>
+      <c r="I52" s="3"/>
+      <c r="J52" s="3"/>
+      <c r="K52" s="3"/>
+    </row>
+    <row r="53" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="B51" s="18"/>
-      <c r="C51" s="18"/>
-      <c r="D51" s="20" t="s">
-        <v>418</v>
-      </c>
-      <c r="E51" s="20"/>
-      <c r="F51" s="20"/>
-      <c r="G51" s="20"/>
-      <c r="H51" s="20"/>
-      <c r="I51" s="20"/>
-      <c r="J51" s="20"/>
-      <c r="K51" s="20"/>
-      <c r="L51" s="20"/>
-      <c r="M51" s="20"/>
-      <c r="N51" s="20"/>
-    </row>
-    <row r="52" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="18" t="s">
-        <v>416</v>
-      </c>
-      <c r="B52" s="18"/>
-      <c r="C52" s="18"/>
-      <c r="D52" s="19" t="str">
-        <f aca="false">T7</f>
-        <v>C7.Sample.xlsx: SAMPLE!A114 (screenshots at A115 and A121); 2026Q2PamBsiSox-Manager rows 95-97; 2026Q2BsiPamCyberark-Manager rows 428-430; Oct10_2026Users row 1597. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 18, 2025 Q3 ISEAdmin row 56, 2026 Q1 CISCO Network Administrators row 106, 2026 Q1 ISEAdmin row 129; 5_Exceptions row 7. This workbook: 2_Item Detail.</v>
-      </c>
-      <c r="E52" s="19"/>
-      <c r="F52" s="19"/>
-      <c r="G52" s="19"/>
-      <c r="H52" s="19"/>
-      <c r="I52" s="19"/>
-      <c r="J52" s="19"/>
-      <c r="K52" s="19"/>
-      <c r="L52" s="19"/>
-      <c r="M52" s="19"/>
-      <c r="N52" s="19"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="17" t="s">
-        <v>421</v>
-      </c>
-      <c r="B54" s="17"/>
-      <c r="C54" s="17"/>
-      <c r="D54" s="17"/>
-      <c r="E54" s="17"/>
-      <c r="F54" s="17"/>
-      <c r="G54" s="17"/>
-      <c r="H54" s="17"/>
-      <c r="I54" s="17"/>
-      <c r="J54" s="17"/>
-      <c r="K54" s="17"/>
-      <c r="L54" s="17"/>
-      <c r="M54" s="17"/>
-      <c r="N54" s="17"/>
-    </row>
-    <row r="55" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="18" t="s">
-        <v>409</v>
-      </c>
-      <c r="B55" s="18"/>
-      <c r="C55" s="18"/>
-      <c r="D55" s="19" t="str">
-        <f aca="false">"Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), "&amp;J8&amp;", "&amp;K8&amp;". No Revoked decision in any review."</f>
-        <v>Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), Approved 7/27/26, 12:45 PM (Borges, Dayam), Approved 8/17/26, 9:23 AM (Borges, Dayam). No Revoked decision in any review.</v>
-      </c>
-      <c r="E55" s="19"/>
-      <c r="F55" s="19"/>
-      <c r="G55" s="19"/>
-      <c r="H55" s="19"/>
-      <c r="I55" s="19"/>
-      <c r="J55" s="19"/>
-      <c r="K55" s="19"/>
-      <c r="L55" s="19"/>
-      <c r="M55" s="19"/>
-      <c r="N55" s="19"/>
-    </row>
-    <row r="56" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="18" t="s">
-        <v>410</v>
-      </c>
-      <c r="B56" s="18"/>
-      <c r="C56" s="18"/>
-      <c r="D56" s="19" t="s">
-        <v>411</v>
-      </c>
+      <c r="B53" s="20"/>
+      <c r="C53" s="20"/>
+      <c r="D53" s="6" t="s">
+        <v>456</v>
+      </c>
+      <c r="E53" s="6"/>
+      <c r="F53" s="6"/>
+      <c r="G53" s="6"/>
+      <c r="H53" s="6"/>
+      <c r="I53" s="6"/>
+      <c r="J53" s="6"/>
+      <c r="K53" s="6"/>
+    </row>
+    <row r="54" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="20" t="s">
+        <v>389</v>
+      </c>
+      <c r="B54" s="20"/>
+      <c r="C54" s="20"/>
+      <c r="D54" s="3" t="str">
+        <f aca="false">R18</f>
+        <v>C7.Sample.xlsx: SAMPLE!A100 (screenshots A101, A107); 2026Q2PamBsiSox-Manager rows 92-94; 2026Q2BsiPamCyberark-Manager rows 425-427; Oct10_2026Users row 1599. Walkthrough: 4_Item Detail 2025 Q3 CISCO Network Administrators row 17, 2025 Q3 ISEAdmin row 55, 2026 Q1 CISCO Network Administrators row 105, 2026 Q1 ISEAdmin row 128; 5_Exceptions row 6. Policy: section B above.</v>
+      </c>
+      <c r="E54" s="3"/>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="3"/>
+      <c r="I54" s="3"/>
+      <c r="J54" s="3"/>
+      <c r="K54" s="3"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="19" t="s">
+        <v>458</v>
+      </c>
+      <c r="B56" s="19"/>
+      <c r="C56" s="19"/>
+      <c r="D56" s="19"/>
       <c r="E56" s="19"/>
       <c r="F56" s="19"/>
       <c r="G56" s="19"/>
@@ -8293,161 +8328,136 @@
       <c r="I56" s="19"/>
       <c r="J56" s="19"/>
       <c r="K56" s="19"/>
-      <c r="L56" s="19"/>
-      <c r="M56" s="19"/>
-      <c r="N56" s="19"/>
-    </row>
-    <row r="57" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="18" t="s">
-        <v>412</v>
-      </c>
-      <c r="B57" s="18"/>
-      <c r="C57" s="18"/>
-      <c r="D57" s="20" t="str">
-        <f aca="false">"NO - SLA not met. IAMS termination date "&amp;TEXT(D8,"mm/dd/yyyy")&amp;"; removal was due by "&amp;TEXT(O8,"mm/dd/yyyy")&amp;" (30 business days after the 08/28/2025 review) and access was still held on "&amp;TEXT(Q8,"mm/dd/yyyy")&amp;", "&amp;R8&amp;" business days past the deadline."</f>
-        <v>NO - SLA not met. IAMS termination date 12/31/2024; removal was due by 10/10/2025 (30 business days after the 08/28/2025 review) and access was still held on 08/17/2026, 211 business days past the deadline.</v>
-      </c>
-      <c r="E57" s="20"/>
-      <c r="F57" s="20"/>
-      <c r="G57" s="20"/>
-      <c r="H57" s="20"/>
-      <c r="I57" s="20"/>
-      <c r="J57" s="20"/>
-      <c r="K57" s="20"/>
-      <c r="L57" s="20"/>
-      <c r="M57" s="20"/>
-      <c r="N57" s="20"/>
-    </row>
-    <row r="58" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="18" t="s">
+    </row>
+    <row r="57" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="20" t="s">
+        <v>447</v>
+      </c>
+      <c r="B57" s="20"/>
+      <c r="C57" s="20"/>
+      <c r="D57" s="3" t="str">
+        <f aca="false">H19&amp;". No Revoked decision in any review (reviewer: Borges, Dayam)."</f>
+        <v>Approved 08/28/2025 / Approved 04/30/2026 / Approved 7/27/26, 12:45 PM (SOX) and 8/17/26, 9:23 AM (CyberArk). No Revoked decision in any review (reviewer: Borges, Dayam).</v>
+      </c>
+      <c r="E57" s="3"/>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="H57" s="3"/>
+      <c r="I57" s="3"/>
+      <c r="J57" s="3"/>
+      <c r="K57" s="3"/>
+    </row>
+    <row r="58" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="B58" s="20"/>
+      <c r="C58" s="20"/>
+      <c r="D58" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="E58" s="3"/>
+      <c r="F58" s="3"/>
+      <c r="G58" s="3"/>
+      <c r="H58" s="3"/>
+      <c r="I58" s="3"/>
+      <c r="J58" s="3"/>
+      <c r="K58" s="3"/>
+    </row>
+    <row r="59" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="20" t="s">
+        <v>450</v>
+      </c>
+      <c r="B59" s="20"/>
+      <c r="C59" s="20"/>
+      <c r="D59" s="12" t="s">
+        <v>451</v>
+      </c>
+      <c r="E59" s="12"/>
+      <c r="F59" s="12"/>
+      <c r="G59" s="12"/>
+      <c r="H59" s="12"/>
+      <c r="I59" s="12"/>
+      <c r="J59" s="12"/>
+      <c r="K59" s="12"/>
+    </row>
+    <row r="60" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B58" s="18"/>
-      <c r="C58" s="18"/>
-      <c r="D58" s="19" t="s">
-        <v>413</v>
-      </c>
-      <c r="E58" s="19"/>
-      <c r="F58" s="19"/>
-      <c r="G58" s="19"/>
-      <c r="H58" s="19"/>
-      <c r="I58" s="19"/>
-      <c r="J58" s="19"/>
-      <c r="K58" s="19"/>
-      <c r="L58" s="19"/>
-      <c r="M58" s="19"/>
-      <c r="N58" s="19"/>
-    </row>
-    <row r="59" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="18" t="s">
-        <v>414</v>
-      </c>
-      <c r="B59" s="18"/>
-      <c r="C59" s="18"/>
-      <c r="D59" s="19" t="str">
-        <f aca="false">"C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = "&amp;IF(G8,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
-        <v>C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = TRUE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
-      </c>
-      <c r="E59" s="19"/>
-      <c r="F59" s="19"/>
-      <c r="G59" s="19"/>
-      <c r="H59" s="19"/>
-      <c r="I59" s="19"/>
-      <c r="J59" s="19"/>
-      <c r="K59" s="19"/>
-      <c r="L59" s="19"/>
-      <c r="M59" s="19"/>
-      <c r="N59" s="19"/>
-    </row>
-    <row r="60" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="18" t="s">
+      <c r="B60" s="20"/>
+      <c r="C60" s="20"/>
+      <c r="D60" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="E60" s="3"/>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
+      <c r="H60" s="3"/>
+      <c r="I60" s="3"/>
+      <c r="J60" s="3"/>
+      <c r="K60" s="3"/>
+    </row>
+    <row r="61" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="20" t="s">
+        <v>453</v>
+      </c>
+      <c r="B61" s="20"/>
+      <c r="C61" s="20"/>
+      <c r="D61" s="3" t="str">
+        <f aca="false">"C7.Sample.xlsx certification exports (all Approved, WorkItemID blank) and AD export (enabled 10/10/2026 = "&amp;IF(F19,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
+        <v>C7.Sample.xlsx certification exports (all Approved, WorkItemID blank) and AD export (enabled 10/10/2026 = TRUE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
+      </c>
+      <c r="E61" s="3"/>
+      <c r="F61" s="3"/>
+      <c r="G61" s="3"/>
+      <c r="H61" s="3"/>
+      <c r="I61" s="3"/>
+      <c r="J61" s="3"/>
+      <c r="K61" s="3"/>
+    </row>
+    <row r="62" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="B60" s="18"/>
-      <c r="C60" s="18"/>
-      <c r="D60" s="20" t="s">
-        <v>422</v>
-      </c>
-      <c r="E60" s="20"/>
-      <c r="F60" s="20"/>
-      <c r="G60" s="20"/>
-      <c r="H60" s="20"/>
-      <c r="I60" s="20"/>
-      <c r="J60" s="20"/>
-      <c r="K60" s="20"/>
-      <c r="L60" s="20"/>
-      <c r="M60" s="20"/>
-      <c r="N60" s="20"/>
-    </row>
-    <row r="61" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="18" t="s">
-        <v>416</v>
-      </c>
-      <c r="B61" s="18"/>
-      <c r="C61" s="18"/>
-      <c r="D61" s="19" t="str">
-        <f aca="false">T8</f>
-        <v>C7.Sample.xlsx: SAMPLE!A128 (screenshots at A129 and A135); 2026Q2PamBsiSox-Manager rows 104-106; 2026Q2BsiPamCyberark-Manager rows 437-439; Oct10_2026Users row 1787. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 23, 2025 Q3 ISEAdmin row 58, 2026 Q1 CISCO Network Administrators row 110, 2026 Q1 ISEAdmin row 133; 5_Exceptions row 11. This workbook: 2_Item Detail.</v>
-      </c>
-      <c r="E61" s="19"/>
-      <c r="F61" s="19"/>
-      <c r="G61" s="19"/>
-      <c r="H61" s="19"/>
-      <c r="I61" s="19"/>
-      <c r="J61" s="19"/>
-      <c r="K61" s="19"/>
-      <c r="L61" s="19"/>
-      <c r="M61" s="19"/>
-      <c r="N61" s="19"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="17" t="s">
-        <v>423</v>
-      </c>
-      <c r="B63" s="17"/>
-      <c r="C63" s="17"/>
-      <c r="D63" s="17"/>
-      <c r="E63" s="17"/>
-      <c r="F63" s="17"/>
-      <c r="G63" s="17"/>
-      <c r="H63" s="17"/>
-      <c r="I63" s="17"/>
-      <c r="J63" s="17"/>
-      <c r="K63" s="17"/>
-      <c r="L63" s="17"/>
-      <c r="M63" s="17"/>
-      <c r="N63" s="17"/>
-    </row>
-    <row r="64" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="18" t="s">
-        <v>409</v>
-      </c>
-      <c r="B64" s="18"/>
-      <c r="C64" s="18"/>
-      <c r="D64" s="19" t="str">
-        <f aca="false">"Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), "&amp;J9&amp;", "&amp;K9&amp;". No Revoked decision in any review."</f>
-        <v>Approved 08/28/2025 (2025 Q3), 04/30/2026 (2026 Q1), Approved 7/27/26, 12:45 PM (Borges, Dayam), Approved 8/17/26, 9:23 AM (Borges, Dayam). No Revoked decision in any review.</v>
-      </c>
-      <c r="E64" s="19"/>
-      <c r="F64" s="19"/>
-      <c r="G64" s="19"/>
-      <c r="H64" s="19"/>
-      <c r="I64" s="19"/>
-      <c r="J64" s="19"/>
-      <c r="K64" s="19"/>
-      <c r="L64" s="19"/>
-      <c r="M64" s="19"/>
-      <c r="N64" s="19"/>
-    </row>
-    <row r="65" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="18" t="s">
-        <v>410</v>
-      </c>
-      <c r="B65" s="18"/>
-      <c r="C65" s="18"/>
-      <c r="D65" s="19" t="s">
-        <v>411</v>
-      </c>
+      <c r="B62" s="20"/>
+      <c r="C62" s="20"/>
+      <c r="D62" s="6" t="s">
+        <v>456</v>
+      </c>
+      <c r="E62" s="6"/>
+      <c r="F62" s="6"/>
+      <c r="G62" s="6"/>
+      <c r="H62" s="6"/>
+      <c r="I62" s="6"/>
+      <c r="J62" s="6"/>
+      <c r="K62" s="6"/>
+    </row>
+    <row r="63" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="20" t="s">
+        <v>389</v>
+      </c>
+      <c r="B63" s="20"/>
+      <c r="C63" s="20"/>
+      <c r="D63" s="3" t="str">
+        <f aca="false">R19</f>
+        <v>C7.Sample.xlsx: SAMPLE!A114 (screenshots A115, A121); 2026Q2PamBsiSox-Manager rows 95-97; 2026Q2BsiPamCyberark-Manager rows 428-430; Oct10_2026Users row 1597. Walkthrough: 4_Item Detail 2025 Q3 CISCO Network Administrators row 18, 2025 Q3 ISEAdmin row 56, 2026 Q1 CISCO Network Administrators row 106, 2026 Q1 ISEAdmin row 129; 5_Exceptions row 7. Policy: section B above.</v>
+      </c>
+      <c r="E63" s="3"/>
+      <c r="F63" s="3"/>
+      <c r="G63" s="3"/>
+      <c r="H63" s="3"/>
+      <c r="I63" s="3"/>
+      <c r="J63" s="3"/>
+      <c r="K63" s="3"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="19" t="s">
+        <v>459</v>
+      </c>
+      <c r="B65" s="19"/>
+      <c r="C65" s="19"/>
+      <c r="D65" s="19"/>
       <c r="E65" s="19"/>
       <c r="F65" s="19"/>
       <c r="G65" s="19"/>
@@ -8455,210 +8465,450 @@
       <c r="I65" s="19"/>
       <c r="J65" s="19"/>
       <c r="K65" s="19"/>
-      <c r="L65" s="19"/>
-      <c r="M65" s="19"/>
-      <c r="N65" s="19"/>
-    </row>
-    <row r="66" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="18" t="s">
-        <v>412</v>
-      </c>
-      <c r="B66" s="18"/>
-      <c r="C66" s="18"/>
-      <c r="D66" s="20" t="str">
-        <f aca="false">"NO - SLA not met. IAMS termination date "&amp;TEXT(D9,"mm/dd/yyyy")&amp;"; removal was due by "&amp;TEXT(O9,"mm/dd/yyyy")&amp;" (30 business days after the 08/28/2025 review) and access was still held on "&amp;TEXT(Q9,"mm/dd/yyyy")&amp;", "&amp;R9&amp;" business days past the deadline."</f>
-        <v>NO - SLA not met. IAMS termination date 12/31/2024; removal was due by 10/10/2025 (30 business days after the 08/28/2025 review) and access was still held on 08/17/2026, 211 business days past the deadline.</v>
-      </c>
-      <c r="E66" s="20"/>
-      <c r="F66" s="20"/>
-      <c r="G66" s="20"/>
-      <c r="H66" s="20"/>
-      <c r="I66" s="20"/>
-      <c r="J66" s="20"/>
-      <c r="K66" s="20"/>
-      <c r="L66" s="20"/>
-      <c r="M66" s="20"/>
-      <c r="N66" s="20"/>
-    </row>
-    <row r="67" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="18" t="s">
+    </row>
+    <row r="66" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="20" t="s">
+        <v>447</v>
+      </c>
+      <c r="B66" s="20"/>
+      <c r="C66" s="20"/>
+      <c r="D66" s="3" t="str">
+        <f aca="false">H20&amp;". No Revoked decision in any review (reviewer: Borges, Dayam)."</f>
+        <v>Approved 08/28/2025 / Approved 04/30/2026 / Approved 7/27/26, 12:45 PM (SOX) and 8/17/26, 9:23 AM (CyberArk). No Revoked decision in any review (reviewer: Borges, Dayam).</v>
+      </c>
+      <c r="E66" s="3"/>
+      <c r="F66" s="3"/>
+      <c r="G66" s="3"/>
+      <c r="H66" s="3"/>
+      <c r="I66" s="3"/>
+      <c r="J66" s="3"/>
+      <c r="K66" s="3"/>
+    </row>
+    <row r="67" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="B67" s="20"/>
+      <c r="C67" s="20"/>
+      <c r="D67" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="E67" s="3"/>
+      <c r="F67" s="3"/>
+      <c r="G67" s="3"/>
+      <c r="H67" s="3"/>
+      <c r="I67" s="3"/>
+      <c r="J67" s="3"/>
+      <c r="K67" s="3"/>
+    </row>
+    <row r="68" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="20" t="s">
+        <v>450</v>
+      </c>
+      <c r="B68" s="20"/>
+      <c r="C68" s="20"/>
+      <c r="D68" s="12" t="s">
+        <v>451</v>
+      </c>
+      <c r="E68" s="12"/>
+      <c r="F68" s="12"/>
+      <c r="G68" s="12"/>
+      <c r="H68" s="12"/>
+      <c r="I68" s="12"/>
+      <c r="J68" s="12"/>
+      <c r="K68" s="12"/>
+    </row>
+    <row r="69" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B67" s="18"/>
-      <c r="C67" s="18"/>
-      <c r="D67" s="19" t="s">
-        <v>413</v>
-      </c>
-      <c r="E67" s="19"/>
-      <c r="F67" s="19"/>
-      <c r="G67" s="19"/>
-      <c r="H67" s="19"/>
-      <c r="I67" s="19"/>
-      <c r="J67" s="19"/>
-      <c r="K67" s="19"/>
-      <c r="L67" s="19"/>
-      <c r="M67" s="19"/>
-      <c r="N67" s="19"/>
-    </row>
-    <row r="68" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="18" t="s">
-        <v>414</v>
-      </c>
-      <c r="B68" s="18"/>
-      <c r="C68" s="18"/>
-      <c r="D68" s="19" t="str">
-        <f aca="false">"C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = "&amp;IF(G9,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
-        <v>C7.Sample.xlsx certification exports and AD export (AD enabled 10/10/2026 = TRUE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
-      </c>
-      <c r="E68" s="19"/>
-      <c r="F68" s="19"/>
-      <c r="G68" s="19"/>
-      <c r="H68" s="19"/>
-      <c r="I68" s="19"/>
-      <c r="J68" s="19"/>
-      <c r="K68" s="19"/>
-      <c r="L68" s="19"/>
-      <c r="M68" s="19"/>
-      <c r="N68" s="19"/>
-    </row>
-    <row r="69" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="18" t="s">
+      <c r="B69" s="20"/>
+      <c r="C69" s="20"/>
+      <c r="D69" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="E69" s="3"/>
+      <c r="F69" s="3"/>
+      <c r="G69" s="3"/>
+      <c r="H69" s="3"/>
+      <c r="I69" s="3"/>
+      <c r="J69" s="3"/>
+      <c r="K69" s="3"/>
+    </row>
+    <row r="70" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="20" t="s">
+        <v>453</v>
+      </c>
+      <c r="B70" s="20"/>
+      <c r="C70" s="20"/>
+      <c r="D70" s="3" t="str">
+        <f aca="false">"C7.Sample.xlsx certification exports (all Approved, WorkItemID blank) and AD export (enabled 10/10/2026 = "&amp;IF(F20,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
+        <v>C7.Sample.xlsx certification exports (all Approved, WorkItemID blank) and AD export (enabled 10/10/2026 = TRUE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
+      </c>
+      <c r="E70" s="3"/>
+      <c r="F70" s="3"/>
+      <c r="G70" s="3"/>
+      <c r="H70" s="3"/>
+      <c r="I70" s="3"/>
+      <c r="J70" s="3"/>
+      <c r="K70" s="3"/>
+    </row>
+    <row r="71" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="B69" s="18"/>
-      <c r="C69" s="18"/>
-      <c r="D69" s="20" t="s">
-        <v>424</v>
-      </c>
-      <c r="E69" s="20"/>
-      <c r="F69" s="20"/>
-      <c r="G69" s="20"/>
-      <c r="H69" s="20"/>
-      <c r="I69" s="20"/>
-      <c r="J69" s="20"/>
-      <c r="K69" s="20"/>
-      <c r="L69" s="20"/>
-      <c r="M69" s="20"/>
-      <c r="N69" s="20"/>
-    </row>
-    <row r="70" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="18" t="s">
-        <v>416</v>
-      </c>
-      <c r="B70" s="18"/>
-      <c r="C70" s="18"/>
-      <c r="D70" s="19" t="str">
-        <f aca="false">T9</f>
-        <v>C7.Sample.xlsx: SAMPLE!A142 (screenshots at A143 and A149); 2026Q2PamBsiSox-Manager rows 101-103; 2026Q2BsiPamCyberark-Manager rows 434-436; Oct10_2026Users row 1785. Walkthrough (BSI.IT.27.C7.05): 4_Item Detail 2025 Q3 CISCO Network Administrators row 24, 2025 Q3 ISEAdmin row 59, 2026 Q1 CISCO Network Administrators row 111, 2026 Q1 ISEAdmin row 134; 5_Exceptions row 12. This workbook: 2_Item Detail.</v>
-      </c>
-      <c r="E70" s="19"/>
-      <c r="F70" s="19"/>
-      <c r="G70" s="19"/>
-      <c r="H70" s="19"/>
-      <c r="I70" s="19"/>
-      <c r="J70" s="19"/>
-      <c r="K70" s="19"/>
-      <c r="L70" s="19"/>
-      <c r="M70" s="19"/>
-      <c r="N70" s="19"/>
+      <c r="B71" s="20"/>
+      <c r="C71" s="20"/>
+      <c r="D71" s="6" t="s">
+        <v>460</v>
+      </c>
+      <c r="E71" s="6"/>
+      <c r="F71" s="6"/>
+      <c r="G71" s="6"/>
+      <c r="H71" s="6"/>
+      <c r="I71" s="6"/>
+      <c r="J71" s="6"/>
+      <c r="K71" s="6"/>
+    </row>
+    <row r="72" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="20" t="s">
+        <v>389</v>
+      </c>
+      <c r="B72" s="20"/>
+      <c r="C72" s="20"/>
+      <c r="D72" s="3" t="str">
+        <f aca="false">R20</f>
+        <v>C7.Sample.xlsx: SAMPLE!A128 (screenshots A129, A135); 2026Q2PamBsiSox-Manager rows 104-106; 2026Q2BsiPamCyberark-Manager rows 437-439; Oct10_2026Users row 1787. Walkthrough: 4_Item Detail 2025 Q3 CISCO Network Administrators row 23, 2025 Q3 ISEAdmin row 58, 2026 Q1 CISCO Network Administrators row 110, 2026 Q1 ISEAdmin row 133; 5_Exceptions row 11. Policy: section B above.</v>
+      </c>
+      <c r="E72" s="3"/>
+      <c r="F72" s="3"/>
+      <c r="G72" s="3"/>
+      <c r="H72" s="3"/>
+      <c r="I72" s="3"/>
+      <c r="J72" s="3"/>
+      <c r="K72" s="3"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="19" t="s">
+        <v>461</v>
+      </c>
+      <c r="B74" s="19"/>
+      <c r="C74" s="19"/>
+      <c r="D74" s="19"/>
+      <c r="E74" s="19"/>
+      <c r="F74" s="19"/>
+      <c r="G74" s="19"/>
+      <c r="H74" s="19"/>
+      <c r="I74" s="19"/>
+      <c r="J74" s="19"/>
+      <c r="K74" s="19"/>
+    </row>
+    <row r="75" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="20" t="s">
+        <v>447</v>
+      </c>
+      <c r="B75" s="20"/>
+      <c r="C75" s="20"/>
+      <c r="D75" s="3" t="str">
+        <f aca="false">H21&amp;". No Revoked decision in any review (reviewer: Borges, Dayam)."</f>
+        <v>Approved 08/28/2025 / Approved 04/30/2026 / Approved 7/27/26, 12:45 PM (SOX) and 8/17/26, 9:23 AM (CyberArk). No Revoked decision in any review (reviewer: Borges, Dayam).</v>
+      </c>
+      <c r="E75" s="3"/>
+      <c r="F75" s="3"/>
+      <c r="G75" s="3"/>
+      <c r="H75" s="3"/>
+      <c r="I75" s="3"/>
+      <c r="J75" s="3"/>
+      <c r="K75" s="3"/>
+    </row>
+    <row r="76" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="B76" s="20"/>
+      <c r="C76" s="20"/>
+      <c r="D76" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="E76" s="3"/>
+      <c r="F76" s="3"/>
+      <c r="G76" s="3"/>
+      <c r="H76" s="3"/>
+      <c r="I76" s="3"/>
+      <c r="J76" s="3"/>
+      <c r="K76" s="3"/>
+    </row>
+    <row r="77" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="20" t="s">
+        <v>450</v>
+      </c>
+      <c r="B77" s="20"/>
+      <c r="C77" s="20"/>
+      <c r="D77" s="12" t="s">
+        <v>451</v>
+      </c>
+      <c r="E77" s="12"/>
+      <c r="F77" s="12"/>
+      <c r="G77" s="12"/>
+      <c r="H77" s="12"/>
+      <c r="I77" s="12"/>
+      <c r="J77" s="12"/>
+      <c r="K77" s="12"/>
+    </row>
+    <row r="78" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B78" s="20"/>
+      <c r="C78" s="20"/>
+      <c r="D78" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="E78" s="3"/>
+      <c r="F78" s="3"/>
+      <c r="G78" s="3"/>
+      <c r="H78" s="3"/>
+      <c r="I78" s="3"/>
+      <c r="J78" s="3"/>
+      <c r="K78" s="3"/>
+    </row>
+    <row r="79" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="20" t="s">
+        <v>453</v>
+      </c>
+      <c r="B79" s="20"/>
+      <c r="C79" s="20"/>
+      <c r="D79" s="3" t="str">
+        <f aca="false">"C7.Sample.xlsx certification exports (all Approved, WorkItemID blank) and AD export (enabled 10/10/2026 = "&amp;IF(F21,"TRUE","FALSE")&amp;"). No Netwrix log, AD audit log or ServiceNow ticket was provided."</f>
+        <v>C7.Sample.xlsx certification exports (all Approved, WorkItemID blank) and AD export (enabled 10/10/2026 = TRUE). No Netwrix log, AD audit log or ServiceNow ticket was provided.</v>
+      </c>
+      <c r="E79" s="3"/>
+      <c r="F79" s="3"/>
+      <c r="G79" s="3"/>
+      <c r="H79" s="3"/>
+      <c r="I79" s="3"/>
+      <c r="J79" s="3"/>
+      <c r="K79" s="3"/>
+    </row>
+    <row r="80" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B80" s="20"/>
+      <c r="C80" s="20"/>
+      <c r="D80" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="E80" s="6"/>
+      <c r="F80" s="6"/>
+      <c r="G80" s="6"/>
+      <c r="H80" s="6"/>
+      <c r="I80" s="6"/>
+      <c r="J80" s="6"/>
+      <c r="K80" s="6"/>
+    </row>
+    <row r="81" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="20" t="s">
+        <v>389</v>
+      </c>
+      <c r="B81" s="20"/>
+      <c r="C81" s="20"/>
+      <c r="D81" s="3" t="str">
+        <f aca="false">R21</f>
+        <v>C7.Sample.xlsx: SAMPLE!A142 (screenshots A143, A149); 2026Q2PamBsiSox-Manager rows 101-103; 2026Q2BsiPamCyberark-Manager rows 434-436; Oct10_2026Users row 1785. Walkthrough: 4_Item Detail 2025 Q3 CISCO Network Administrators row 24, 2025 Q3 ISEAdmin row 59, 2026 Q1 CISCO Network Administrators row 111, 2026 Q1 ISEAdmin row 134; 5_Exceptions row 12. Policy: section B above.</v>
+      </c>
+      <c r="E81" s="3"/>
+      <c r="F81" s="3"/>
+      <c r="G81" s="3"/>
+      <c r="H81" s="3"/>
+      <c r="I81" s="3"/>
+      <c r="J81" s="3"/>
+      <c r="K81" s="3"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="14" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A84" s="21" t="s">
+        <v>464</v>
+      </c>
+      <c r="B84" s="21"/>
+      <c r="C84" s="21"/>
+      <c r="D84" s="21"/>
+      <c r="E84" s="21"/>
+      <c r="F84" s="21"/>
+      <c r="G84" s="21"/>
+      <c r="H84" s="21"/>
+      <c r="I84" s="21"/>
+      <c r="J84" s="21"/>
+      <c r="K84" s="21"/>
+    </row>
+    <row r="85" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="21" t="s">
+        <v>465</v>
+      </c>
+      <c r="B85" s="21"/>
+      <c r="C85" s="21"/>
+      <c r="D85" s="21"/>
+      <c r="E85" s="21"/>
+      <c r="F85" s="21"/>
+      <c r="G85" s="21"/>
+      <c r="H85" s="21"/>
+      <c r="I85" s="21"/>
+      <c r="J85" s="21"/>
+      <c r="K85" s="21"/>
+    </row>
+    <row r="86" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A86" s="21" t="s">
+        <v>466</v>
+      </c>
+      <c r="B86" s="21"/>
+      <c r="C86" s="21"/>
+      <c r="D86" s="21"/>
+      <c r="E86" s="21"/>
+      <c r="F86" s="21"/>
+      <c r="G86" s="21"/>
+      <c r="H86" s="21"/>
+      <c r="I86" s="21"/>
+      <c r="J86" s="21"/>
+      <c r="K86" s="21"/>
+    </row>
+    <row r="87" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A87" s="21" t="s">
+        <v>467</v>
+      </c>
+      <c r="B87" s="21"/>
+      <c r="C87" s="21"/>
+      <c r="D87" s="21"/>
+      <c r="E87" s="21"/>
+      <c r="F87" s="21"/>
+      <c r="G87" s="21"/>
+      <c r="H87" s="21"/>
+      <c r="I87" s="21"/>
+      <c r="J87" s="21"/>
+      <c r="K87" s="21"/>
     </row>
   </sheetData>
-  <mergeCells count="95">
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A12:N12"/>
-    <mergeCell ref="A13:N13"/>
-    <mergeCell ref="A14:N14"/>
-    <mergeCell ref="A15:N15"/>
-    <mergeCell ref="A18:N18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:N19"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="D20:N20"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="D21:N21"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="D22:N22"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="D23:N23"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="D24:N24"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="D25:N25"/>
-    <mergeCell ref="A27:N27"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="D28:N28"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="D29:N29"/>
+  <mergeCells count="117">
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D7:G7"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="A23:G23"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A26:K26"/>
+    <mergeCell ref="A29:K29"/>
     <mergeCell ref="A30:C30"/>
-    <mergeCell ref="D30:N30"/>
+    <mergeCell ref="D30:K30"/>
     <mergeCell ref="A31:C31"/>
-    <mergeCell ref="D31:N31"/>
+    <mergeCell ref="D31:K31"/>
     <mergeCell ref="A32:C32"/>
-    <mergeCell ref="D32:N32"/>
+    <mergeCell ref="D32:K32"/>
     <mergeCell ref="A33:C33"/>
-    <mergeCell ref="D33:N33"/>
+    <mergeCell ref="D33:K33"/>
     <mergeCell ref="A34:C34"/>
-    <mergeCell ref="D34:N34"/>
-    <mergeCell ref="A36:N36"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="D37:N37"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="D38:N38"/>
+    <mergeCell ref="D34:K34"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="D35:K35"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="D36:K36"/>
+    <mergeCell ref="A38:K38"/>
     <mergeCell ref="A39:C39"/>
-    <mergeCell ref="D39:N39"/>
+    <mergeCell ref="D39:K39"/>
     <mergeCell ref="A40:C40"/>
-    <mergeCell ref="D40:N40"/>
+    <mergeCell ref="D40:K40"/>
     <mergeCell ref="A41:C41"/>
-    <mergeCell ref="D41:N41"/>
+    <mergeCell ref="D41:K41"/>
     <mergeCell ref="A42:C42"/>
-    <mergeCell ref="D42:N42"/>
+    <mergeCell ref="D42:K42"/>
     <mergeCell ref="A43:C43"/>
-    <mergeCell ref="D43:N43"/>
-    <mergeCell ref="A45:N45"/>
-    <mergeCell ref="A46:C46"/>
-    <mergeCell ref="D46:N46"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="D47:N47"/>
+    <mergeCell ref="D43:K43"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="D44:K44"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="D45:K45"/>
+    <mergeCell ref="A47:K47"/>
     <mergeCell ref="A48:C48"/>
-    <mergeCell ref="D48:N48"/>
+    <mergeCell ref="D48:K48"/>
     <mergeCell ref="A49:C49"/>
-    <mergeCell ref="D49:N49"/>
+    <mergeCell ref="D49:K49"/>
     <mergeCell ref="A50:C50"/>
-    <mergeCell ref="D50:N50"/>
+    <mergeCell ref="D50:K50"/>
     <mergeCell ref="A51:C51"/>
-    <mergeCell ref="D51:N51"/>
+    <mergeCell ref="D51:K51"/>
     <mergeCell ref="A52:C52"/>
-    <mergeCell ref="D52:N52"/>
-    <mergeCell ref="A54:N54"/>
-    <mergeCell ref="A55:C55"/>
-    <mergeCell ref="D55:N55"/>
-    <mergeCell ref="A56:C56"/>
-    <mergeCell ref="D56:N56"/>
+    <mergeCell ref="D52:K52"/>
+    <mergeCell ref="A53:C53"/>
+    <mergeCell ref="D53:K53"/>
+    <mergeCell ref="A54:C54"/>
+    <mergeCell ref="D54:K54"/>
+    <mergeCell ref="A56:K56"/>
     <mergeCell ref="A57:C57"/>
-    <mergeCell ref="D57:N57"/>
+    <mergeCell ref="D57:K57"/>
     <mergeCell ref="A58:C58"/>
-    <mergeCell ref="D58:N58"/>
+    <mergeCell ref="D58:K58"/>
     <mergeCell ref="A59:C59"/>
-    <mergeCell ref="D59:N59"/>
+    <mergeCell ref="D59:K59"/>
     <mergeCell ref="A60:C60"/>
-    <mergeCell ref="D60:N60"/>
+    <mergeCell ref="D60:K60"/>
     <mergeCell ref="A61:C61"/>
-    <mergeCell ref="D61:N61"/>
-    <mergeCell ref="A63:N63"/>
-    <mergeCell ref="A64:C64"/>
-    <mergeCell ref="D64:N64"/>
-    <mergeCell ref="A65:C65"/>
-    <mergeCell ref="D65:N65"/>
+    <mergeCell ref="D61:K61"/>
+    <mergeCell ref="A62:C62"/>
+    <mergeCell ref="D62:K62"/>
+    <mergeCell ref="A63:C63"/>
+    <mergeCell ref="D63:K63"/>
+    <mergeCell ref="A65:K65"/>
     <mergeCell ref="A66:C66"/>
-    <mergeCell ref="D66:N66"/>
+    <mergeCell ref="D66:K66"/>
     <mergeCell ref="A67:C67"/>
-    <mergeCell ref="D67:N67"/>
+    <mergeCell ref="D67:K67"/>
     <mergeCell ref="A68:C68"/>
-    <mergeCell ref="D68:N68"/>
+    <mergeCell ref="D68:K68"/>
     <mergeCell ref="A69:C69"/>
-    <mergeCell ref="D69:N69"/>
+    <mergeCell ref="D69:K69"/>
     <mergeCell ref="A70:C70"/>
-    <mergeCell ref="D70:N70"/>
+    <mergeCell ref="D70:K70"/>
+    <mergeCell ref="A71:C71"/>
+    <mergeCell ref="D71:K71"/>
+    <mergeCell ref="A72:C72"/>
+    <mergeCell ref="D72:K72"/>
+    <mergeCell ref="A74:K74"/>
+    <mergeCell ref="A75:C75"/>
+    <mergeCell ref="D75:K75"/>
+    <mergeCell ref="A76:C76"/>
+    <mergeCell ref="D76:K76"/>
+    <mergeCell ref="A77:C77"/>
+    <mergeCell ref="D77:K77"/>
+    <mergeCell ref="A78:C78"/>
+    <mergeCell ref="D78:K78"/>
+    <mergeCell ref="A79:C79"/>
+    <mergeCell ref="D79:K79"/>
+    <mergeCell ref="A80:C80"/>
+    <mergeCell ref="D80:K80"/>
+    <mergeCell ref="A81:C81"/>
+    <mergeCell ref="D81:K81"/>
+    <mergeCell ref="A84:K84"/>
+    <mergeCell ref="A85:K85"/>
+    <mergeCell ref="A86:K86"/>
+    <mergeCell ref="A87:K87"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -8684,175 +8934,175 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>425</v>
+        <v>468</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>426</v>
+        <v>469</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>427</v>
+        <v>470</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="21" t="n">
+      <c r="A4" s="22" t="n">
         <v>45658</v>
       </c>
-      <c r="B4" s="22" t="s">
-        <v>428</v>
+      <c r="B4" s="23" t="s">
+        <v>471</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="21" t="n">
+      <c r="A5" s="22" t="n">
         <v>45677</v>
       </c>
-      <c r="B5" s="22" t="s">
-        <v>429</v>
+      <c r="B5" s="23" t="s">
+        <v>472</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="n">
+      <c r="A6" s="22" t="n">
         <v>45705</v>
       </c>
-      <c r="B6" s="22" t="s">
-        <v>430</v>
+      <c r="B6" s="23" t="s">
+        <v>473</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="n">
+      <c r="A7" s="22" t="n">
         <v>45803</v>
       </c>
-      <c r="B7" s="22" t="s">
-        <v>431</v>
+      <c r="B7" s="23" t="s">
+        <v>474</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="n">
+      <c r="A8" s="22" t="n">
         <v>45827</v>
       </c>
-      <c r="B8" s="22" t="s">
-        <v>432</v>
+      <c r="B8" s="23" t="s">
+        <v>475</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="n">
+      <c r="A9" s="22" t="n">
         <v>45842</v>
       </c>
-      <c r="B9" s="22" t="s">
-        <v>433</v>
+      <c r="B9" s="23" t="s">
+        <v>476</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="n">
+      <c r="A10" s="22" t="n">
         <v>45901</v>
       </c>
-      <c r="B10" s="22" t="s">
-        <v>434</v>
+      <c r="B10" s="23" t="s">
+        <v>477</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="n">
+      <c r="A11" s="22" t="n">
         <v>45943</v>
       </c>
-      <c r="B11" s="22" t="s">
-        <v>435</v>
+      <c r="B11" s="23" t="s">
+        <v>478</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="n">
+      <c r="A12" s="22" t="n">
         <v>45972</v>
       </c>
-      <c r="B12" s="22" t="s">
-        <v>436</v>
+      <c r="B12" s="23" t="s">
+        <v>479</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="n">
+      <c r="A13" s="22" t="n">
         <v>45988</v>
       </c>
-      <c r="B13" s="22" t="s">
-        <v>437</v>
+      <c r="B13" s="23" t="s">
+        <v>480</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="n">
+      <c r="A14" s="22" t="n">
         <v>46016</v>
       </c>
-      <c r="B14" s="22" t="s">
-        <v>438</v>
+      <c r="B14" s="23" t="s">
+        <v>481</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="n">
+      <c r="A15" s="22" t="n">
         <v>46023</v>
       </c>
-      <c r="B15" s="22" t="s">
-        <v>428</v>
+      <c r="B15" s="23" t="s">
+        <v>471</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="n">
+      <c r="A16" s="22" t="n">
         <v>46041</v>
       </c>
-      <c r="B16" s="22" t="s">
-        <v>429</v>
+      <c r="B16" s="23" t="s">
+        <v>472</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="n">
+      <c r="A17" s="22" t="n">
         <v>46069</v>
       </c>
-      <c r="B17" s="22" t="s">
-        <v>430</v>
+      <c r="B17" s="23" t="s">
+        <v>473</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="n">
+      <c r="A18" s="22" t="n">
         <v>46167</v>
       </c>
-      <c r="B18" s="22" t="s">
-        <v>431</v>
+      <c r="B18" s="23" t="s">
+        <v>474</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="n">
+      <c r="A19" s="22" t="n">
         <v>46192</v>
       </c>
-      <c r="B19" s="22" t="s">
-        <v>432</v>
+      <c r="B19" s="23" t="s">
+        <v>475</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="n">
+      <c r="A20" s="22" t="n">
         <v>46206</v>
       </c>
-      <c r="B20" s="22" t="s">
-        <v>439</v>
+      <c r="B20" s="23" t="s">
+        <v>482</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="n">
+      <c r="A21" s="22" t="n">
         <v>46272</v>
       </c>
-      <c r="B21" s="22" t="s">
-        <v>434</v>
+      <c r="B21" s="23" t="s">
+        <v>477</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="n">
+      <c r="A22" s="22" t="n">
         <v>46307</v>
       </c>
-      <c r="B22" s="22" t="s">
-        <v>435</v>
+      <c r="B22" s="23" t="s">
+        <v>478</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="n">
+      <c r="A23" s="22" t="n">
         <v>46337</v>
       </c>
-      <c r="B23" s="22" t="s">
-        <v>436</v>
+      <c r="B23" s="23" t="s">
+        <v>479</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add policy references to the conclusions
Cites IAM Standard v11.0 and PAM Recertification Procedure v2.0 clauses
(with page numbers) in the 9_Sample Tab Review conclusion, a new policy
reference table, the R1 per-account conclusions, the R7 answers and the
R3 step results.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015rwvi2ZZV7Ac5SymUE9zfu
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7.06 Sample Response Evaluation - 2026 Q2.xlsx
+++ b/BSI.IT.27.C7.06 Sample Response Evaluation - 2026 Q2.xlsx
@@ -257,7 +257,7 @@
     <t xml:space="preserve">HR / vendor contract evidence that the engagement was active on each decision date (IAMS shows termination 12/31/2024); rationale for approving terminated / AD-disabled identities; AD audit (whenChanged / Netwrix) for the enable / disable history; ServiceNow ticket or exception record; group-membership extract</t>
   </si>
   <si>
-    <t xml:space="preserve">Exception (A5 - E1, E2) NOT cleared. Account is disabled in AD (11/25/2025, 05/15/2026 and 10/10/2026), yet its Cisco Network Administrators / ISEAdmin access was approved again in 2026 Q2 (7/27/2026, 8/17/2026). IAMS termination 12/31/2024. No revocation raised.</t>
+    <t xml:space="preserve">Exception (A5 - E1, E2) NOT cleared. Account is disabled in AD (11/25/2025, 05/15/2026 and 10/10/2026), yet its Cisco Network Administrators / ISEAdmin access was approved again in 2026 Q2 (7/27/2026, 8/17/2026). IAMS termination 12/31/2024. No revocation raised. Policy: SLA N/A - SUS.IAMS.4.2.5.21 (p.22) and PAM Procedure sec. 8 step 9 (p.10, "if the manager approves the user access, the process ends") start the 30-business-day clock only from a revocation. Exception basis - PAM Procedure sec. 8 step 9 (p.10): PAM submits revocation tickets for "reject" decisions or terminated users; SUS.IAMS.4.2.5.1 (p.14): review must confirm access remains valid. Leaver SLA (observation, outside C7) - SUS.IAMS.4.2.4.2 / 4.2.4.3 (p.12-13) and Appendix G (p.53): 1 business day (AD) / 30 business days (privileged access) from termination, look-back if missed.</t>
   </si>
   <si>
     <t xml:space="preserve">MIA25104</t>
@@ -284,7 +284,7 @@
     <t xml:space="preserve">C7.Sample.xlsx: SAMPLE tab screenshots; 2026Q2PamBsiSox-Manager; 2026Q2BsiPamCyberark-Manager; Oct10_2026Users row 1596; Screenshot tab (Get-ADUser export command).</t>
   </si>
   <si>
-    <t xml:space="preserve">Exception (A5 - E2) NOT cleared. Access was approved, not revoked, so there is no removal or SLA to test. IAMS still shows termination 12/31/2024 in 2026 Q2 and the access was re-approved.</t>
+    <t xml:space="preserve">Exception (A5 - E2) NOT cleared. Access was approved, not revoked, so there is no removal or SLA to test. IAMS still shows termination 12/31/2024 in 2026 Q2 and the access was re-approved. Policy: SLA N/A - SUS.IAMS.4.2.5.21 (p.22) and PAM Procedure sec. 8 step 9 (p.10, "if the manager approves the user access, the process ends") start the 30-business-day clock only from a revocation. Exception basis - PAM Procedure sec. 8 step 9 (p.10): PAM submits revocation tickets for "reject" decisions or terminated users; SUS.IAMS.4.2.5.1 (p.14): review must confirm access remains valid. Leaver SLA (observation, outside C7) - SUS.IAMS.4.2.4.2 / 4.2.4.3 (p.12-13) and Appendix G (p.53): 1 business day (AD) / 30 business days (privileged access) from termination, look-back if missed.</t>
   </si>
   <si>
     <t xml:space="preserve">MIA25105</t>
@@ -353,7 +353,7 @@
     <t xml:space="preserve">C7.Sample.xlsx: SAMPLE tab screenshots; 2026Q2PamBsiSox-Manager; 2026Q2BsiPamCyberark-Manager; Oct10_2026Users row 1787; Screenshot tab (Get-ADUser export command).</t>
   </si>
   <si>
-    <t xml:space="preserve">Exception (A5 - E2) NOT cleared. Access was approved, not revoked, so there is no removal or SLA to test. IAMS still shows termination 12/31/2024 in 2026 Q2 and the access was re-approved. AD shows the account disabled on 05/15/2026 and ENABLED again on 10/10/2026 - re-enable not explained or evidenced.</t>
+    <t xml:space="preserve">Exception (A5 - E2) NOT cleared. Access was approved, not revoked, so there is no removal or SLA to test. IAMS still shows termination 12/31/2024 in 2026 Q2 and the access was re-approved. AD shows the account disabled on 05/15/2026 and ENABLED again on 10/10/2026 - re-enable not explained or evidenced. Policy: SLA N/A - SUS.IAMS.4.2.5.21 (p.22) and PAM Procedure sec. 8 step 9 (p.10, "if the manager approves the user access, the process ends") start the 30-business-day clock only from a revocation. Exception basis - PAM Procedure sec. 8 step 9 (p.10): PAM submits revocation tickets for "reject" decisions or terminated users; SUS.IAMS.4.2.5.1 (p.14): review must confirm access remains valid. Leaver SLA (observation, outside C7) - SUS.IAMS.4.2.4.2 / 4.2.4.3 (p.12-13) and Appendix G (p.53): 1 business day (AD) / 30 business days (privileged access) from termination, look-back if missed.</t>
   </si>
   <si>
     <t xml:space="preserve">MIA25250</t>
@@ -380,7 +380,7 @@
     <t xml:space="preserve">C7.Sample.xlsx: SAMPLE tab screenshots; 2026Q2PamBsiSox-Manager; 2026Q2BsiPamCyberark-Manager; Oct10_2026Users row 1785; Screenshot tab (Get-ADUser export command).</t>
   </si>
   <si>
-    <t xml:space="preserve">Exception (A5 - E2) NOT cleared. Access was approved, not revoked, so there is no removal or SLA to test. IAMS still shows termination 12/31/2024 in 2026 Q2 and the access was re-approved. AD shows the account disabled on 05/15/2026 and ENABLED again on 10/10/2026 - re-enable not explained or evidenced. AD employeeID / employeeNumber blank on 10/10/2026; the SAMPLE tab hard-codes identity 100592068 instead of the VLOOKUP used for the other rows (A7 observation).</t>
+    <t xml:space="preserve">Exception (A5 - E2) NOT cleared. Access was approved, not revoked, so there is no removal or SLA to test. IAMS still shows termination 12/31/2024 in 2026 Q2 and the access was re-approved. AD shows the account disabled on 05/15/2026 and ENABLED again on 10/10/2026 - re-enable not explained or evidenced. AD employeeID / employeeNumber blank on 10/10/2026; the SAMPLE tab hard-codes identity 100592068 instead of the VLOOKUP used for the other rows (A7 observation). Policy: SLA N/A - SUS.IAMS.4.2.5.21 (p.22) and PAM Procedure sec. 8 step 9 (p.10, "if the manager approves the user access, the process ends") start the 30-business-day clock only from a revocation. Exception basis - PAM Procedure sec. 8 step 9 (p.10): PAM submits revocation tickets for "reject" decisions or terminated users; SUS.IAMS.4.2.5.1 (p.14): review must confirm access remains valid. Leaver SLA (observation, outside C7) - SUS.IAMS.4.2.4.2 / 4.2.4.3 (p.12-13) and Appendix G (p.53): 1 business day (AD) / 30 business days (privileged access) from termination, look-back if missed.</t>
   </si>
   <si>
     <t xml:space="preserve">Blue text = dates taken from the prior-period evidence (BSI.IT.27.C7.05 Testing Walkthrough tabs 4 / 5: 2025 Q3 SailPoint decision 08/28/2025 and Netwrix removal 09/02/2025 or 09/08/2025). They are NOT in C7.Sample.xlsx; they are restated so the SLA can be recalculated.</t>
@@ -815,7 +815,7 @@
     <t xml:space="preserve">For the 4 A6 accounts: decision date, removal date, SLA, persistence.</t>
   </si>
   <si>
-    <t xml:space="preserve">Decision 08/28/2025 (2025 Q3 Revoked). Removal 09/02/2025 (MIA25142, MIA25172) and 09/08/2025 (MIA25175, X453396) per the prior Netwrix logs = 2 and 6 business days, within the SLA deadline of 10/10/2025. Persistence: NOT sustained - the sample file shows all 4 still holding Cisco Network Administrators / ISEAdmin and approved again in 2026 Q2. The response provides no removal date, Netwrix log or ticket. The 6 supplemental accounts were never revoked, so no SLA applies.</t>
+    <t xml:space="preserve">Decision 08/28/2025 (2025 Q3 Revoked). Removal 09/02/2025 (MIA25142, MIA25172) and 09/08/2025 (MIA25175, X453396) per the prior Netwrix logs = 2 and 6 business days, within the SLA deadline of 10/10/2025. Persistence: NOT sustained - the sample file shows all 4 still holding Cisco Network Administrators / ISEAdmin and approved again in 2026 Q2. The response provides no removal date, Netwrix log or ticket. The 6 supplemental accounts were never revoked, so the 30-business-day SLA is not triggered (SUS.IAMS.4.2.5.21 p.22; PAM Procedure sec. 8 step 9 p.10); they fail A5 instead (PAM Procedure sec. 8 step 9 - revocation required for terminated users; SUS.IAMS.4.2.5.1 p.14). Persistence criterion: SUS.IAMS.4.2.5.10 (p.19), PAM Procedure 4.1.1 C4 (p.6) and sec. 4.2 (p.7).</t>
   </si>
   <si>
     <t xml:space="preserve">Fail (A6 - persistence)</t>
@@ -884,7 +884,7 @@
     <t xml:space="preserve">Coverage per attribute.</t>
   </si>
   <si>
-    <t xml:space="preserve">Completeness &amp; accuracy: Observation (no group data). Scope: Partial. Initiation: Pass. Reviewer authorization: Pass. Certification execution: Pass. Revocation decisions / appropriateness: Fail. Timeliness of removal: Pass (2025 Q3, 2 and 6 business days). Persistence: Fail. Exception management: Fail. Escalation: Fail. Risk mitigation: Fail. The response does not clear any of the 10 exceptions; the prior conclusion (Needs Improvement) stands.</t>
+    <t xml:space="preserve">Completeness &amp; accuracy: Observation (no group data). Scope: Partial. Initiation: Pass. Reviewer authorization: Pass. Certification execution: Pass. Revocation decisions / appropriateness: Fail. Timeliness of removal: Pass (2025 Q3, 2 and 6 business days). Persistence: Fail. Exception management: Fail. Escalation: Fail. Risk mitigation: Fail. The response does not clear any of the 10 exceptions; the prior conclusion (Needs Improvement) stands. Criteria: IAM Standard v11.0 SUS.IAMS.4.2.5.1, 4.2.5.6, 4.2.5.10, 4.2.5.21 and 4.2.4.2-4.2.4.3 / Appendix G; PAM Recertification Procedure v2.0 sec. 3, 4.1.1, 4.2, 5 and 8 steps 9-10.</t>
   </si>
   <si>
     <t xml:space="preserve">Evidence still needed after the C7.Sample.xlsx response</t>
@@ -1398,13 +1398,13 @@
     <t xml:space="preserve">Supporting evidence</t>
   </si>
   <si>
-    <t xml:space="preserve">Exception A5 - not an SLA exception. IAMS shows termination 12/31/2024; under PAM Procedure sec. 8 step 9 terminated users require a PAM revocation ticket, but the reviewer approved and none was raised. The AD account is disabled (11/25/2025, 05/15/2026, 10/10/2026) yet keeps and is re-approved for privileged network access - E1 stands even if the contract was active. If HR confirms the termination, the leaver SLA (SUS.IAMS.4.2.4.3, 30 business days from termination) was also missed - refer to the leaver control owner and request a look-back.</t>
+    <t xml:space="preserve">Exception A5 - not an SLA exception. IAMS shows termination 12/31/2024; under PAM Procedure sec. 8 step 9 terminated users require a PAM revocation ticket, but the reviewer approved and none was raised. The AD account is disabled (11/25/2025, 05/15/2026, 10/10/2026) yet keeps and is re-approved for privileged network access - E1 stands even if the contract was active. If HR confirms the termination, the leaver SLA (SUS.IAMS.4.2.4.3, 30 business days from termination) was also missed - refer to the leaver control owner and request a look-back. Policy: SLA N/A - SUS.IAMS.4.2.5.21 (p.22) and PAM Procedure sec. 8 step 9 (p.10, "if the manager approves the user access, the process ends") start the 30-business-day clock only from a revocation. Exception basis - PAM Procedure sec. 8 step 9 (p.10): PAM submits revocation tickets for "reject" decisions or terminated users; SUS.IAMS.4.2.5.1 (p.14): review must confirm access remains valid. Leaver SLA (observation, outside C7) - SUS.IAMS.4.2.4.2 / 4.2.4.3 (p.12-13) and Appendix G (p.53): 1 business day (AD) / 30 business days (privileged access) from termination, look-back if missed.</t>
   </si>
   <si>
     <t xml:space="preserve">Jefferson Paez Venegas (MIA25104)</t>
   </si>
   <si>
-    <t xml:space="preserve">Exception A5 - not an SLA exception. IAMS shows termination 12/31/2024; under PAM Procedure sec. 8 step 9 terminated users require a PAM revocation ticket, but the reviewer approved and none was raised. If HR confirms the termination, the leaver SLA (SUS.IAMS.4.2.4.3, 30 business days from termination) was also missed - refer to the leaver control owner and request a look-back.</t>
+    <t xml:space="preserve">Exception A5 - not an SLA exception. IAMS shows termination 12/31/2024; under PAM Procedure sec. 8 step 9 terminated users require a PAM revocation ticket, but the reviewer approved and none was raised. If HR confirms the termination, the leaver SLA (SUS.IAMS.4.2.4.3, 30 business days from termination) was also missed - refer to the leaver control owner and request a look-back. Policy: SLA N/A - SUS.IAMS.4.2.5.21 (p.22) and PAM Procedure sec. 8 step 9 (p.10, "if the manager approves the user access, the process ends") start the 30-business-day clock only from a revocation. Exception basis - PAM Procedure sec. 8 step 9 (p.10): PAM submits revocation tickets for "reject" decisions or terminated users; SUS.IAMS.4.2.5.1 (p.14): review must confirm access remains valid. Leaver SLA (observation, outside C7) - SUS.IAMS.4.2.4.2 / 4.2.4.3 (p.12-13) and Appendix G (p.53): 1 business day (AD) / 30 business days (privileged access) from termination, look-back if missed.</t>
   </si>
   <si>
     <t xml:space="preserve">David Serrano Aguirre (MIA25105)</t>
@@ -1416,13 +1416,13 @@
     <t xml:space="preserve">Richard Harris (MIA25249)</t>
   </si>
   <si>
-    <t xml:space="preserve">Exception A5 - not an SLA exception. IAMS shows termination 12/31/2024; under PAM Procedure sec. 8 step 9 terminated users require a PAM revocation ticket, but the reviewer approved and none was raised. AD shows the account disabled on 05/15/2026 and enabled again on 10/10/2026, with no request or audit event provided. If HR confirms the termination, the leaver SLA (SUS.IAMS.4.2.4.3, 30 business days from termination) was also missed - refer to the leaver control owner and request a look-back.</t>
+    <t xml:space="preserve">Exception A5 - not an SLA exception. IAMS shows termination 12/31/2024; under PAM Procedure sec. 8 step 9 terminated users require a PAM revocation ticket, but the reviewer approved and none was raised. AD shows the account disabled on 05/15/2026 and enabled again on 10/10/2026, with no request or audit event provided. If HR confirms the termination, the leaver SLA (SUS.IAMS.4.2.4.3, 30 business days from termination) was also missed - refer to the leaver control owner and request a look-back. Policy: SLA N/A - SUS.IAMS.4.2.5.21 (p.22) and PAM Procedure sec. 8 step 9 (p.10, "if the manager approves the user access, the process ends") start the 30-business-day clock only from a revocation. Exception basis - PAM Procedure sec. 8 step 9 (p.10): PAM submits revocation tickets for "reject" decisions or terminated users; SUS.IAMS.4.2.5.1 (p.14): review must confirm access remains valid. Leaver SLA (observation, outside C7) - SUS.IAMS.4.2.4.2 / 4.2.4.3 (p.12-13) and Appendix G (p.53): 1 business day (AD) / 30 business days (privileged access) from termination, look-back if missed.</t>
   </si>
   <si>
     <t xml:space="preserve">Kevin Ackley (MIA25250)</t>
   </si>
   <si>
-    <t xml:space="preserve">Exception A5 - not an SLA exception. IAMS shows termination 12/31/2024; under PAM Procedure sec. 8 step 9 terminated users require a PAM revocation ticket, but the reviewer approved and none was raised. AD shows the account disabled on 05/15/2026 and enabled again on 10/10/2026, with no request or audit event provided. AD employeeID / employeeNumber are blank, so the SAMPLE tab hard-codes identity 100592068. If HR confirms the termination, the leaver SLA (SUS.IAMS.4.2.4.3, 30 business days from termination) was also missed - refer to the leaver control owner and request a look-back.</t>
+    <t xml:space="preserve">Exception A5 - not an SLA exception. IAMS shows termination 12/31/2024; under PAM Procedure sec. 8 step 9 terminated users require a PAM revocation ticket, but the reviewer approved and none was raised. AD shows the account disabled on 05/15/2026 and enabled again on 10/10/2026, with no request or audit event provided. AD employeeID / employeeNumber are blank, so the SAMPLE tab hard-codes identity 100592068. If HR confirms the termination, the leaver SLA (SUS.IAMS.4.2.4.3, 30 business days from termination) was also missed - refer to the leaver control owner and request a look-back. Policy: SLA N/A - SUS.IAMS.4.2.5.21 (p.22) and PAM Procedure sec. 8 step 9 (p.10, "if the manager approves the user access, the process ends") start the 30-business-day clock only from a revocation. Exception basis - PAM Procedure sec. 8 step 9 (p.10): PAM submits revocation tickets for "reject" decisions or terminated users; SUS.IAMS.4.2.5.1 (p.14): review must confirm access remains valid. Leaver SLA (observation, outside C7) - SUS.IAMS.4.2.4.2 / 4.2.4.3 (p.12-13) and Appendix G (p.53): 1 business day (AD) / 30 business days (privileged access) from termination, look-back if missed.</t>
   </si>
   <si>
     <t xml:space="preserve">E. Draft response to the process owner</t>
@@ -2143,7 +2143,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="165" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="259.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="n">
         <v>1</v>
       </c>
@@ -2208,11 +2208,11 @@
         <v>35</v>
       </c>
       <c r="U4" s="6" t="str">
-        <f aca="false">"Exception (A6 - E3) NOT cleared. Removal was within the SLA ("&amp;H4&amp;" business days) but did not stay in place. The sample file shows no new revocation and no removal date; it shows the access approved again in 2026 Q2. Management to provide the re-grant request / approval or treat as an unauthorized re-grant."</f>
-        <v>Exception (A6 - E3) NOT cleared. Removal was within the SLA (2 business days) but did not stay in place. The sample file shows no new revocation and no removal date; it shows the access approved again in 2026 Q2. Management to provide the re-grant request / approval or treat as an unauthorized re-grant.</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="165" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <f aca="false">"Exception (A6 - E3) NOT cleared. Removal was within the SLA ("&amp;H4&amp;" business days) but did not stay in place. The sample file shows no new revocation and no removal date; it shows the access approved again in 2026 Q2. Management to provide the re-grant request / approval or treat as an unauthorized re-grant. Policy: SUS.IAMS.4.2.5.21 (p.22) - revocation from the review within 30 business days of the close of the review; SUS.IAMS.4.2.5.10 (p.19) - confirm all access marked for removal was removed; PAM Procedure v2.0 sec. 4.1.1 C3-C4 (p.6) - PAM confirms de-provisioning; sec. 4.2 (p.7) - rejected access that is maintained must be escalated to senior management."</f>
+        <v>Exception (A6 - E3) NOT cleared. Removal was within the SLA (2 business days) but did not stay in place. The sample file shows no new revocation and no removal date; it shows the access approved again in 2026 Q2. Management to provide the re-grant request / approval or treat as an unauthorized re-grant. Policy: SUS.IAMS.4.2.5.21 (p.22) - revocation from the review within 30 business days of the close of the review; SUS.IAMS.4.2.5.10 (p.19) - confirm all access marked for removal was removed; PAM Procedure v2.0 sec. 4.1.1 C3-C4 (p.6) - PAM confirms de-provisioning; sec. 4.2 (p.7) - rejected access that is maintained must be escalated to senior management.</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="259.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="n">
         <v>2</v>
       </c>
@@ -2277,11 +2277,11 @@
         <v>35</v>
       </c>
       <c r="U5" s="6" t="str">
-        <f aca="false">"Exception (A6 - E3) NOT cleared. Removal was within the SLA ("&amp;H5&amp;" business days) but did not stay in place. The sample file shows no new revocation and no removal date; it shows the access approved again in 2026 Q2. Management to provide the re-grant request / approval or treat as an unauthorized re-grant."</f>
-        <v>Exception (A6 - E3) NOT cleared. Removal was within the SLA (2 business days) but did not stay in place. The sample file shows no new revocation and no removal date; it shows the access approved again in 2026 Q2. Management to provide the re-grant request / approval or treat as an unauthorized re-grant.</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="165" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <f aca="false">"Exception (A6 - E3) NOT cleared. Removal was within the SLA ("&amp;H5&amp;" business days) but did not stay in place. The sample file shows no new revocation and no removal date; it shows the access approved again in 2026 Q2. Management to provide the re-grant request / approval or treat as an unauthorized re-grant. Policy: SUS.IAMS.4.2.5.21 (p.22) - revocation from the review within 30 business days of the close of the review; SUS.IAMS.4.2.5.10 (p.19) - confirm all access marked for removal was removed; PAM Procedure v2.0 sec. 4.1.1 C3-C4 (p.6) - PAM confirms de-provisioning; sec. 4.2 (p.7) - rejected access that is maintained must be escalated to senior management."</f>
+        <v>Exception (A6 - E3) NOT cleared. Removal was within the SLA (2 business days) but did not stay in place. The sample file shows no new revocation and no removal date; it shows the access approved again in 2026 Q2. Management to provide the re-grant request / approval or treat as an unauthorized re-grant. Policy: SUS.IAMS.4.2.5.21 (p.22) - revocation from the review within 30 business days of the close of the review; SUS.IAMS.4.2.5.10 (p.19) - confirm all access marked for removal was removed; PAM Procedure v2.0 sec. 4.1.1 C3-C4 (p.6) - PAM confirms de-provisioning; sec. 4.2 (p.7) - rejected access that is maintained must be escalated to senior management.</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="259.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="n">
         <v>3</v>
       </c>
@@ -2346,11 +2346,11 @@
         <v>35</v>
       </c>
       <c r="U6" s="6" t="str">
-        <f aca="false">"Exception (A6 - E3) NOT cleared. Removal was within the SLA ("&amp;H6&amp;" business days) but did not stay in place. The sample file shows no new revocation and no removal date; it shows the access approved again in 2026 Q2. Management to provide the re-grant request / approval or treat as an unauthorized re-grant."</f>
-        <v>Exception (A6 - E3) NOT cleared. Removal was within the SLA (6 business days) but did not stay in place. The sample file shows no new revocation and no removal date; it shows the access approved again in 2026 Q2. Management to provide the re-grant request / approval or treat as an unauthorized re-grant.</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="165" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <f aca="false">"Exception (A6 - E3) NOT cleared. Removal was within the SLA ("&amp;H6&amp;" business days) but did not stay in place. The sample file shows no new revocation and no removal date; it shows the access approved again in 2026 Q2. Management to provide the re-grant request / approval or treat as an unauthorized re-grant. Policy: SUS.IAMS.4.2.5.21 (p.22) - revocation from the review within 30 business days of the close of the review; SUS.IAMS.4.2.5.10 (p.19) - confirm all access marked for removal was removed; PAM Procedure v2.0 sec. 4.1.1 C3-C4 (p.6) - PAM confirms de-provisioning; sec. 4.2 (p.7) - rejected access that is maintained must be escalated to senior management."</f>
+        <v>Exception (A6 - E3) NOT cleared. Removal was within the SLA (6 business days) but did not stay in place. The sample file shows no new revocation and no removal date; it shows the access approved again in 2026 Q2. Management to provide the re-grant request / approval or treat as an unauthorized re-grant. Policy: SUS.IAMS.4.2.5.21 (p.22) - revocation from the review within 30 business days of the close of the review; SUS.IAMS.4.2.5.10 (p.19) - confirm all access marked for removal was removed; PAM Procedure v2.0 sec. 4.1.1 C3-C4 (p.6) - PAM confirms de-provisioning; sec. 4.2 (p.7) - rejected access that is maintained must be escalated to senior management.</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="259.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="n">
         <v>4</v>
       </c>
@@ -2415,11 +2415,11 @@
         <v>35</v>
       </c>
       <c r="U7" s="6" t="str">
-        <f aca="false">"Exception (A6 - E3) NOT cleared. Removal was within the SLA ("&amp;H7&amp;" business days) but did not stay in place. The sample file shows no new revocation and no removal date; it shows the access approved again in 2026 Q2. Management to provide the re-grant request / approval or treat as an unauthorized re-grant."</f>
-        <v>Exception (A6 - E3) NOT cleared. Removal was within the SLA (6 business days) but did not stay in place. The sample file shows no new revocation and no removal date; it shows the access approved again in 2026 Q2. Management to provide the re-grant request / approval or treat as an unauthorized re-grant.</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="165" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <f aca="false">"Exception (A6 - E3) NOT cleared. Removal was within the SLA ("&amp;H7&amp;" business days) but did not stay in place. The sample file shows no new revocation and no removal date; it shows the access approved again in 2026 Q2. Management to provide the re-grant request / approval or treat as an unauthorized re-grant. Policy: SUS.IAMS.4.2.5.21 (p.22) - revocation from the review within 30 business days of the close of the review; SUS.IAMS.4.2.5.10 (p.19) - confirm all access marked for removal was removed; PAM Procedure v2.0 sec. 4.1.1 C3-C4 (p.6) - PAM confirms de-provisioning; sec. 4.2 (p.7) - rejected access that is maintained must be escalated to senior management."</f>
+        <v>Exception (A6 - E3) NOT cleared. Removal was within the SLA (6 business days) but did not stay in place. The sample file shows no new revocation and no removal date; it shows the access approved again in 2026 Q2. Management to provide the re-grant request / approval or treat as an unauthorized re-grant. Policy: SUS.IAMS.4.2.5.21 (p.22) - revocation from the review within 30 business days of the close of the review; SUS.IAMS.4.2.5.10 (p.19) - confirm all access marked for removal was removed; PAM Procedure v2.0 sec. 4.1.1 C3-C4 (p.6) - PAM confirms de-provisioning; sec. 4.2 (p.7) - rejected access that is maintained must be escalated to senior management.</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="259.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="n">
         <v>5</v>
       </c>
@@ -2484,7 +2484,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="165" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="259.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="n">
         <v>6</v>
       </c>
@@ -2549,7 +2549,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="165" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="259.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="n">
         <v>7</v>
       </c>
@@ -2614,7 +2614,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="165" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="259.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="n">
         <v>8</v>
       </c>
@@ -2679,7 +2679,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="165" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="259.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="n">
         <v>9</v>
       </c>
@@ -2744,7 +2744,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="165" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="259.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="n">
         <v>10</v>
       </c>
@@ -8005,7 +8005,7 @@
       <c r="J34" s="3"/>
       <c r="K34" s="3"/>
     </row>
-    <row r="35" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="20" t="s">
         <v>21</v>
       </c>
@@ -8142,7 +8142,7 @@
       <c r="J43" s="3"/>
       <c r="K43" s="3"/>
     </row>
-    <row r="44" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="20" t="s">
         <v>21</v>
       </c>
@@ -8279,7 +8279,7 @@
       <c r="J52" s="3"/>
       <c r="K52" s="3"/>
     </row>
-    <row r="53" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="20" t="s">
         <v>21</v>
       </c>
@@ -8416,7 +8416,7 @@
       <c r="J61" s="3"/>
       <c r="K61" s="3"/>
     </row>
-    <row r="62" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="20" t="s">
         <v>21</v>
       </c>
@@ -8553,7 +8553,7 @@
       <c r="J70" s="3"/>
       <c r="K70" s="3"/>
     </row>
-    <row r="71" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="20" t="s">
         <v>21</v>
       </c>
@@ -8690,7 +8690,7 @@
       <c r="J79" s="3"/>
       <c r="K79" s="3"/>
     </row>
-    <row r="80" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="20" t="s">
         <v>21</v>
       </c>

</xml_diff>